<commit_message>
Fixed issue with payload.
</commit_message>
<xml_diff>
--- a/src/assets/payload.xlsx
+++ b/src/assets/payload.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hoccdc-my.sharepoint.com/personal/remy_vanherweghem_parl_gc_ca/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="277" documentId="8_{1586D9BE-0BEE-4142-9B86-AB9744788D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E48D9BDF-D2F1-40E6-B876-B98927FE8F76}"/>
+  <xr:revisionPtr revIDLastSave="292" documentId="8_{1586D9BE-0BEE-4142-9B86-AB9744788D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02D6D90D-0016-492E-9317-86E8AA99FE7C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{983CEFC8-2B83-4647-BCB1-636BCC2A5490}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{983CEFC8-2B83-4647-BCB1-636BCC2A5490}"/>
   </bookViews>
   <sheets>
     <sheet name="How to interface with Web tool" sheetId="8" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="314">
   <si>
     <t>INPUTS</t>
   </si>
@@ -976,6 +976,12 @@
   </si>
   <si>
     <t>Share (post 2024-25)</t>
+  </si>
+  <si>
+    <t>2029-2030</t>
+  </si>
+  <si>
+    <t>2030-2031</t>
   </si>
 </sst>
 </file>
@@ -1398,6 +1404,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{18D3F2AD-386C-47D7-A08A-D0F9FA78FC08}" name="Table12" displayName="Table12" ref="A1:C14" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:C14" xr:uid="{18D3F2AD-386C-47D7-A08A-D0F9FA78FC08}">
@@ -1973,10 +1983,10 @@
         <v>176</v>
       </c>
       <c r="Q1" s="75" t="s">
-        <v>96</v>
+        <v>312</v>
       </c>
       <c r="R1" s="75" t="s">
-        <v>97</v>
+        <v>313</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Restored initial payload (testing).
</commit_message>
<xml_diff>
--- a/src/assets/payload.xlsx
+++ b/src/assets/payload.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hoccdc-my.sharepoint.com/personal/remy_vanherweghem_parl_gc_ca/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hoccdc-my.sharepoint.com/personal/remy_vanherweghem_parl_gc_ca/Documents/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="292" documentId="8_{1586D9BE-0BEE-4142-9B86-AB9744788D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02D6D90D-0016-492E-9317-86E8AA99FE7C}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{277030AF-9D42-4CAB-874E-E19592415F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E1B38D7-C58A-4351-96F7-5FA85BC716C1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{983CEFC8-2B83-4647-BCB1-636BCC2A5490}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{983CEFC8-2B83-4647-BCB1-636BCC2A5490}"/>
   </bookViews>
   <sheets>
     <sheet name="How to interface with Web tool" sheetId="8" r:id="rId1"/>
     <sheet name="machine_readable" sheetId="7" r:id="rId2"/>
     <sheet name="Model" sheetId="1" r:id="rId3"/>
-    <sheet name="For user (EN)" sheetId="2" r:id="rId4"/>
-    <sheet name="Model Quarterly" sheetId="9" r:id="rId5"/>
+    <sheet name="Model Quarterly" sheetId="9" r:id="rId4"/>
+    <sheet name="For user (EN)" sheetId="2" r:id="rId5"/>
     <sheet name="Decomposition" sheetId="6" r:id="rId6"/>
     <sheet name="Fiscal Model Import" sheetId="5" r:id="rId7"/>
   </sheets>
@@ -1404,10 +1404,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{18D3F2AD-386C-47D7-A08A-D0F9FA78FC08}" name="Table12" displayName="Table12" ref="A1:C14" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:C14" xr:uid="{18D3F2AD-386C-47D7-A08A-D0F9FA78FC08}">
@@ -1930,7 +1926,10 @@
     <col min="8" max="8" width="18.7109375" customWidth="1"/>
     <col min="9" max="9" width="16.7109375" customWidth="1"/>
     <col min="10" max="12" width="25.7109375" customWidth="1"/>
-    <col min="13" max="17" width="9.140625" style="75"/>
+    <col min="13" max="13" width="13.7109375" style="75" customWidth="1"/>
+    <col min="14" max="15" width="9.140625" style="75"/>
+    <col min="16" max="16" width="14.5703125" style="75" customWidth="1"/>
+    <col min="17" max="17" width="9.140625" style="75"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -2012,30 +2011,7 @@
       <c r="L2" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="M2" s="75">
-        <f>'For user (EN)'!C4</f>
-        <v>0</v>
-      </c>
-      <c r="N2" s="75">
-        <f>'For user (EN)'!D4</f>
-        <v>0</v>
-      </c>
-      <c r="O2" s="75">
-        <f>'For user (EN)'!E4</f>
-        <v>0</v>
-      </c>
-      <c r="P2" s="75">
-        <f>'For user (EN)'!F4</f>
-        <v>0</v>
-      </c>
-      <c r="Q2" s="75">
-        <f>'For user (EN)'!G4</f>
-        <v>0</v>
-      </c>
-      <c r="R2" s="75">
-        <f>'For user (EN)'!H4</f>
-        <v>0</v>
-      </c>
+      <c r="R2" s="75"/>
     </row>
     <row r="3" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -2060,30 +2036,7 @@
       <c r="L3" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="M3" s="75">
-        <f>'For user (EN)'!C5</f>
-        <v>0</v>
-      </c>
-      <c r="N3" s="75">
-        <f>'For user (EN)'!D5</f>
-        <v>0</v>
-      </c>
-      <c r="O3" s="75">
-        <f>'For user (EN)'!E5</f>
-        <v>0</v>
-      </c>
-      <c r="P3" s="75">
-        <f>'For user (EN)'!F5</f>
-        <v>0</v>
-      </c>
-      <c r="Q3" s="75">
-        <f>'For user (EN)'!G5</f>
-        <v>0</v>
-      </c>
-      <c r="R3" s="75">
-        <f>'For user (EN)'!H5</f>
-        <v>0</v>
-      </c>
+      <c r="R3" s="75"/>
     </row>
     <row r="4" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -3429,7 +3382,7 @@
       </c>
       <c r="C20" s="30"/>
       <c r="D20" s="9">
-        <f t="shared" ref="D20:H20" si="2">-(D6+D18+D19)</f>
+        <f t="shared" ref="D20:I20" si="2">-(D6+D18+D19)</f>
         <v>0</v>
       </c>
       <c r="E20" s="9">
@@ -3449,7 +3402,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="9">
-        <f>-(I6+I18+I19)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4023,327 +3976,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E8F7545-787E-47D5-A81D-527FE013B894}">
-  <sheetPr>
-    <tabColor theme="5"/>
-  </sheetPr>
-  <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="34.5703125" customWidth="1"/>
-    <col min="3" max="7" width="9.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1">
-        <v>2025</v>
-      </c>
-      <c r="D1">
-        <f>C1+1</f>
-        <v>2026</v>
-      </c>
-      <c r="E1">
-        <f t="shared" ref="E1:H1" si="0">D1+1</f>
-        <v>2027</v>
-      </c>
-      <c r="F1">
-        <f t="shared" si="0"/>
-        <v>2028</v>
-      </c>
-      <c r="G1">
-        <f t="shared" si="0"/>
-        <v>2029</v>
-      </c>
-      <c r="H1">
-        <f t="shared" si="0"/>
-        <v>2030</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C2">
-        <v>2026</v>
-      </c>
-      <c r="D2">
-        <f>C2+1</f>
-        <v>2027</v>
-      </c>
-      <c r="E2">
-        <f t="shared" ref="E2:H2" si="1">D2+1</f>
-        <v>2028</v>
-      </c>
-      <c r="F2">
-        <f t="shared" si="1"/>
-        <v>2029</v>
-      </c>
-      <c r="G2">
-        <f t="shared" si="1"/>
-        <v>2030</v>
-      </c>
-      <c r="H2">
-        <f t="shared" si="1"/>
-        <v>2031</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4">
-        <v>0</v>
-      </c>
-      <c r="E4" s="4">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4">
-        <v>0</v>
-      </c>
-      <c r="G4" s="4">
-        <v>0</v>
-      </c>
-      <c r="H4" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="4">
-        <v>0</v>
-      </c>
-      <c r="D5" s="4">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4">
-        <v>0</v>
-      </c>
-      <c r="F5" s="4">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="68">
-        <f t="shared" ref="C6:G6" si="2">C4-C5</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E6" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F6" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H6" s="68">
-        <f t="shared" ref="H6" si="3">H4-H5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="13">
-        <f>Model!D38</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="13">
-        <f>Model!E38</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="13">
-        <f>Model!F38</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="13">
-        <f>Model!G38</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="13">
-        <f>Model!H38</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="13">
-        <f>Model!I38</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="13">
-        <f>Model!D39</f>
-        <v>0</v>
-      </c>
-      <c r="D11" s="13">
-        <f>Model!E39</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="13">
-        <f>Model!F39</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="13">
-        <f>Model!G39</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="13">
-        <f>Model!H39</f>
-        <v>0</v>
-      </c>
-      <c r="H11" s="13">
-        <f>Model!I39</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="13">
-        <f>Model!D38+Model!D6</f>
-        <v>0</v>
-      </c>
-      <c r="D12" s="13">
-        <f>Model!E38+Model!E6</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="13">
-        <f>Model!F38+Model!F6</f>
-        <v>0</v>
-      </c>
-      <c r="F12" s="13">
-        <f>Model!G38+Model!G6</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="13">
-        <f>Model!H38+Model!H6</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="13">
-        <f>Model!I38+Model!I6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="51">
-        <f>SUM($C10:C10)</f>
-        <v>0</v>
-      </c>
-      <c r="D13" s="51">
-        <f>SUM($C10:D10)</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="51">
-        <f>SUM($C10:E10)</f>
-        <v>0</v>
-      </c>
-      <c r="F13" s="51">
-        <f>SUM($C10:F10)</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="51">
-        <f>SUM($C10:G10)</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="51">
-        <f>SUM($C10:H10)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="90" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="B15" s="15"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6850CC84-2C73-4E9A-9D27-7F30E585FDDE}">
   <dimension ref="A1:AA83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4811,19 +4443,19 @@
         <v>0</v>
       </c>
       <c r="X6" s="4">
-        <f>'For user (EN)'!$H5/4</f>
+        <f>'For user (EN)'!$G5/4</f>
         <v>0</v>
       </c>
       <c r="Y6" s="4">
-        <f>'For user (EN)'!$H5/4</f>
+        <f>'For user (EN)'!$G5/4</f>
         <v>0</v>
       </c>
       <c r="Z6" s="4">
-        <f>'For user (EN)'!$H5/4</f>
+        <f>'For user (EN)'!$G5/4</f>
         <v>0</v>
       </c>
       <c r="AA6" s="4">
-        <f>'For user (EN)'!$H5/4</f>
+        <f>'For user (EN)'!$G5/4</f>
         <v>0</v>
       </c>
     </row>
@@ -4916,19 +4548,19 @@
         <v>0</v>
       </c>
       <c r="X7" s="4">
-        <f>'For user (EN)'!$H6/4</f>
+        <f>'For user (EN)'!$G6/4</f>
         <v>0</v>
       </c>
       <c r="Y7" s="4">
-        <f>'For user (EN)'!$H6/4</f>
+        <f>'For user (EN)'!$G6/4</f>
         <v>0</v>
       </c>
       <c r="Z7" s="4">
-        <f>'For user (EN)'!$H6/4</f>
+        <f>'For user (EN)'!$G6/4</f>
         <v>0</v>
       </c>
       <c r="AA7" s="4">
-        <f>'For user (EN)'!$H6/4</f>
+        <f>'For user (EN)'!$G6/4</f>
         <v>0</v>
       </c>
     </row>
@@ -10348,6 +9980,339 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E8F7545-787E-47D5-A81D-527FE013B894}">
+  <sheetPr>
+    <tabColor theme="5"/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.5703125" customWidth="1"/>
+    <col min="3" max="7" width="9.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1">
+        <v>2025</v>
+      </c>
+      <c r="D1">
+        <f>C1+1</f>
+        <v>2026</v>
+      </c>
+      <c r="E1">
+        <f t="shared" ref="E1:H1" si="0">D1+1</f>
+        <v>2027</v>
+      </c>
+      <c r="F1">
+        <f t="shared" si="0"/>
+        <v>2028</v>
+      </c>
+      <c r="G1">
+        <f t="shared" si="0"/>
+        <v>2029</v>
+      </c>
+      <c r="H1">
+        <f t="shared" si="0"/>
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C2">
+        <v>2026</v>
+      </c>
+      <c r="D2">
+        <f>C2+1</f>
+        <v>2027</v>
+      </c>
+      <c r="E2">
+        <f t="shared" ref="E2:H2" si="1">D2+1</f>
+        <v>2028</v>
+      </c>
+      <c r="F2">
+        <f t="shared" si="1"/>
+        <v>2029</v>
+      </c>
+      <c r="G2">
+        <f t="shared" si="1"/>
+        <v>2030</v>
+      </c>
+      <c r="H2">
+        <f t="shared" si="1"/>
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4">
+        <f>machine_readable!M2</f>
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <f>machine_readable!N2</f>
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <f>machine_readable!O2</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <f>machine_readable!P2</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <f>machine_readable!Q2</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <f>machine_readable!R2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4">
+        <f>machine_readable!M3</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="4">
+        <f>machine_readable!N3</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <f>machine_readable!O3</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <f>machine_readable!P3</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <f>machine_readable!Q3</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <f>machine_readable!R3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="68">
+        <f t="shared" ref="C6:G6" si="2">C4-C5</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="68">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="68">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F6" s="68">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="68">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H6" s="68">
+        <f t="shared" ref="H6" si="3">H4-H5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="13">
+        <f>Model!D38</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="13">
+        <f>Model!E38</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="13">
+        <f>Model!F38</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="13">
+        <f>Model!G38</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="13">
+        <f>Model!H38</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="13">
+        <f>Model!I38</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="13">
+        <f>Model!D39</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="13">
+        <f>Model!E39</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="13">
+        <f>Model!F39</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="13">
+        <f>Model!G39</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="13">
+        <f>Model!H39</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="13">
+        <f>Model!I39</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="13">
+        <f>Model!D38+Model!D6</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="13">
+        <f>Model!E38+Model!E6</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="13">
+        <f>Model!F38+Model!F6</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="13">
+        <f>Model!G38+Model!G6</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="13">
+        <f>Model!H38+Model!H6</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="13">
+        <f>Model!I38+Model!I6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="51">
+        <f>SUM($C10:C10)</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="51">
+        <f>SUM($C10:D10)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="51">
+        <f>SUM($C10:E10)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="51">
+        <f>SUM($C10:F10)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="51">
+        <f>SUM($C10:G10)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="51">
+        <f>SUM($C10:H10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A15" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="B15" s="15"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fixed issue with 0 results sheet.
</commit_message>
<xml_diff>
--- a/src/assets/payload.xlsx
+++ b/src/assets/payload.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hoccdc-my.sharepoint.com/personal/remy_vanherweghem_parl_gc_ca/Documents/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hoccdc-my.sharepoint.com/personal/remy_vanherweghem_parl_gc_ca/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{277030AF-9D42-4CAB-874E-E19592415F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E1B38D7-C58A-4351-96F7-5FA85BC716C1}"/>
+  <xr:revisionPtr revIDLastSave="338" documentId="8_{1586D9BE-0BEE-4142-9B86-AB9744788D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A95AB208-8A3A-43FF-A059-E587C9532F79}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{983CEFC8-2B83-4647-BCB1-636BCC2A5490}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="How to interface with Web tool" sheetId="8" r:id="rId1"/>
     <sheet name="machine_readable" sheetId="7" r:id="rId2"/>
     <sheet name="Model" sheetId="1" r:id="rId3"/>
-    <sheet name="Model Quarterly" sheetId="9" r:id="rId4"/>
-    <sheet name="For user (EN)" sheetId="2" r:id="rId5"/>
+    <sheet name="For user (EN)" sheetId="2" r:id="rId4"/>
+    <sheet name="Model Quarterly" sheetId="9" r:id="rId5"/>
     <sheet name="Decomposition" sheetId="6" r:id="rId6"/>
     <sheet name="Fiscal Model Import" sheetId="5" r:id="rId7"/>
   </sheets>
@@ -1404,6 +1404,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{18D3F2AD-386C-47D7-A08A-D0F9FA78FC08}" name="Table12" displayName="Table12" ref="A1:C14" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:C14" xr:uid="{18D3F2AD-386C-47D7-A08A-D0F9FA78FC08}">
@@ -1926,10 +1930,7 @@
     <col min="8" max="8" width="18.7109375" customWidth="1"/>
     <col min="9" max="9" width="16.7109375" customWidth="1"/>
     <col min="10" max="12" width="25.7109375" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" style="75" customWidth="1"/>
-    <col min="14" max="15" width="9.140625" style="75"/>
-    <col min="16" max="16" width="14.5703125" style="75" customWidth="1"/>
-    <col min="17" max="17" width="9.140625" style="75"/>
+    <col min="13" max="17" width="9.140625" style="75"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -2011,7 +2012,24 @@
       <c r="L2" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="R2" s="75"/>
+      <c r="M2" s="75">
+        <v>0</v>
+      </c>
+      <c r="N2" s="75">
+        <v>0</v>
+      </c>
+      <c r="O2" s="75">
+        <v>0</v>
+      </c>
+      <c r="P2" s="75">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="75">
+        <v>0</v>
+      </c>
+      <c r="R2" s="75">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -2036,7 +2054,24 @@
       <c r="L3" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="R3" s="75"/>
+      <c r="M3" s="75">
+        <v>0</v>
+      </c>
+      <c r="N3" s="75">
+        <v>0</v>
+      </c>
+      <c r="O3" s="75">
+        <v>0</v>
+      </c>
+      <c r="P3" s="75">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="75">
+        <v>0</v>
+      </c>
+      <c r="R3" s="75">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
@@ -3382,7 +3417,7 @@
       </c>
       <c r="C20" s="30"/>
       <c r="D20" s="9">
-        <f t="shared" ref="D20:I20" si="2">-(D6+D18+D19)</f>
+        <f t="shared" ref="D20:H20" si="2">-(D6+D18+D19)</f>
         <v>0</v>
       </c>
       <c r="E20" s="9">
@@ -3402,7 +3437,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="9">
-        <f t="shared" si="2"/>
+        <f>-(I6+I18+I19)</f>
         <v>0</v>
       </c>
     </row>
@@ -3976,6 +4011,339 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E8F7545-787E-47D5-A81D-527FE013B894}">
+  <sheetPr>
+    <tabColor theme="5"/>
+  </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.5703125" customWidth="1"/>
+    <col min="3" max="7" width="9.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1">
+        <v>2025</v>
+      </c>
+      <c r="D1">
+        <f>C1+1</f>
+        <v>2026</v>
+      </c>
+      <c r="E1">
+        <f t="shared" ref="E1:H1" si="0">D1+1</f>
+        <v>2027</v>
+      </c>
+      <c r="F1">
+        <f t="shared" si="0"/>
+        <v>2028</v>
+      </c>
+      <c r="G1">
+        <f t="shared" si="0"/>
+        <v>2029</v>
+      </c>
+      <c r="H1">
+        <f t="shared" si="0"/>
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C2">
+        <v>2026</v>
+      </c>
+      <c r="D2">
+        <f>C2+1</f>
+        <v>2027</v>
+      </c>
+      <c r="E2">
+        <f t="shared" ref="E2:H2" si="1">D2+1</f>
+        <v>2028</v>
+      </c>
+      <c r="F2">
+        <f t="shared" si="1"/>
+        <v>2029</v>
+      </c>
+      <c r="G2">
+        <f t="shared" si="1"/>
+        <v>2030</v>
+      </c>
+      <c r="H2">
+        <f t="shared" si="1"/>
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="4">
+        <f>machine_readable!M2</f>
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <f>machine_readable!N2</f>
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <f>machine_readable!O2</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <f>machine_readable!P2</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <f>machine_readable!Q2</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <f>machine_readable!R2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4">
+        <f>machine_readable!M3</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="4">
+        <f>machine_readable!N3</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <f>machine_readable!O3</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <f>machine_readable!P3</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <f>machine_readable!Q3</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <f>machine_readable!R3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="68">
+        <f t="shared" ref="C6:G6" si="2">C4-C5</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="68">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="68">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F6" s="68">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="68">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H6" s="68">
+        <f t="shared" ref="H6" si="3">H4-H5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="13">
+        <f>Model!D38</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="13">
+        <f>Model!E38</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="13">
+        <f>Model!F38</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="13">
+        <f>Model!G38</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="13">
+        <f>Model!H38</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="13">
+        <f>Model!I38</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="13">
+        <f>Model!D39</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="13">
+        <f>Model!E39</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="13">
+        <f>Model!F39</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="13">
+        <f>Model!G39</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="13">
+        <f>Model!H39</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="13">
+        <f>Model!I39</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="13">
+        <f>Model!D38+Model!D6</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="13">
+        <f>Model!E38+Model!E6</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="13">
+        <f>Model!F38+Model!F6</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="13">
+        <f>Model!G38+Model!G6</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="13">
+        <f>Model!H38+Model!H6</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="13">
+        <f>Model!I38+Model!I6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="51">
+        <f>SUM($C10:C10)</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="51">
+        <f>SUM($C10:D10)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="51">
+        <f>SUM($C10:E10)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="51">
+        <f>SUM($C10:F10)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="51">
+        <f>SUM($C10:G10)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="51">
+        <f>SUM($C10:H10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A15" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="B15" s="15"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6850CC84-2C73-4E9A-9D27-7F30E585FDDE}">
   <dimension ref="A1:AA83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4443,19 +4811,19 @@
         <v>0</v>
       </c>
       <c r="X6" s="4">
-        <f>'For user (EN)'!$G5/4</f>
+        <f>'For user (EN)'!$H5/4</f>
         <v>0</v>
       </c>
       <c r="Y6" s="4">
-        <f>'For user (EN)'!$G5/4</f>
+        <f>'For user (EN)'!$H5/4</f>
         <v>0</v>
       </c>
       <c r="Z6" s="4">
-        <f>'For user (EN)'!$G5/4</f>
+        <f>'For user (EN)'!$H5/4</f>
         <v>0</v>
       </c>
       <c r="AA6" s="4">
-        <f>'For user (EN)'!$G5/4</f>
+        <f>'For user (EN)'!$H5/4</f>
         <v>0</v>
       </c>
     </row>
@@ -4548,19 +4916,19 @@
         <v>0</v>
       </c>
       <c r="X7" s="4">
-        <f>'For user (EN)'!$G6/4</f>
+        <f>'For user (EN)'!$H6/4</f>
         <v>0</v>
       </c>
       <c r="Y7" s="4">
-        <f>'For user (EN)'!$G6/4</f>
+        <f>'For user (EN)'!$H6/4</f>
         <v>0</v>
       </c>
       <c r="Z7" s="4">
-        <f>'For user (EN)'!$G6/4</f>
+        <f>'For user (EN)'!$H6/4</f>
         <v>0</v>
       </c>
       <c r="AA7" s="4">
-        <f>'For user (EN)'!$G6/4</f>
+        <f>'For user (EN)'!$H6/4</f>
         <v>0</v>
       </c>
     </row>
@@ -9980,339 +10348,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E8F7545-787E-47D5-A81D-527FE013B894}">
-  <sheetPr>
-    <tabColor theme="5"/>
-  </sheetPr>
-  <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="34.5703125" customWidth="1"/>
-    <col min="3" max="7" width="9.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1">
-        <v>2025</v>
-      </c>
-      <c r="D1">
-        <f>C1+1</f>
-        <v>2026</v>
-      </c>
-      <c r="E1">
-        <f t="shared" ref="E1:H1" si="0">D1+1</f>
-        <v>2027</v>
-      </c>
-      <c r="F1">
-        <f t="shared" si="0"/>
-        <v>2028</v>
-      </c>
-      <c r="G1">
-        <f t="shared" si="0"/>
-        <v>2029</v>
-      </c>
-      <c r="H1">
-        <f t="shared" si="0"/>
-        <v>2030</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C2">
-        <v>2026</v>
-      </c>
-      <c r="D2">
-        <f>C2+1</f>
-        <v>2027</v>
-      </c>
-      <c r="E2">
-        <f t="shared" ref="E2:H2" si="1">D2+1</f>
-        <v>2028</v>
-      </c>
-      <c r="F2">
-        <f t="shared" si="1"/>
-        <v>2029</v>
-      </c>
-      <c r="G2">
-        <f t="shared" si="1"/>
-        <v>2030</v>
-      </c>
-      <c r="H2">
-        <f t="shared" si="1"/>
-        <v>2031</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4">
-        <f>machine_readable!M2</f>
-        <v>0</v>
-      </c>
-      <c r="D4" s="4">
-        <f>machine_readable!N2</f>
-        <v>0</v>
-      </c>
-      <c r="E4" s="4">
-        <f>machine_readable!O2</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="4">
-        <f>machine_readable!P2</f>
-        <v>0</v>
-      </c>
-      <c r="G4" s="4">
-        <f>machine_readable!Q2</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="4">
-        <f>machine_readable!R2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="4">
-        <f>machine_readable!M3</f>
-        <v>0</v>
-      </c>
-      <c r="D5" s="4">
-        <f>machine_readable!N3</f>
-        <v>0</v>
-      </c>
-      <c r="E5" s="4">
-        <f>machine_readable!O3</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="4">
-        <f>machine_readable!P3</f>
-        <v>0</v>
-      </c>
-      <c r="G5" s="4">
-        <f>machine_readable!Q3</f>
-        <v>0</v>
-      </c>
-      <c r="H5" s="4">
-        <f>machine_readable!R3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="68">
-        <f t="shared" ref="C6:G6" si="2">C4-C5</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E6" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F6" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H6" s="68">
-        <f t="shared" ref="H6" si="3">H4-H5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="13">
-        <f>Model!D38</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="13">
-        <f>Model!E38</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="13">
-        <f>Model!F38</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="13">
-        <f>Model!G38</f>
-        <v>0</v>
-      </c>
-      <c r="G10" s="13">
-        <f>Model!H38</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="13">
-        <f>Model!I38</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="13">
-        <f>Model!D39</f>
-        <v>0</v>
-      </c>
-      <c r="D11" s="13">
-        <f>Model!E39</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="13">
-        <f>Model!F39</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="13">
-        <f>Model!G39</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="13">
-        <f>Model!H39</f>
-        <v>0</v>
-      </c>
-      <c r="H11" s="13">
-        <f>Model!I39</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="13">
-        <f>Model!D38+Model!D6</f>
-        <v>0</v>
-      </c>
-      <c r="D12" s="13">
-        <f>Model!E38+Model!E6</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="13">
-        <f>Model!F38+Model!F6</f>
-        <v>0</v>
-      </c>
-      <c r="F12" s="13">
-        <f>Model!G38+Model!G6</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="13">
-        <f>Model!H38+Model!H6</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="13">
-        <f>Model!I38+Model!I6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="51">
-        <f>SUM($C10:C10)</f>
-        <v>0</v>
-      </c>
-      <c r="D13" s="51">
-        <f>SUM($C10:D10)</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="51">
-        <f>SUM($C10:E10)</f>
-        <v>0</v>
-      </c>
-      <c r="F13" s="51">
-        <f>SUM($C10:F10)</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="51">
-        <f>SUM($C10:G10)</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="51">
-        <f>SUM($C10:H10)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="90" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="B15" s="15"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feature: added missing id and type to workbook.
</commit_message>
<xml_diff>
--- a/src/assets/payload.xlsx
+++ b/src/assets/payload.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hoccdc-my.sharepoint.com/personal/remy_vanherweghem_parl_gc_ca/Documents/Workdir/PDCC2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{9EACF287-414D-4DCA-A8EA-CEC80B65AC39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7543C824-E5BA-4CF1-89EA-BCEC8523BB4E}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="8_{9EACF287-414D-4DCA-A8EA-CEC80B65AC39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C866D539-850E-4583-80E8-DB6530283A65}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{983CEFC8-2B83-4647-BCB1-636BCC2A5490}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{983CEFC8-2B83-4647-BCB1-636BCC2A5490}"/>
   </bookViews>
   <sheets>
     <sheet name="How to interface with Web tool" sheetId="8" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="328">
   <si>
     <t>INPUTS</t>
   </si>
@@ -2632,8 +2632,12 @@
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A10" s="33"/>
-      <c r="B10" s="15"/>
+      <c r="A10" s="70" t="s">
+        <v>290</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>162</v>
+      </c>
       <c r="C10" s="70" t="s">
         <v>290</v>
       </c>
@@ -2676,8 +2680,12 @@
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A11" s="33"/>
-      <c r="B11" s="15"/>
+      <c r="A11" s="70" t="s">
+        <v>291</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>162</v>
+      </c>
       <c r="C11" s="70" t="s">
         <v>291</v>
       </c>
@@ -2720,8 +2728,12 @@
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A12" s="33"/>
-      <c r="B12" s="15"/>
+      <c r="A12" s="70" t="s">
+        <v>292</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>162</v>
+      </c>
       <c r="C12" s="70" t="s">
         <v>292</v>
       </c>
@@ -3092,8 +3104,12 @@
       </c>
     </row>
     <row r="20" spans="1:17" ht="29" x14ac:dyDescent="0.35">
-      <c r="A20" s="7"/>
-      <c r="B20" s="15"/>
+      <c r="A20" s="135" t="s">
+        <v>297</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>162</v>
+      </c>
       <c r="C20" s="135" t="s">
         <v>297</v>
       </c>
@@ -3134,8 +3150,12 @@
       </c>
     </row>
     <row r="21" spans="1:17" ht="29" x14ac:dyDescent="0.35">
-      <c r="A21" s="7"/>
-      <c r="B21" s="15"/>
+      <c r="A21" s="135" t="s">
+        <v>298</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>162</v>
+      </c>
       <c r="C21" s="135" t="s">
         <v>298</v>
       </c>
@@ -3176,8 +3196,12 @@
       </c>
     </row>
     <row r="22" spans="1:17" ht="29" x14ac:dyDescent="0.35">
-      <c r="A22" s="7"/>
-      <c r="B22" s="15"/>
+      <c r="A22" s="135" t="s">
+        <v>320</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>162</v>
+      </c>
       <c r="C22" s="135" t="s">
         <v>320</v>
       </c>
@@ -3218,8 +3242,12 @@
       </c>
     </row>
     <row r="23" spans="1:17" ht="29" x14ac:dyDescent="0.35">
-      <c r="A23" s="7"/>
-      <c r="B23" s="15"/>
+      <c r="A23" s="135" t="s">
+        <v>299</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>162</v>
+      </c>
       <c r="C23" s="135" t="s">
         <v>299</v>
       </c>
@@ -3260,8 +3288,12 @@
       </c>
     </row>
     <row r="24" spans="1:17" ht="29" x14ac:dyDescent="0.35">
-      <c r="A24" s="7"/>
-      <c r="B24" s="15"/>
+      <c r="A24" s="135" t="s">
+        <v>300</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>162</v>
+      </c>
       <c r="C24" s="135" t="s">
         <v>300</v>
       </c>

</xml_diff>

<commit_message>
feat: add missing years to payload.
</commit_message>
<xml_diff>
--- a/src/assets/payload.xlsx
+++ b/src/assets/payload.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RoberJe\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D8622B1-0631-455E-B756-555AB00DD8CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5306A69-D3D3-41AC-9ACF-B25481407061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" firstSheet="1" activeTab="1" xr2:uid="{983CEFC8-2B83-4647-BCB1-636BCC2A5490}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="328">
   <si>
     <t>INPUTS</t>
   </si>
@@ -1018,6 +1018,12 @@
   </si>
   <si>
     <t>Interest on surplus/(deficit)</t>
+  </si>
+  <si>
+    <t>2029-2030</t>
+  </si>
+  <si>
+    <t>2030-2031</t>
   </si>
 </sst>
 </file>
@@ -2337,10 +2343,10 @@
         <v>152</v>
       </c>
       <c r="P1" s="134" t="s">
-        <v>77</v>
+        <v>326</v>
       </c>
       <c r="Q1" s="134" t="s">
-        <v>78</v>
+        <v>327</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2406,7 +2412,7 @@
         <v>149</v>
       </c>
       <c r="M3" s="151">
-        <v>0</v>
+        <v>123456</v>
       </c>
       <c r="N3" s="151">
         <v>0</v>
@@ -2446,7 +2452,7 @@
       </c>
       <c r="M4" s="140">
         <f>'For user (EN)'!D6</f>
-        <v>0</v>
+        <v>-123456</v>
       </c>
       <c r="N4" s="140">
         <f>'For user (EN)'!E6</f>
@@ -2490,23 +2496,23 @@
       </c>
       <c r="M5" s="140">
         <f>'For user (EN)'!D10</f>
-        <v>0</v>
+        <v>-2097.3963156339423</v>
       </c>
       <c r="N5" s="140">
         <f>'For user (EN)'!E10</f>
-        <v>0</v>
+        <v>-3785.6994555609681</v>
       </c>
       <c r="O5" s="140">
         <f>'For user (EN)'!F10</f>
-        <v>0</v>
+        <v>-4077.4454991796802</v>
       </c>
       <c r="P5" s="140">
         <f>'For user (EN)'!G10</f>
-        <v>0</v>
+        <v>-4406.0519385792704</v>
       </c>
       <c r="Q5" s="140">
         <f>'For user (EN)'!H10</f>
-        <v>0</v>
+        <v>-4603.6209930941995</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="105" x14ac:dyDescent="0.25">
@@ -2538,23 +2544,23 @@
       </c>
       <c r="M6" s="140">
         <f>'For user (EN)'!D12</f>
-        <v>0</v>
+        <v>-125553.39631563395</v>
       </c>
       <c r="N6" s="140">
         <f>'For user (EN)'!E12</f>
-        <v>0</v>
+        <v>-3785.6994555609681</v>
       </c>
       <c r="O6" s="140">
         <f>'For user (EN)'!F12</f>
-        <v>0</v>
+        <v>-4077.4454991796802</v>
       </c>
       <c r="P6" s="140">
         <f>'For user (EN)'!G12</f>
-        <v>0</v>
+        <v>-4406.0519385792704</v>
       </c>
       <c r="Q6" s="140">
         <f>'For user (EN)'!H12</f>
-        <v>0</v>
+        <v>-4603.6209930941995</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -2582,23 +2588,23 @@
       </c>
       <c r="M7" s="140">
         <f>'For user (EN)'!D11</f>
-        <v>0</v>
+        <v>-125553.39631563395</v>
       </c>
       <c r="N7" s="140">
         <f>'For user (EN)'!E11</f>
-        <v>0</v>
+        <v>-129339.09577119492</v>
       </c>
       <c r="O7" s="140">
         <f>'For user (EN)'!F11</f>
-        <v>0</v>
+        <v>-133416.54127037461</v>
       </c>
       <c r="P7" s="140">
         <f>'For user (EN)'!G11</f>
-        <v>0</v>
+        <v>-137822.59320895391</v>
       </c>
       <c r="Q7" s="140">
         <f>'For user (EN)'!H11</f>
-        <v>0</v>
+        <v>-142426.21420204811</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -2626,23 +2632,23 @@
       </c>
       <c r="M8" s="140">
         <f>'For user (EN)'!D13</f>
-        <v>0</v>
+        <v>-2097.3963156339423</v>
       </c>
       <c r="N8" s="140">
         <f>'For user (EN)'!E13</f>
-        <v>0</v>
+        <v>-5883.0957711949104</v>
       </c>
       <c r="O8" s="140">
         <f>'For user (EN)'!F13</f>
-        <v>0</v>
+        <v>-9960.5412703745897</v>
       </c>
       <c r="P8" s="140">
         <f>'For user (EN)'!G13</f>
-        <v>0</v>
+        <v>-14366.59320895386</v>
       </c>
       <c r="Q8" s="140">
         <f>'For user (EN)'!H13</f>
-        <v>0</v>
+        <v>-18970.214202048061</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -3008,23 +3014,23 @@
       <c r="L16" s="142"/>
       <c r="M16" s="145">
         <f>SUM(Model!E20,Model!E21)</f>
-        <v>0</v>
+        <v>-2097.3963156339423</v>
       </c>
       <c r="N16" s="145">
         <f>SUM(Model!F20,Model!F21)</f>
-        <v>0</v>
+        <v>-3785.6994555609681</v>
       </c>
       <c r="O16" s="145">
         <f>SUM(Model!G20,Model!G21)</f>
-        <v>0</v>
+        <v>-4077.4454991796802</v>
       </c>
       <c r="P16" s="145">
         <f>SUM(Model!H20,Model!H21)</f>
-        <v>0</v>
+        <v>-4406.0519385792704</v>
       </c>
       <c r="Q16" s="145">
         <f>SUM(Model!I20,Model!I21)</f>
-        <v>0</v>
+        <v>-4603.6209930941995</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
@@ -3054,23 +3060,23 @@
       <c r="L17" s="142"/>
       <c r="M17" s="145">
         <f>Model!E22</f>
-        <v>0</v>
+        <v>125553.39631563393</v>
       </c>
       <c r="N17" s="145">
         <f>Model!F22</f>
-        <v>0</v>
+        <v>3785.6994555609681</v>
       </c>
       <c r="O17" s="145">
         <f>Model!G22</f>
-        <v>0</v>
+        <v>4077.4454991796802</v>
       </c>
       <c r="P17" s="145">
         <f>Model!H22</f>
-        <v>0</v>
+        <v>4406.0519385792704</v>
       </c>
       <c r="Q17" s="145">
         <f>Model!I22</f>
-        <v>0</v>
+        <v>4603.6209930941995</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
@@ -3100,23 +3106,23 @@
       <c r="L18" s="142"/>
       <c r="M18" s="145">
         <f>Model!E23</f>
-        <v>0</v>
+        <v>125553.39631563395</v>
       </c>
       <c r="N18" s="145">
         <f>Model!F23</f>
-        <v>0</v>
+        <v>129339.09577119492</v>
       </c>
       <c r="O18" s="145">
         <f>Model!G23</f>
-        <v>0</v>
+        <v>133416.54127037461</v>
       </c>
       <c r="P18" s="145">
         <f>Model!H23</f>
-        <v>0</v>
+        <v>137822.59320895391</v>
       </c>
       <c r="Q18" s="145">
         <f>Model!I23</f>
-        <v>0</v>
+        <v>142426.21420204811</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
@@ -3146,23 +3152,23 @@
       <c r="L19" s="142"/>
       <c r="M19" s="145">
         <f>Model!E26</f>
-        <v>0</v>
+        <v>88879.415512061503</v>
       </c>
       <c r="N19" s="145">
         <f>Model!F26</f>
-        <v>0</v>
+        <v>25830.01913345986</v>
       </c>
       <c r="O19" s="145">
         <f>Model!G26</f>
-        <v>0</v>
+        <v>30231.985080879742</v>
       </c>
       <c r="P19" s="145">
         <f>Model!H26</f>
-        <v>0</v>
+        <v>20275.796400470554</v>
       </c>
       <c r="Q19" s="145">
         <f>Model!I26</f>
-        <v>0</v>
+        <v>14202.285043145159</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.25">
@@ -3192,23 +3198,23 @@
       <c r="L20" s="142"/>
       <c r="M20" s="145">
         <f>Model!E30</f>
-        <v>0</v>
+        <v>63396.506169442466</v>
       </c>
       <c r="N20" s="145">
         <f>Model!F30</f>
-        <v>0</v>
+        <v>18424.209451838502</v>
       </c>
       <c r="O20" s="145">
         <f>Model!G30</f>
-        <v>0</v>
+        <v>21564.073274473656</v>
       </c>
       <c r="P20" s="145">
         <f>Model!H30</f>
-        <v>0</v>
+        <v>14462.45617376221</v>
       </c>
       <c r="Q20" s="145">
         <f>Model!I30</f>
-        <v>0</v>
+        <v>10130.301219586054</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
@@ -3238,23 +3244,23 @@
       <c r="L21" s="142"/>
       <c r="M21" s="145">
         <f>Model!E31</f>
-        <v>0</v>
+        <v>35116.692142877444</v>
       </c>
       <c r="N21" s="145">
         <f>Model!F31</f>
-        <v>0</v>
+        <v>10205.56700028309</v>
       </c>
       <c r="O21" s="145">
         <f>Model!G31</f>
-        <v>0</v>
+        <v>11944.805294193742</v>
       </c>
       <c r="P21" s="145">
         <f>Model!H31</f>
-        <v>0</v>
+        <v>8011.066409976127</v>
       </c>
       <c r="Q21" s="145">
         <f>Model!I31</f>
-        <v>0</v>
+        <v>5611.3923422216876</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
@@ -3284,23 +3290,23 @@
       <c r="L22" s="142"/>
       <c r="M22" s="145">
         <f>Model!E33</f>
-        <v>0</v>
+        <v>61839.217508747482</v>
       </c>
       <c r="N22" s="145">
         <f>Model!F33</f>
-        <v>0</v>
+        <v>50674.096130020487</v>
       </c>
       <c r="O22" s="145">
         <f>Model!G33</f>
-        <v>0</v>
+        <v>22371.355697754247</v>
       </c>
       <c r="P22" s="145">
         <f>Model!H33</f>
-        <v>0</v>
+        <v>27505.496779842266</v>
       </c>
       <c r="Q22" s="145">
         <f>Model!I33</f>
-        <v>0</v>
+        <v>12655.608626874198</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
@@ -3338,15 +3344,15 @@
       </c>
       <c r="O23" s="145">
         <f>Model!G37</f>
-        <v>0</v>
+        <v>37292.062452613216</v>
       </c>
       <c r="P23" s="145">
         <f>Model!H37</f>
-        <v>0</v>
+        <v>10837.770265787354</v>
       </c>
       <c r="Q23" s="145">
         <f>Model!I37</f>
-        <v>0</v>
+        <v>12684.748984984504</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
@@ -3376,23 +3382,23 @@
       <c r="L24" s="142"/>
       <c r="M24" s="145">
         <f>Model!E39</f>
-        <v>0</v>
+        <v>27040.198003314028</v>
       </c>
       <c r="N24" s="145">
         <f>Model!F39</f>
-        <v>0</v>
+        <v>2196.1210067534025</v>
       </c>
       <c r="O24" s="145">
         <f>Model!G39</f>
-        <v>0</v>
+        <v>10056.750389878895</v>
       </c>
       <c r="P24" s="145">
         <f>Model!H39</f>
-        <v>0</v>
+        <v>2827.0500105071801</v>
       </c>
       <c r="Q24" s="145">
         <f>Model!I39</f>
-        <v>0</v>
+        <v>4373.7264267781402</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
@@ -3422,23 +3428,23 @@
       <c r="L25" s="142"/>
       <c r="M25" s="145">
         <f>Model!E43</f>
-        <v>0</v>
+        <v>63396.506169442466</v>
       </c>
       <c r="N25" s="145">
         <f>Model!F43</f>
-        <v>0</v>
+        <v>81820.715621280979</v>
       </c>
       <c r="O25" s="145">
         <f>Model!G43</f>
-        <v>0</v>
+        <v>66092.726443141408</v>
       </c>
       <c r="P25" s="145">
         <f>Model!H43</f>
-        <v>0</v>
+        <v>69717.412351116276</v>
       </c>
       <c r="Q25" s="145">
         <f>Model!I43</f>
-        <v>0</v>
+        <v>67162.964585717826</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
@@ -3468,23 +3474,23 @@
       <c r="L26" s="142"/>
       <c r="M26" s="145">
         <f>Model!E44</f>
-        <v>0</v>
+        <v>35116.692142877444</v>
       </c>
       <c r="N26" s="145">
         <f>Model!F44</f>
-        <v>0</v>
+        <v>45322.259143160532</v>
       </c>
       <c r="O26" s="145">
         <f>Model!G44</f>
-        <v>0</v>
+        <v>57267.064437354275</v>
       </c>
       <c r="P26" s="145">
         <f>Model!H44</f>
-        <v>0</v>
+        <v>65278.130847330402</v>
       </c>
       <c r="Q26" s="145">
         <f>Model!I44</f>
-        <v>0</v>
+        <v>70889.523189552085</v>
       </c>
     </row>
     <row r="33" spans="16:16" x14ac:dyDescent="0.25">
@@ -3608,7 +3614,7 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4">
         <f>machine_readable!M3</f>
-        <v>0</v>
+        <v>123456</v>
       </c>
       <c r="E5" s="4">
         <f>machine_readable!N3</f>
@@ -3637,7 +3643,7 @@
       <c r="C6" s="59"/>
       <c r="D6" s="59">
         <f t="shared" ref="D6:G6" si="2">D4-D5</f>
-        <v>0</v>
+        <v>-123456</v>
       </c>
       <c r="E6" s="59">
         <f t="shared" si="2"/>
@@ -3678,23 +3684,23 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13">
         <f>Model!E53</f>
-        <v>0</v>
+        <v>-2097.3963156339423</v>
       </c>
       <c r="E10" s="13">
         <f>Model!F53</f>
-        <v>0</v>
+        <v>-3785.6994555609681</v>
       </c>
       <c r="F10" s="13">
         <f>Model!G53</f>
-        <v>0</v>
+        <v>-4077.4454991796802</v>
       </c>
       <c r="G10" s="13">
         <f>Model!H53</f>
-        <v>0</v>
+        <v>-4406.0519385792704</v>
       </c>
       <c r="H10" s="13">
         <f>Model!I53</f>
-        <v>0</v>
+        <v>-4603.6209930941995</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -3707,23 +3713,23 @@
       <c r="C11" s="13"/>
       <c r="D11" s="13">
         <f>Model!E54</f>
-        <v>0</v>
+        <v>-125553.39631563395</v>
       </c>
       <c r="E11" s="13">
         <f>Model!F54</f>
-        <v>0</v>
+        <v>-129339.09577119492</v>
       </c>
       <c r="F11" s="13">
         <f>Model!G54</f>
-        <v>0</v>
+        <v>-133416.54127037461</v>
       </c>
       <c r="G11" s="13">
         <f>Model!H54</f>
-        <v>0</v>
+        <v>-137822.59320895391</v>
       </c>
       <c r="H11" s="13">
         <f>Model!I54</f>
-        <v>0</v>
+        <v>-142426.21420204811</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -3736,23 +3742,23 @@
       <c r="C12" s="13"/>
       <c r="D12" s="13">
         <f>Model!E53+Model!E6</f>
-        <v>0</v>
+        <v>-125553.39631563395</v>
       </c>
       <c r="E12" s="13">
         <f>Model!F53+Model!F6</f>
-        <v>0</v>
+        <v>-3785.6994555609681</v>
       </c>
       <c r="F12" s="13">
         <f>Model!G53+Model!G6</f>
-        <v>0</v>
+        <v>-4077.4454991796802</v>
       </c>
       <c r="G12" s="13">
         <f>Model!H53+Model!H6</f>
-        <v>0</v>
+        <v>-4406.0519385792704</v>
       </c>
       <c r="H12" s="13">
         <f>Model!I53+Model!I6</f>
-        <v>0</v>
+        <v>-4603.6209930941995</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -3765,23 +3771,23 @@
       <c r="C13" s="50"/>
       <c r="D13" s="50">
         <f>SUM($C10:D10)</f>
-        <v>0</v>
+        <v>-2097.3963156339423</v>
       </c>
       <c r="E13" s="50">
         <f>SUM($C10:E10)</f>
-        <v>0</v>
+        <v>-5883.0957711949104</v>
       </c>
       <c r="F13" s="50">
         <f>SUM($C10:F10)</f>
-        <v>0</v>
+        <v>-9960.5412703745897</v>
       </c>
       <c r="G13" s="50">
         <f>SUM($C10:G10)</f>
-        <v>0</v>
+        <v>-14366.59320895386</v>
       </c>
       <c r="H13" s="50">
         <f>SUM($C10:H10)</f>
-        <v>0</v>
+        <v>-18970.214202048061</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="90" x14ac:dyDescent="0.25">
@@ -3935,7 +3941,7 @@
       </c>
       <c r="E5" s="59">
         <f>'For user (EN)'!D5</f>
-        <v>0</v>
+        <v>123456</v>
       </c>
       <c r="F5" s="59">
         <f>'For user (EN)'!E5</f>
@@ -3968,7 +3974,7 @@
       </c>
       <c r="E6" s="59">
         <f>'For user (EN)'!D6</f>
-        <v>0</v>
+        <v>-123456</v>
       </c>
       <c r="F6" s="59">
         <f>'For user (EN)'!E6</f>
@@ -4340,7 +4346,7 @@
       </c>
       <c r="E20" s="9">
         <f>SUM('Model Quarterly'!H19:K19)</f>
-        <v>0</v>
+        <v>-813.95439603616876</v>
       </c>
       <c r="F20" s="9">
         <f>SUM('Model Quarterly'!L19:O19)</f>
@@ -4374,23 +4380,23 @@
       </c>
       <c r="E21" s="9">
         <f>E53-E20</f>
-        <v>0</v>
+        <v>-1283.4419195977734</v>
       </c>
       <c r="F21" s="9">
         <f>F53-F20</f>
-        <v>0</v>
+        <v>-3785.6994555609681</v>
       </c>
       <c r="G21" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-4077.4454991796802</v>
       </c>
       <c r="H21" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-4406.0519385792704</v>
       </c>
       <c r="I21" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>-4603.6209930941995</v>
       </c>
     </row>
     <row r="22" spans="1:23" ht="26.25" x14ac:dyDescent="0.25">
@@ -4407,23 +4413,23 @@
       </c>
       <c r="E22" s="9">
         <f>-(E6+E20+E21)</f>
-        <v>0</v>
+        <v>125553.39631563393</v>
       </c>
       <c r="F22" s="9">
         <f>-(F6+F20+F21)</f>
-        <v>0</v>
+        <v>3785.6994555609681</v>
       </c>
       <c r="G22" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>4077.4454991796802</v>
       </c>
       <c r="H22" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>4406.0519385792704</v>
       </c>
       <c r="I22" s="9">
         <f>-(I6+I20+I21)</f>
-        <v>0</v>
+        <v>4603.6209930941995</v>
       </c>
     </row>
     <row r="23" spans="1:23" ht="26.25" x14ac:dyDescent="0.25">
@@ -4440,23 +4446,23 @@
       </c>
       <c r="E23" s="9">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>125553.39631563395</v>
       </c>
       <c r="F23" s="9">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>129339.09577119492</v>
       </c>
       <c r="G23" s="9">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>133416.54127037461</v>
       </c>
       <c r="H23" s="9">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>137822.59320895391</v>
       </c>
       <c r="I23" s="9">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>142426.21420204811</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -4497,23 +4503,23 @@
       </c>
       <c r="E26" s="60">
         <f>SUM('Model Quarterly'!H28:K28)</f>
-        <v>0</v>
+        <v>88879.415512061503</v>
       </c>
       <c r="F26" s="60">
         <f>SUM('Model Quarterly'!L28:O28)</f>
-        <v>0</v>
+        <v>25830.01913345986</v>
       </c>
       <c r="G26" s="60">
         <f>SUM('Model Quarterly'!P28:S28)</f>
-        <v>0</v>
+        <v>30231.985080879742</v>
       </c>
       <c r="H26" s="60">
         <f>SUM('Model Quarterly'!T28:W28)</f>
-        <v>0</v>
+        <v>20275.796400470554</v>
       </c>
       <c r="I26" s="60">
         <f>SUM('Model Quarterly'!X28:AA28)</f>
-        <v>0</v>
+        <v>14202.285043145159</v>
       </c>
     </row>
     <row r="27" spans="1:23" ht="26.25" x14ac:dyDescent="0.25">
@@ -4530,23 +4536,23 @@
       </c>
       <c r="E27" s="60">
         <f>SUM('Model Quarterly'!H29:K29)</f>
-        <v>0</v>
+        <v>37292.062452613216</v>
       </c>
       <c r="F27" s="60">
         <f>SUM('Model Quarterly'!L29:O29)</f>
-        <v>0</v>
+        <v>10837.770265787354</v>
       </c>
       <c r="G27" s="60">
         <f>SUM('Model Quarterly'!P29:S29)</f>
-        <v>0</v>
+        <v>12684.748984984504</v>
       </c>
       <c r="H27" s="60">
         <f>SUM('Model Quarterly'!T29:W29)</f>
-        <v>0</v>
+        <v>8507.3271610365955</v>
       </c>
       <c r="I27" s="60">
         <f>SUM('Model Quarterly'!X29:AA29)</f>
-        <v>0</v>
+        <v>5959.0007174035618</v>
       </c>
     </row>
     <row r="28" spans="1:23" ht="26.25" x14ac:dyDescent="0.25">
@@ -4596,23 +4602,23 @@
       </c>
       <c r="E29" s="60">
         <f>SUM('Model Quarterly'!H31:K31)</f>
-        <v>0</v>
+        <v>26104.44371682925</v>
       </c>
       <c r="F29" s="60">
         <f>SUM('Model Quarterly'!L31:O31)</f>
-        <v>0</v>
+        <v>7586.4391860511469</v>
       </c>
       <c r="G29" s="60">
         <f>SUM('Model Quarterly'!P31:S31)</f>
-        <v>0</v>
+        <v>8879.3242894891519</v>
       </c>
       <c r="H29" s="60">
         <f>SUM('Model Quarterly'!T31:W31)</f>
-        <v>0</v>
+        <v>5955.1290127256152</v>
       </c>
       <c r="I29" s="60">
         <f>SUM('Model Quarterly'!X31:AA31)</f>
-        <v>0</v>
+        <v>4171.3005021824929</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
@@ -4629,23 +4635,23 @@
       </c>
       <c r="E30" s="131">
         <f t="shared" ref="E30:I30" si="4">SUM(E27:E29)</f>
-        <v>0</v>
+        <v>63396.506169442466</v>
       </c>
       <c r="F30" s="131">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>18424.209451838502</v>
       </c>
       <c r="G30" s="131">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>21564.073274473656</v>
       </c>
       <c r="H30" s="131">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>14462.45617376221</v>
       </c>
       <c r="I30" s="131">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>10130.301219586054</v>
       </c>
     </row>
     <row r="31" spans="1:23" ht="26.25" x14ac:dyDescent="0.25">
@@ -4662,23 +4668,23 @@
       </c>
       <c r="E31" s="60">
         <f>SUM('Model Quarterly'!H32:K32)</f>
-        <v>0</v>
+        <v>35116.692142877444</v>
       </c>
       <c r="F31" s="60">
         <f>SUM('Model Quarterly'!L32:O32)</f>
-        <v>0</v>
+        <v>10205.56700028309</v>
       </c>
       <c r="G31" s="60">
         <f>SUM('Model Quarterly'!P32:S32)</f>
-        <v>0</v>
+        <v>11944.805294193742</v>
       </c>
       <c r="H31" s="60">
         <f>SUM('Model Quarterly'!T32:W32)</f>
-        <v>0</v>
+        <v>8011.066409976127</v>
       </c>
       <c r="I31" s="60">
         <f>SUM('Model Quarterly'!X32:AA32)</f>
-        <v>0</v>
+        <v>5611.3923422216876</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
@@ -4706,23 +4712,23 @@
       </c>
       <c r="E33" s="60">
         <f>SUM('Model Quarterly'!H55:K55)</f>
-        <v>0</v>
+        <v>61839.217508747482</v>
       </c>
       <c r="F33" s="60">
         <f>SUM('Model Quarterly'!L55:O55)</f>
-        <v>0</v>
+        <v>50674.096130020487</v>
       </c>
       <c r="G33" s="60">
         <f>SUM('Model Quarterly'!P55:S55)</f>
-        <v>0</v>
+        <v>22371.355697754247</v>
       </c>
       <c r="H33" s="60">
         <f>SUM('Model Quarterly'!T55:W55)</f>
-        <v>0</v>
+        <v>27505.496779842266</v>
       </c>
       <c r="I33" s="60">
         <f>SUM('Model Quarterly'!X55:AA55)</f>
-        <v>0</v>
+        <v>12655.608626874198</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -4747,15 +4753,15 @@
       </c>
       <c r="G34" s="60">
         <f>SUM('Model Quarterly'!P56:S56)</f>
-        <v>0</v>
+        <v>37292.062452613216</v>
       </c>
       <c r="H34" s="60">
         <f>SUM('Model Quarterly'!T56:W56)</f>
-        <v>0</v>
+        <v>10837.770265787354</v>
       </c>
       <c r="I34" s="60">
         <f>SUM('Model Quarterly'!X56:AA56)</f>
-        <v>0</v>
+        <v>12684.748984984504</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -4846,15 +4852,15 @@
       </c>
       <c r="G37" s="60">
         <f>SUM('Model Quarterly'!P59:S59)</f>
-        <v>0</v>
+        <v>37292.062452613216</v>
       </c>
       <c r="H37" s="60">
         <f>SUM('Model Quarterly'!T59:W59)</f>
-        <v>0</v>
+        <v>10837.770265787354</v>
       </c>
       <c r="I37" s="60">
         <f>SUM('Model Quarterly'!X59:AA59)</f>
-        <v>0</v>
+        <v>12684.748984984504</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -4882,23 +4888,23 @@
       </c>
       <c r="E39" s="60">
         <f>'Model Quarterly'!K36</f>
-        <v>0</v>
+        <v>27040.198003314028</v>
       </c>
       <c r="F39" s="60">
         <f>'Model Quarterly'!O36</f>
-        <v>0</v>
+        <v>2196.1210067534025</v>
       </c>
       <c r="G39" s="60">
         <f>'Model Quarterly'!S36</f>
-        <v>0</v>
+        <v>10056.750389878895</v>
       </c>
       <c r="H39" s="60">
         <f>'Model Quarterly'!W36</f>
-        <v>0</v>
+        <v>2827.0500105071801</v>
       </c>
       <c r="I39" s="60">
         <f>'Model Quarterly'!AA36</f>
-        <v>0</v>
+        <v>4373.7264267781402</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="26.25" x14ac:dyDescent="0.25">
@@ -4915,23 +4921,23 @@
       </c>
       <c r="E40" s="60">
         <f>'Model Quarterly'!K37</f>
-        <v>0</v>
+        <v>37292.062452613216</v>
       </c>
       <c r="F40" s="60">
         <f>'Model Quarterly'!O37</f>
-        <v>0</v>
+        <v>48129.832718400576</v>
       </c>
       <c r="G40" s="60">
         <f>'Model Quarterly'!S37</f>
-        <v>0</v>
+        <v>23522.519250771864</v>
       </c>
       <c r="H40" s="60">
         <f>'Model Quarterly'!W37</f>
-        <v>0</v>
+        <v>21192.076146021111</v>
       </c>
       <c r="I40" s="60">
         <f>'Model Quarterly'!AA37</f>
-        <v>0</v>
+        <v>14466.32787844017</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="26.25" x14ac:dyDescent="0.25">
@@ -4981,23 +4987,23 @@
       </c>
       <c r="E42" s="60">
         <f>'Model Quarterly'!K39</f>
-        <v>0</v>
+        <v>26104.44371682925</v>
       </c>
       <c r="F42" s="60">
         <f>'Model Quarterly'!O39</f>
-        <v>0</v>
+        <v>33690.882902880396</v>
       </c>
       <c r="G42" s="60">
         <f>'Model Quarterly'!S39</f>
-        <v>0</v>
+        <v>42570.207192369548</v>
       </c>
       <c r="H42" s="60">
         <f>'Model Quarterly'!W39</f>
-        <v>0</v>
+        <v>48525.336205095162</v>
       </c>
       <c r="I42" s="60">
         <f>'Model Quarterly'!AA39</f>
-        <v>0</v>
+        <v>52696.636707277656</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -5014,23 +5020,23 @@
       </c>
       <c r="E43" s="60">
         <f>'Model Quarterly'!K40</f>
-        <v>0</v>
+        <v>63396.506169442466</v>
       </c>
       <c r="F43" s="60">
         <f>'Model Quarterly'!O40</f>
-        <v>0</v>
+        <v>81820.715621280979</v>
       </c>
       <c r="G43" s="60">
         <f>'Model Quarterly'!S40</f>
-        <v>0</v>
+        <v>66092.726443141408</v>
       </c>
       <c r="H43" s="60">
         <f>'Model Quarterly'!W40</f>
-        <v>0</v>
+        <v>69717.412351116276</v>
       </c>
       <c r="I43" s="60">
         <f>'Model Quarterly'!AA40</f>
-        <v>0</v>
+        <v>67162.964585717826</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="26.25" x14ac:dyDescent="0.25">
@@ -5047,23 +5053,23 @@
       </c>
       <c r="E44" s="60">
         <f>'Model Quarterly'!K41</f>
-        <v>0</v>
+        <v>35116.692142877444</v>
       </c>
       <c r="F44" s="60">
         <f>'Model Quarterly'!O41</f>
-        <v>0</v>
+        <v>45322.259143160532</v>
       </c>
       <c r="G44" s="60">
         <f>'Model Quarterly'!S41</f>
-        <v>0</v>
+        <v>57267.064437354275</v>
       </c>
       <c r="H44" s="60">
         <f>'Model Quarterly'!W41</f>
-        <v>0</v>
+        <v>65278.130847330402</v>
       </c>
       <c r="I44" s="60">
         <f>'Model Quarterly'!AA41</f>
-        <v>0</v>
+        <v>70889.523189552085</v>
       </c>
       <c r="J44" s="67"/>
     </row>
@@ -5081,23 +5087,23 @@
       </c>
       <c r="E45" s="58">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.21536811266607667</v>
       </c>
       <c r="F45" s="58">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1.6979560539362455E-2</v>
       </c>
       <c r="G45" s="58">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>7.5378587198557626E-2</v>
       </c>
       <c r="H45" s="58">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>2.051223928301122E-2</v>
       </c>
       <c r="I45" s="58">
         <f>IF(I23=0,0,I39/I23)</f>
-        <v>0</v>
+        <v>3.0708717852835025E-2</v>
       </c>
       <c r="J45" s="66"/>
       <c r="K45" s="66"/>
@@ -5119,23 +5125,23 @@
       </c>
       <c r="E46" s="58">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.29702153463744729</v>
       </c>
       <c r="F46" s="58">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.37212130200402688</v>
       </c>
       <c r="G46" s="58">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.17630886715240521</v>
       </c>
       <c r="H46" s="58">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.15376344075816104</v>
       </c>
       <c r="I46" s="58">
         <f>IF(I$23=0,0,I40/I$23)</f>
-        <v>0</v>
+        <v>0.10157068317436287</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -5185,23 +5191,23 @@
       </c>
       <c r="E48" s="58">
         <f t="shared" ref="E48:H48" si="7">IF(E$23=0,0,E42/E$23)</f>
-        <v>0</v>
+        <v>0.20791507424621311</v>
       </c>
       <c r="F48" s="58">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.26048491140281876</v>
       </c>
       <c r="G48" s="58">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.31907743063207666</v>
       </c>
       <c r="H48" s="58">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>0.35208549683523599</v>
       </c>
       <c r="I48" s="58">
         <f>IF(I$23=0,0,I42/I$23)</f>
-        <v>0</v>
+        <v>0.36999253966352963</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
@@ -5218,23 +5224,23 @@
       </c>
       <c r="E49" s="58">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>0.27969527845026287</v>
       </c>
       <c r="F49" s="58">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>0.35041422605379186</v>
       </c>
       <c r="G49" s="58">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>0.42923511501696027</v>
       </c>
       <c r="H49" s="58">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>0.47363882312359135</v>
       </c>
       <c r="I49" s="58">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>0.49772805930927205</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -5280,23 +5286,23 @@
       </c>
       <c r="E53" s="13">
         <f>SUM('Model Quarterly'!H74:K74)</f>
-        <v>0</v>
+        <v>-2097.3963156339423</v>
       </c>
       <c r="F53" s="13">
         <f>SUM('Model Quarterly'!L74:O74)</f>
-        <v>0</v>
+        <v>-3785.6994555609681</v>
       </c>
       <c r="G53" s="13">
         <f>SUM('Model Quarterly'!P74:S74)</f>
-        <v>0</v>
+        <v>-4077.4454991796802</v>
       </c>
       <c r="H53" s="13">
         <f>SUM('Model Quarterly'!T74:W74)</f>
-        <v>0</v>
+        <v>-4406.0519385792704</v>
       </c>
       <c r="I53" s="13">
         <f>SUM('Model Quarterly'!X74:AA74)</f>
-        <v>0</v>
+        <v>-4603.6209930941995</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5311,23 +5317,23 @@
       </c>
       <c r="E54" s="13">
         <f>'Model Quarterly'!K75</f>
-        <v>0</v>
+        <v>-125553.39631563395</v>
       </c>
       <c r="F54" s="13">
         <f>'Model Quarterly'!O75</f>
-        <v>0</v>
+        <v>-129339.09577119492</v>
       </c>
       <c r="G54" s="13">
         <f>'Model Quarterly'!S75</f>
-        <v>0</v>
+        <v>-133416.54127037461</v>
       </c>
       <c r="H54" s="13">
         <f>'Model Quarterly'!W75</f>
-        <v>0</v>
+        <v>-137822.59320895391</v>
       </c>
       <c r="I54" s="13">
         <f>'Model Quarterly'!AA75</f>
-        <v>0</v>
+        <v>-142426.21420204811</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5342,23 +5348,23 @@
       </c>
       <c r="E55" s="13">
         <f>SUM($D53:E53)</f>
-        <v>0</v>
+        <v>-2097.3963156339423</v>
       </c>
       <c r="F55" s="13">
         <f>SUM($D53:F53)</f>
-        <v>0</v>
+        <v>-5883.0957711949104</v>
       </c>
       <c r="G55" s="13">
         <f>SUM($D53:G53)</f>
-        <v>0</v>
+        <v>-9960.5412703745897</v>
       </c>
       <c r="H55" s="13">
         <f>SUM($D53:H53)</f>
-        <v>0</v>
+        <v>-14366.59320895386</v>
       </c>
       <c r="I55" s="13">
         <f>SUM($D53:I53)</f>
-        <v>0</v>
+        <v>-18970.214202048061</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5825,19 +5831,19 @@
       </c>
       <c r="H6" s="59">
         <f>'For user (EN)'!D5/4</f>
-        <v>0</v>
+        <v>30864</v>
       </c>
       <c r="I6" s="59">
         <f>'For user (EN)'!$D5/4</f>
-        <v>0</v>
+        <v>30864</v>
       </c>
       <c r="J6" s="59">
         <f>'For user (EN)'!$D5/4</f>
-        <v>0</v>
+        <v>30864</v>
       </c>
       <c r="K6" s="59">
         <f>'For user (EN)'!$D5/4</f>
-        <v>0</v>
+        <v>30864</v>
       </c>
       <c r="L6" s="4">
         <f>'For user (EN)'!$E5/4</f>
@@ -5930,19 +5936,19 @@
       </c>
       <c r="H7" s="59">
         <f>'For user (EN)'!D6/4</f>
-        <v>0</v>
+        <v>-30864</v>
       </c>
       <c r="I7" s="59">
         <f>'For user (EN)'!$D6/4</f>
-        <v>0</v>
+        <v>-30864</v>
       </c>
       <c r="J7" s="59">
         <f>'For user (EN)'!$D6/4</f>
-        <v>0</v>
+        <v>-30864</v>
       </c>
       <c r="K7" s="59">
         <f>'For user (EN)'!$D6/4</f>
-        <v>0</v>
+        <v>-30864</v>
       </c>
       <c r="L7" s="4">
         <f>'For user (EN)'!$E6/4</f>
@@ -6787,19 +6793,19 @@
       </c>
       <c r="H19" s="9">
         <f>(H16/100)*H7/4</f>
-        <v>0</v>
+        <v>-201.81034552475003</v>
       </c>
       <c r="I19" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-202.52156529639294</v>
       </c>
       <c r="J19" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-204.02013832074425</v>
       </c>
       <c r="K19" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-205.60234689428162</v>
       </c>
       <c r="L19" s="9">
         <f>(L16/100)*L7/4</f>
@@ -6896,79 +6902,79 @@
       </c>
       <c r="I20" s="9">
         <f>(H71/100)*H75/4</f>
-        <v>0</v>
+        <v>-203.12992223421153</v>
       </c>
       <c r="J20" s="9">
         <f>(I71/100)*I75/4</f>
-        <v>0</v>
+        <v>-423.95734198623109</v>
       </c>
       <c r="K20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-656.35465537733103</v>
       </c>
       <c r="L20" s="9">
         <f>(K71/100)*K75/4</f>
-        <v>0</v>
+        <v>-897.06941973413893</v>
       </c>
       <c r="M20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-944.93078222515908</v>
       </c>
       <c r="N20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-963.97265559273126</v>
       </c>
       <c r="O20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-979.72659800893848</v>
       </c>
       <c r="P20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-989.37120580302053</v>
       </c>
       <c r="Q20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1006.5780005652127</v>
       </c>
       <c r="R20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1028.694808936199</v>
       </c>
       <c r="S20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1052.8014838752481</v>
       </c>
       <c r="T20" s="9">
         <f>(S71/100)*S75/4</f>
-        <v>0</v>
+        <v>-1077.2722536865842</v>
       </c>
       <c r="U20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1095.497885214302</v>
       </c>
       <c r="V20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1110.4200784701648</v>
       </c>
       <c r="W20" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1122.8617212082197</v>
       </c>
       <c r="X20" s="9">
         <f>(W71/100)*W75/4</f>
-        <v>0</v>
+        <v>-1134.0669699318119</v>
       </c>
       <c r="Y20" s="9">
         <f t="shared" ref="Y20" si="3">(X71/100)*X75/4</f>
-        <v>0</v>
+        <v>-1144.9765154434508</v>
       </c>
       <c r="Z20" s="9">
         <f t="shared" ref="Z20" si="4">(Y71/100)*Y75/4</f>
-        <v>0</v>
+        <v>-1156.2945269574238</v>
       </c>
       <c r="AA20" s="9">
         <f t="shared" ref="AA20" si="5">(Z71/100)*Z75/4</f>
-        <v>0</v>
+        <v>-1168.2829807615133</v>
       </c>
     </row>
     <row r="21" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -6997,83 +7003,83 @@
       </c>
       <c r="H21" s="9">
         <f>-(H7+H19+H20)</f>
-        <v>0</v>
+        <v>31065.810345524751</v>
       </c>
       <c r="I21" s="9">
         <f>-(I7+I19+I20)</f>
-        <v>0</v>
+        <v>31269.651487530606</v>
       </c>
       <c r="J21" s="9">
         <f>-(J7+J19+J20)</f>
-        <v>0</v>
+        <v>31491.977480306978</v>
       </c>
       <c r="K21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>31725.957002271611</v>
       </c>
       <c r="L21" s="9">
         <f>-(L7+L19+L20)</f>
-        <v>0</v>
+        <v>897.06941973413893</v>
       </c>
       <c r="M21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>944.93078222515908</v>
       </c>
       <c r="N21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>963.97265559273126</v>
       </c>
       <c r="O21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>979.72659800893848</v>
       </c>
       <c r="P21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>989.37120580302053</v>
       </c>
       <c r="Q21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>1006.5780005652127</v>
       </c>
       <c r="R21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>1028.694808936199</v>
       </c>
       <c r="S21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>1052.8014838752481</v>
       </c>
       <c r="T21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>1077.2722536865842</v>
       </c>
       <c r="U21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>1095.497885214302</v>
       </c>
       <c r="V21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>1110.4200784701648</v>
       </c>
       <c r="W21" s="9">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>1122.8617212082197</v>
       </c>
       <c r="X21" s="9">
         <f t="shared" ref="X21:AA21" si="7">-(X7+X19+X20)</f>
-        <v>0</v>
+        <v>1134.0669699318119</v>
       </c>
       <c r="Y21" s="9">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1144.9765154434508</v>
       </c>
       <c r="Z21" s="9">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1156.2945269574238</v>
       </c>
       <c r="AA21" s="9">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1168.2829807615133</v>
       </c>
     </row>
     <row r="22" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -7102,83 +7108,83 @@
       </c>
       <c r="H22" s="9">
         <f>MAX(0,SUM($D21:H21))</f>
-        <v>0</v>
+        <v>31065.810345524751</v>
       </c>
       <c r="I22" s="9">
         <f>MAX(0,SUM($D21:I21))</f>
-        <v>0</v>
+        <v>62335.461833055357</v>
       </c>
       <c r="J22" s="9">
         <f>MAX(0,SUM($D21:J21))</f>
-        <v>0</v>
+        <v>93827.439313362338</v>
       </c>
       <c r="K22" s="9">
         <f>MAX(0,SUM($D21:K21))</f>
-        <v>0</v>
+        <v>125553.39631563395</v>
       </c>
       <c r="L22" s="9">
         <f>MAX(0,SUM($D21:L21))</f>
-        <v>0</v>
+        <v>126450.46573536808</v>
       </c>
       <c r="M22" s="9">
         <f>MAX(0,SUM($D21:M21))</f>
-        <v>0</v>
+        <v>127395.39651759324</v>
       </c>
       <c r="N22" s="9">
         <f>MAX(0,SUM($D21:N21))</f>
-        <v>0</v>
+        <v>128359.36917318597</v>
       </c>
       <c r="O22" s="9">
         <f>MAX(0,SUM($D21:O21))</f>
-        <v>0</v>
+        <v>129339.09577119492</v>
       </c>
       <c r="P22" s="9">
         <f>MAX(0,SUM($D21:P21))</f>
-        <v>0</v>
+        <v>130328.46697699794</v>
       </c>
       <c r="Q22" s="9">
         <f>MAX(0,SUM($D21:Q21))</f>
-        <v>0</v>
+        <v>131335.04497756314</v>
       </c>
       <c r="R22" s="9">
         <f>MAX(0,SUM($D21:R21))</f>
-        <v>0</v>
+        <v>132363.73978649935</v>
       </c>
       <c r="S22" s="9">
         <f>MAX(0,SUM($D21:S21))</f>
-        <v>0</v>
+        <v>133416.54127037461</v>
       </c>
       <c r="T22" s="9">
         <f>MAX(0,SUM($D21:T21))</f>
-        <v>0</v>
+        <v>134493.8135240612</v>
       </c>
       <c r="U22" s="9">
         <f>MAX(0,SUM($D21:U21))</f>
-        <v>0</v>
+        <v>135589.31140927551</v>
       </c>
       <c r="V22" s="9">
         <f>MAX(0,SUM($D21:V21))</f>
-        <v>0</v>
+        <v>136699.73148774568</v>
       </c>
       <c r="W22" s="9">
         <f>MAX(0,SUM($D21:W21))</f>
-        <v>0</v>
+        <v>137822.59320895391</v>
       </c>
       <c r="X22" s="9">
         <f>MAX(0,SUM($D21:X21))</f>
-        <v>0</v>
+        <v>138956.66017888574</v>
       </c>
       <c r="Y22" s="9">
         <f>MAX(0,SUM($D21:Y21))</f>
-        <v>0</v>
+        <v>140101.63669432918</v>
       </c>
       <c r="Z22" s="9">
         <f>MAX(0,SUM($D21:Z21))</f>
-        <v>0</v>
+        <v>141257.93122128659</v>
       </c>
       <c r="AA22" s="9">
         <f>MAX(0,SUM($D21:AA21))</f>
-        <v>0</v>
+        <v>142426.21420204811</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
@@ -7267,83 +7273,83 @@
       </c>
       <c r="H25" s="9">
         <f>IF(H$22&gt;0,MIN(MAX(SUM(H$21,H$55,H$59),0),H$22)*'Fiscal Model Import'!S44,0)</f>
-        <v>0</v>
+        <v>14734.364442487693</v>
       </c>
       <c r="I25" s="9">
         <f>IF(I$22&gt;0,MIN(MAX(SUM(I$21,I$55,I$59),0),I$22)*'Fiscal Model Import'!T44,0)</f>
-        <v>0</v>
+        <v>21819.483509096575</v>
       </c>
       <c r="J25" s="9">
         <f>IF(J$22&gt;0,MIN(MAX(SUM(J$21,J$55,J$59),0),J$22)*'Fiscal Model Import'!U44,0)</f>
-        <v>0</v>
+        <v>25285.369557163212</v>
       </c>
       <c r="K25" s="9">
         <f>IF(K$22&gt;0,MIN(MAX(SUM(K$21,K$55,K$59),0),K$22)*'Fiscal Model Import'!V44,0)</f>
-        <v>0</v>
+        <v>27040.198003314028</v>
       </c>
       <c r="L25" s="9">
         <f>IF(L$22&gt;0,MIN(MAX(SUM(L$21,L$55,L$59),0),L$22)*'Fiscal Model Import'!W44,0)</f>
-        <v>0</v>
+        <v>13250.511580417538</v>
       </c>
       <c r="M25" s="9">
         <f>IF(M$22&gt;0,MIN(MAX(SUM(M$21,M$55,M$59),0),M$22)*'Fiscal Model Import'!X44,0)</f>
-        <v>0</v>
+        <v>6732.8300426464539</v>
       </c>
       <c r="N25" s="9">
         <f>IF(N$22&gt;0,MIN(MAX(SUM(N$21,N$55,N$59),0),N$22)*'Fiscal Model Import'!Y44,0)</f>
-        <v>0</v>
+        <v>3650.5565036424659</v>
       </c>
       <c r="O25" s="9">
         <f>IF(O$22&gt;0,MIN(MAX(SUM(O$21,O$55,O$59),0),O$22)*'Fiscal Model Import'!Z44,0)</f>
-        <v>0</v>
+        <v>2196.1210067534025</v>
       </c>
       <c r="P25" s="9">
         <f>IF(P$22&gt;0,MIN(MAX(SUM(P$21,P$55,P$59),0),P$22)*'Fiscal Model Import'!AA44,0)</f>
-        <v>0</v>
+        <v>4443.0754658203323</v>
       </c>
       <c r="Q25" s="9">
         <f>IF(Q$22&gt;0,MIN(MAX(SUM(Q$21,Q$55,Q$59),0),Q$22)*'Fiscal Model Import'!AB44,0)</f>
-        <v>0</v>
+        <v>6926.930203114187</v>
       </c>
       <c r="R25" s="9">
         <f>IF(R$22&gt;0,MIN(MAX(SUM(R$21,R$55,R$59),0),R$22)*'Fiscal Model Import'!AC44,0)</f>
-        <v>0</v>
+        <v>8805.2290220663272</v>
       </c>
       <c r="S25" s="9">
         <f>IF(S$22&gt;0,MIN(MAX(SUM(S$21,S$55,S$59),0),S$22)*'Fiscal Model Import'!AD44,0)</f>
-        <v>0</v>
+        <v>10056.750389878895</v>
       </c>
       <c r="T25" s="9">
         <f>IF(T$22&gt;0,MIN(MAX(SUM(T$21,T$55,T$59),0),T$22)*'Fiscal Model Import'!AE44,0)</f>
-        <v>0</v>
+        <v>7917.7311205801516</v>
       </c>
       <c r="U25" s="9">
         <f>IF(U$22&gt;0,MIN(MAX(SUM(U$21,U$55,U$59),0),U$22)*'Fiscal Model Import'!AF44,0)</f>
-        <v>0</v>
+        <v>5614.7978453976593</v>
       </c>
       <c r="V25" s="9">
         <f>IF(V$22&gt;0,MIN(MAX(SUM(V$21,V$55,V$59),0),V$22)*'Fiscal Model Import'!AG44,0)</f>
-        <v>0</v>
+        <v>3916.2174239855613</v>
       </c>
       <c r="W25" s="9">
         <f>IF(W$22&gt;0,MIN(MAX(SUM(W$21,W$55,W$59),0),W$22)*'Fiscal Model Import'!AH44,0)</f>
-        <v>0</v>
+        <v>2827.0500105071801</v>
       </c>
       <c r="X25" s="9">
         <f>IF(X$22&gt;0,MIN(MAX(SUM(X$21,X$55,X$59),0),X$22)*'Fiscal Model Import'!AI44,0)</f>
-        <v>0</v>
+        <v>2762.932856225525</v>
       </c>
       <c r="Y25" s="9">
         <f>IF(Y$22&gt;0,MIN(MAX(SUM(Y$21,Y$55,Y$59),0),Y$22)*'Fiscal Model Import'!AJ44,0)</f>
-        <v>0</v>
+        <v>3231.9961934842941</v>
       </c>
       <c r="Z25" s="9">
         <f>IF(Z$22&gt;0,MIN(MAX(SUM(Z$21,Z$55,Z$59),0),Z$22)*'Fiscal Model Import'!AK44,0)</f>
-        <v>0</v>
+        <v>3833.6295666571982</v>
       </c>
       <c r="AA25" s="9">
         <f>IF(AA$22&gt;0,MIN(MAX(SUM(AA$21,AA$55,AA$59),0),AA$22)*'Fiscal Model Import'!AL44,0)</f>
-        <v>0</v>
+        <v>4373.7264267781402</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.25">
@@ -7430,83 +7436,83 @@
       </c>
       <c r="H28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>14734.364442487693</v>
       </c>
       <c r="I28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>21819.483509096575</v>
       </c>
       <c r="J28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>25285.369557163212</v>
       </c>
       <c r="K28" s="9">
         <f>SUM(K25:K27)</f>
-        <v>0</v>
+        <v>27040.198003314028</v>
       </c>
       <c r="L28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>13250.511580417538</v>
       </c>
       <c r="M28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>6732.8300426464539</v>
       </c>
       <c r="N28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>3650.5565036424659</v>
       </c>
       <c r="O28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>2196.1210067534025</v>
       </c>
       <c r="P28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>4443.0754658203323</v>
       </c>
       <c r="Q28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>6926.930203114187</v>
       </c>
       <c r="R28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>8805.2290220663272</v>
       </c>
       <c r="S28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>10056.750389878895</v>
       </c>
       <c r="T28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>7917.7311205801516</v>
       </c>
       <c r="U28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>5614.7978453976593</v>
       </c>
       <c r="V28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>3916.2174239855613</v>
       </c>
       <c r="W28" s="9">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>2827.0500105071801</v>
       </c>
       <c r="X28" s="9">
         <f t="shared" ref="X28:AA28" si="9">SUM(X25:X27)</f>
-        <v>0</v>
+        <v>2762.932856225525</v>
       </c>
       <c r="Y28" s="9">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>3231.9961934842941</v>
       </c>
       <c r="Z28" s="9">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>3833.6295666571982</v>
       </c>
       <c r="AA28" s="9">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>4373.7264267781402</v>
       </c>
     </row>
     <row r="29" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -7535,83 +7541,83 @@
       </c>
       <c r="H29" s="60">
         <f>IF(H22&gt;0,MIN(H22,MAX(0,SUM(H$21,H$55,H$59)))*'Fiscal Model Import'!S38,0)</f>
-        <v>0</v>
+        <v>6182.2508150298008</v>
       </c>
       <c r="I29" s="60">
         <f>IF(I22&gt;0,MIN(I22,MAX(0,SUM(I$21,I$55,I$59)))*'Fiscal Model Import'!T38,0)</f>
-        <v>0</v>
+        <v>9155.0280457747849</v>
       </c>
       <c r="J29" s="60">
         <f>IF(J22&gt;0,MIN(J22,MAX(0,SUM(J$21,J$55,J$59)))*'Fiscal Model Import'!U38,0)</f>
-        <v>0</v>
+        <v>10609.245968040506</v>
       </c>
       <c r="K29" s="60">
         <f>IF(K22&gt;0,MIN(K22,MAX(0,SUM(K$21,K$55,K$59)))*'Fiscal Model Import'!V38,0)</f>
-        <v>0</v>
+        <v>11345.537623768123</v>
       </c>
       <c r="L29" s="60">
         <f>IF(L22&gt;0,MIN(L22,MAX(0,SUM(L$21,L$55,L$59)))*'Fiscal Model Import'!W38,0)</f>
-        <v>0</v>
+        <v>5559.655208566799</v>
       </c>
       <c r="M29" s="60">
         <f>IF(M22&gt;0,MIN(M22,MAX(0,SUM(M$21,M$55,M$59)))*'Fiscal Model Import'!X38,0)</f>
-        <v>0</v>
+        <v>2824.963654257253</v>
       </c>
       <c r="N29" s="60">
         <f>IF(N22&gt;0,MIN(N22,MAX(0,SUM(N$21,N$55,N$59)))*'Fiscal Model Import'!Y38,0)</f>
-        <v>0</v>
+        <v>1531.7020295003351</v>
       </c>
       <c r="O29" s="60">
         <f>IF(O22&gt;0,MIN(O22,MAX(0,SUM(O$21,O$55,O$59)))*'Fiscal Model Import'!Z38,0)</f>
-        <v>0</v>
+        <v>921.44937346296604</v>
       </c>
       <c r="P29" s="60">
         <f>IF(P22&gt;0,MIN(P22,MAX(0,SUM(P$21,P$55,P$59)))*'Fiscal Model Import'!AA38,0)</f>
-        <v>0</v>
+        <v>1864.2274681763629</v>
       </c>
       <c r="Q29" s="60">
         <f>IF(Q22&gt;0,MIN(Q22,MAX(0,SUM(Q$21,Q$55,Q$59)))*'Fiscal Model Import'!AB38,0)</f>
-        <v>0</v>
+        <v>2906.4042810269311</v>
       </c>
       <c r="R29" s="60">
         <f>IF(R22&gt;0,MIN(R22,MAX(0,SUM(R$21,R$55,R$59)))*'Fiscal Model Import'!AC38,0)</f>
-        <v>0</v>
+        <v>3694.5016875802767</v>
       </c>
       <c r="S29" s="60">
         <f>IF(S22&gt;0,MIN(S22,MAX(0,SUM(S$21,S$55,S$59)))*'Fiscal Model Import'!AD38,0)</f>
-        <v>0</v>
+        <v>4219.6155482009344</v>
       </c>
       <c r="T29" s="60">
         <f>IF(T22&gt;0,MIN(T22,MAX(0,SUM(T$21,T$55,T$59)))*'Fiscal Model Import'!AE38,0)</f>
-        <v>0</v>
+        <v>3322.1249456979654</v>
       </c>
       <c r="U29" s="60">
         <f>IF(U22&gt;0,MIN(U22,MAX(0,SUM(U$21,U$55,U$59)))*'Fiscal Model Import'!AF38,0)</f>
-        <v>0</v>
+        <v>2355.8592358311853</v>
       </c>
       <c r="V29" s="60">
         <f>IF(V22&gt;0,MIN(V22,MAX(0,SUM(V$21,V$55,V$59)))*'Fiscal Model Import'!AG38,0)</f>
-        <v>0</v>
+        <v>1643.1681499240115</v>
       </c>
       <c r="W29" s="60">
         <f>IF(W22&gt;0,MIN(W22,MAX(0,SUM(W$21,W$55,W$59)))*'Fiscal Model Import'!AH38,0)</f>
-        <v>0</v>
+        <v>1186.1748295834323</v>
       </c>
       <c r="X29" s="60">
         <f>IF(X22&gt;0,MIN(X22,MAX(0,SUM(X$21,X$55,X$59)))*'Fiscal Model Import'!AI38,0)</f>
-        <v>0</v>
+        <v>1159.2725270876326</v>
       </c>
       <c r="Y29" s="60">
         <f>IF(Y22&gt;0,MIN(Y22,MAX(0,SUM(Y$21,Y$55,Y$59)))*'Fiscal Model Import'!AJ38,0)</f>
-        <v>0</v>
+        <v>1356.0823189444591</v>
       </c>
       <c r="Z29" s="60">
         <f>IF(Z22&gt;0,MIN(Z22,MAX(0,SUM(Z$21,Z$55,Z$59)))*'Fiscal Model Import'!AK38,0)</f>
-        <v>0</v>
+        <v>1608.5159020939291</v>
       </c>
       <c r="AA29" s="60">
         <f>IF(AA22&gt;0,MIN(AA22,MAX(0,SUM(AA$21,AA$55,AA$59)))*'Fiscal Model Import'!AL38,0)</f>
-        <v>0</v>
+        <v>1835.1299692775412</v>
       </c>
     </row>
     <row r="30" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -7745,83 +7751,83 @@
       </c>
       <c r="H31" s="60">
         <f>IF(H22&gt;0,MIN(H22,MAX(SUM(H$21,H$55,H$59),0))*'Fiscal Model Import'!S40,0)</f>
-        <v>0</v>
+        <v>4327.5755705208603</v>
       </c>
       <c r="I31" s="60">
         <f>IF(I22&gt;0,MIN(I22,MAX(SUM(I$21,I$55,I$59),0))*'Fiscal Model Import'!T40,0)</f>
-        <v>0</v>
+        <v>6408.5196320423493</v>
       </c>
       <c r="J31" s="60">
         <f>IF(J22&gt;0,MIN(J22,MAX(SUM(J$21,J$55,J$59),0))*'Fiscal Model Import'!U40,0)</f>
-        <v>0</v>
+        <v>7426.4721776283541</v>
       </c>
       <c r="K31" s="60">
         <f>IF(K22&gt;0,MIN(K22,MAX(SUM(K$21,K$55,K$59),0))*'Fiscal Model Import'!V40,0)</f>
-        <v>0</v>
+        <v>7941.8763366376852</v>
       </c>
       <c r="L31" s="60">
         <f>IF(L22&gt;0,MIN(L22,MAX(SUM(L$21,L$55,L$59),0))*'Fiscal Model Import'!W40,0)</f>
-        <v>0</v>
+        <v>3891.7586459967592</v>
       </c>
       <c r="M31" s="60">
         <f>IF(M22&gt;0,MIN(M22,MAX(SUM(M$21,M$55,M$59),0))*'Fiscal Model Import'!X40,0)</f>
-        <v>0</v>
+        <v>1977.474557980077</v>
       </c>
       <c r="N31" s="60">
         <f>IF(N22&gt;0,MIN(N22,MAX(SUM(N$21,N$55,N$59),0))*'Fiscal Model Import'!Y40,0)</f>
-        <v>0</v>
+        <v>1072.1914206502345</v>
       </c>
       <c r="O31" s="60">
         <f>IF(O22&gt;0,MIN(O22,MAX(SUM(O$21,O$55,O$59),0))*'Fiscal Model Import'!Z40,0)</f>
-        <v>0</v>
+        <v>645.01456142407619</v>
       </c>
       <c r="P31" s="60">
         <f>IF(P22&gt;0,MIN(P22,MAX(SUM(P$21,P$55,P$59),0))*'Fiscal Model Import'!AA40,0)</f>
-        <v>0</v>
+        <v>1304.959227723454</v>
       </c>
       <c r="Q31" s="60">
         <f>IF(Q22&gt;0,MIN(Q22,MAX(SUM(Q$21,Q$55,Q$59),0))*'Fiscal Model Import'!AB40,0)</f>
-        <v>0</v>
+        <v>2034.4829967188516</v>
       </c>
       <c r="R31" s="60">
         <f>IF(R22&gt;0,MIN(R22,MAX(SUM(R$21,R$55,R$59),0))*'Fiscal Model Import'!AC40,0)</f>
-        <v>0</v>
+        <v>2586.1511813061934</v>
       </c>
       <c r="S31" s="60">
         <f>IF(S22&gt;0,MIN(S22,MAX(SUM(S$21,S$55,S$59),0))*'Fiscal Model Import'!AD40,0)</f>
-        <v>0</v>
+        <v>2953.7308837406536</v>
       </c>
       <c r="T31" s="60">
         <f>IF(T22&gt;0,MIN(T22,MAX(SUM(T$21,T$55,T$59),0))*'Fiscal Model Import'!AE40,0)</f>
-        <v>0</v>
+        <v>2325.4874619885754</v>
       </c>
       <c r="U31" s="60">
         <f>IF(U22&gt;0,MIN(U22,MAX(SUM(U$21,U$55,U$59),0))*'Fiscal Model Import'!AF40,0)</f>
-        <v>0</v>
+        <v>1649.1014650818295</v>
       </c>
       <c r="V31" s="60">
         <f>IF(V22&gt;0,MIN(V22,MAX(SUM(V$21,V$55,V$59),0))*'Fiscal Model Import'!AG40,0)</f>
-        <v>0</v>
+        <v>1150.217704946808</v>
       </c>
       <c r="W31" s="60">
         <f>IF(W22&gt;0,MIN(W22,MAX(SUM(W$21,W$55,W$59),0))*'Fiscal Model Import'!AH40,0)</f>
-        <v>0</v>
+        <v>830.32238070840242</v>
       </c>
       <c r="X31" s="60">
         <f>IF(X22&gt;0,MIN(X22,MAX(SUM(X$21,X$55,X$59),0))*'Fiscal Model Import'!AI40,0)</f>
-        <v>0</v>
+        <v>811.49076896134284</v>
       </c>
       <c r="Y31" s="60">
         <f>IF(Y22&gt;0,MIN(Y22,MAX(SUM(Y$21,Y$55,Y$59),0))*'Fiscal Model Import'!AJ40,0)</f>
-        <v>0</v>
+        <v>949.25762326112124</v>
       </c>
       <c r="Z31" s="60">
         <f>IF(Z22&gt;0,MIN(Z22,MAX(SUM(Z$21,Z$55,Z$59),0))*'Fiscal Model Import'!AK40,0)</f>
-        <v>0</v>
+        <v>1125.9611314657502</v>
       </c>
       <c r="AA31" s="60">
         <f>IF(AA22&gt;0,MIN(AA22,MAX(SUM(AA$21,AA$55,AA$59),0))*'Fiscal Model Import'!AL40,0)</f>
-        <v>0</v>
+        <v>1284.5909784942787</v>
       </c>
     </row>
     <row r="32" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -7850,83 +7856,83 @@
       </c>
       <c r="H32" s="60">
         <f>IF(H22&gt;0,MIN(H22,MAX(0,SUM(H21,H55,H59)))*'Fiscal Model Import'!S36,0)</f>
-        <v>0</v>
+        <v>5821.6195174863951</v>
       </c>
       <c r="I32" s="60">
         <f>IF(I22&gt;0,MIN(I22,MAX(0,SUM(I21,I55,I59)))*'Fiscal Model Import'!T36,0)</f>
-        <v>0</v>
+        <v>8620.9847431045891</v>
       </c>
       <c r="J32" s="60">
         <f>IF(J22&gt;0,MIN(J22,MAX(0,SUM(J21,J55,J59)))*'Fiscal Model Import'!U36,0)</f>
-        <v>0</v>
+        <v>9990.3732865714774</v>
       </c>
       <c r="K32" s="60">
         <f>IF(K22&gt;0,MIN(K22,MAX(0,SUM(K21,K55,K59)))*'Fiscal Model Import'!V36,0)</f>
-        <v>0</v>
+        <v>10683.714595714982</v>
       </c>
       <c r="L32" s="60">
         <f>IF(L22&gt;0,MIN(L22,MAX(0,SUM(L21,L55,L59)))*'Fiscal Model Import'!W36,0)</f>
-        <v>0</v>
+        <v>5235.341988067069</v>
       </c>
       <c r="M32" s="60">
         <f>IF(M22&gt;0,MIN(M22,MAX(0,SUM(M21,M55,M59)))*'Fiscal Model Import'!X36,0)</f>
-        <v>0</v>
+        <v>2660.1741077589131</v>
       </c>
       <c r="N32" s="60">
         <f>IF(N22&gt;0,MIN(N22,MAX(0,SUM(N21,N55,N59)))*'Fiscal Model Import'!Y36,0)</f>
-        <v>0</v>
+        <v>1442.3527444461488</v>
       </c>
       <c r="O32" s="60">
         <f>IF(O22&gt;0,MIN(O22,MAX(0,SUM(O21,O55,O59)))*'Fiscal Model Import'!Z36,0)</f>
-        <v>0</v>
+        <v>867.69816001095967</v>
       </c>
       <c r="P32" s="60">
         <f>IF(P22&gt;0,MIN(P22,MAX(0,SUM(P21,P55,P59)))*'Fiscal Model Import'!AA36,0)</f>
-        <v>0</v>
+        <v>1755.480865866075</v>
       </c>
       <c r="Q32" s="60">
         <f>IF(Q22&gt;0,MIN(Q22,MAX(0,SUM(Q21,Q55,Q59)))*'Fiscal Model Import'!AB36,0)</f>
-        <v>0</v>
+        <v>2736.8640313003602</v>
       </c>
       <c r="R32" s="60">
         <f>IF(R22&gt;0,MIN(R22,MAX(0,SUM(R21,R55,R59)))*'Fiscal Model Import'!AC36,0)</f>
-        <v>0</v>
+        <v>3478.9890891380937</v>
       </c>
       <c r="S32" s="60">
         <f>IF(S22&gt;0,MIN(S22,MAX(0,SUM(S21,S55,S59)))*'Fiscal Model Import'!AD36,0)</f>
-        <v>0</v>
+        <v>3973.4713078892128</v>
       </c>
       <c r="T32" s="60">
         <f>IF(T22&gt;0,MIN(T22,MAX(0,SUM(T21,T55,T59)))*'Fiscal Model Import'!AE36,0)</f>
-        <v>0</v>
+        <v>3128.3343238655839</v>
       </c>
       <c r="U32" s="60">
         <f>IF(U22&gt;0,MIN(U22,MAX(0,SUM(U21,U55,U59)))*'Fiscal Model Import'!AF36,0)</f>
-        <v>0</v>
+        <v>2218.4341137410329</v>
       </c>
       <c r="V32" s="60">
         <f>IF(V22&gt;0,MIN(V22,MAX(0,SUM(V21,V55,V59)))*'Fiscal Model Import'!AG36,0)</f>
-        <v>0</v>
+        <v>1547.3166745117774</v>
       </c>
       <c r="W32" s="60">
         <f>IF(W22&gt;0,MIN(W22,MAX(0,SUM(W21,W55,W59)))*'Fiscal Model Import'!AH36,0)</f>
-        <v>0</v>
+        <v>1116.981297857732</v>
       </c>
       <c r="X32" s="60">
         <f>IF(X22&gt;0,MIN(X22,MAX(0,SUM(X21,X55,X59)))*'Fiscal Model Import'!AI36,0)</f>
-        <v>0</v>
+        <v>1091.6482963408541</v>
       </c>
       <c r="Y32" s="60">
         <f>IF(Y22&gt;0,MIN(Y22,MAX(0,SUM(Y21,Y55,Y59)))*'Fiscal Model Import'!AJ36,0)</f>
-        <v>0</v>
+        <v>1276.9775170060323</v>
       </c>
       <c r="Z32" s="60">
         <f>IF(Z22&gt;0,MIN(Z22,MAX(0,SUM(Z21,Z55,Z59)))*'Fiscal Model Import'!AK36,0)</f>
-        <v>0</v>
+        <v>1514.6858078051166</v>
       </c>
       <c r="AA32" s="60">
         <f>IF(AA22&gt;0,MIN(AA22,MAX(0,SUM(AA21,AA55,AA59)))*'Fiscal Model Import'!AL36,0)</f>
-        <v>0</v>
+        <v>1728.0807210696846</v>
       </c>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
@@ -7955,83 +7961,83 @@
       </c>
       <c r="H33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>14734.364442487693</v>
       </c>
       <c r="I33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>21819.483509096575</v>
       </c>
       <c r="J33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>25285.369557163212</v>
       </c>
       <c r="K33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>27040.198003314028</v>
       </c>
       <c r="L33" s="60">
         <f>L25</f>
-        <v>0</v>
+        <v>13250.511580417538</v>
       </c>
       <c r="M33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6732.8300426464539</v>
       </c>
       <c r="N33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>3650.5565036424659</v>
       </c>
       <c r="O33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2196.1210067534025</v>
       </c>
       <c r="P33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>4443.0754658203323</v>
       </c>
       <c r="Q33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6926.930203114187</v>
       </c>
       <c r="R33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>8805.2290220663272</v>
       </c>
       <c r="S33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>10056.750389878895</v>
       </c>
       <c r="T33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>7917.7311205801516</v>
       </c>
       <c r="U33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>5614.7978453976593</v>
       </c>
       <c r="V33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>3916.2174239855613</v>
       </c>
       <c r="W33" s="60">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2827.0500105071801</v>
       </c>
       <c r="X33" s="60">
         <f t="shared" ref="X33:AA33" si="11">X25</f>
-        <v>0</v>
+        <v>2762.932856225525</v>
       </c>
       <c r="Y33" s="60">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>3231.9961934842941</v>
       </c>
       <c r="Z33" s="60">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>3833.6295666571982</v>
       </c>
       <c r="AA33" s="60">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>4373.7264267781402</v>
       </c>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.25">
@@ -8118,83 +8124,83 @@
       </c>
       <c r="H36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>14734.364442487693</v>
       </c>
       <c r="I36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>21819.483509096575</v>
       </c>
       <c r="J36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>25285.369557163212</v>
       </c>
       <c r="K36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>27040.198003314028</v>
       </c>
       <c r="L36" s="9">
         <f>SUM(L33:L35)</f>
-        <v>0</v>
+        <v>13250.511580417538</v>
       </c>
       <c r="M36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>6732.8300426464539</v>
       </c>
       <c r="N36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>3650.5565036424659</v>
       </c>
       <c r="O36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>2196.1210067534025</v>
       </c>
       <c r="P36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>4443.0754658203323</v>
       </c>
       <c r="Q36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>6926.930203114187</v>
       </c>
       <c r="R36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>8805.2290220663272</v>
       </c>
       <c r="S36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>10056.750389878895</v>
       </c>
       <c r="T36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>7917.7311205801516</v>
       </c>
       <c r="U36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>5614.7978453976593</v>
       </c>
       <c r="V36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>3916.2174239855613</v>
       </c>
       <c r="W36" s="9">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>2827.0500105071801</v>
       </c>
       <c r="X36" s="9">
         <f t="shared" ref="X36:AA36" si="13">SUM(X33:X35)</f>
-        <v>0</v>
+        <v>2762.932856225525</v>
       </c>
       <c r="Y36" s="9">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>3231.9961934842941</v>
       </c>
       <c r="Z36" s="9">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>3833.6295666571982</v>
       </c>
       <c r="AA36" s="9">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>4373.7264267781402</v>
       </c>
     </row>
     <row r="37" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -8223,83 +8229,83 @@
       </c>
       <c r="H37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>6182.2508150298008</v>
       </c>
       <c r="I37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>15337.278860804585</v>
       </c>
       <c r="J37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>25946.524828845089</v>
       </c>
       <c r="K37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>37292.062452613216</v>
       </c>
       <c r="L37" s="60">
         <f>IF(AND(L$22&gt;0,L$21+L$55+L$59&gt;0),K37+L29-L56,L$22*K46)</f>
-        <v>0</v>
+        <v>42851.717661180017</v>
       </c>
       <c r="M37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>45676.681315437272</v>
       </c>
       <c r="N37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>47208.383344937611</v>
       </c>
       <c r="O37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>48129.832718400576</v>
       </c>
       <c r="P37" s="60">
         <f>IF(AND(P$22&gt;0,P$21+P$55+P$59&gt;0),O37+P29-P56,P$22*O46)</f>
-        <v>0</v>
+        <v>43811.80937154714</v>
       </c>
       <c r="Q37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>37563.185606799285</v>
       </c>
       <c r="R37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>30648.441326339052</v>
       </c>
       <c r="S37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>23522.519250771864</v>
       </c>
       <c r="T37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>21284.988987903031</v>
       </c>
       <c r="U37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>20815.884569476966</v>
       </c>
       <c r="V37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>20927.350689900642</v>
       </c>
       <c r="W37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>21192.076146021111</v>
       </c>
       <c r="X37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>20487.12120493238</v>
       </c>
       <c r="Y37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>18936.799242849909</v>
       </c>
       <c r="Z37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>16850.813457363562</v>
       </c>
       <c r="AA37" s="60">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>14466.32787844017</v>
       </c>
     </row>
     <row r="38" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -8433,83 +8439,83 @@
       </c>
       <c r="H39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>4327.5755705208603</v>
       </c>
       <c r="I39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>10736.09520256321</v>
       </c>
       <c r="J39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>18162.567380191565</v>
       </c>
       <c r="K39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>26104.44371682925</v>
       </c>
       <c r="L39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>29996.20236282601</v>
       </c>
       <c r="M39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>31973.676920806087</v>
       </c>
       <c r="N39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>33045.86834145632</v>
       </c>
       <c r="O39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>33690.882902880396</v>
       </c>
       <c r="P39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>34995.842130603851</v>
       </c>
       <c r="Q39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>37030.3251273227</v>
       </c>
       <c r="R39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>39616.476308628895</v>
       </c>
       <c r="S39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>42570.207192369548</v>
       </c>
       <c r="T39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>44895.694654358122</v>
       </c>
       <c r="U39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>46544.796119439954</v>
       </c>
       <c r="V39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>47695.013824386762</v>
       </c>
       <c r="W39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>48525.336205095162</v>
       </c>
       <c r="X39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>49336.826974056501</v>
       </c>
       <c r="Y39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>50286.084597317626</v>
       </c>
       <c r="Z39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>51412.045728783378</v>
       </c>
       <c r="AA39" s="60">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>52696.636707277656</v>
       </c>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.25">
@@ -8538,83 +8544,83 @@
       </c>
       <c r="H40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>10509.826385550661</v>
       </c>
       <c r="I40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>26073.374063367795</v>
       </c>
       <c r="J40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>44109.092209036651</v>
       </c>
       <c r="K40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>63396.506169442466</v>
       </c>
       <c r="L40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>72847.920024006031</v>
       </c>
       <c r="M40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>77650.358236243366</v>
       </c>
       <c r="N40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>80254.251686393924</v>
       </c>
       <c r="O40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>81820.715621280979</v>
       </c>
       <c r="P40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>78807.651502150984</v>
       </c>
       <c r="Q40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>74593.510734121985</v>
       </c>
       <c r="R40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>70264.917634967947</v>
       </c>
       <c r="S40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>66092.726443141408</v>
       </c>
       <c r="T40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>66180.683642261152</v>
       </c>
       <c r="U40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>67360.680688916924</v>
       </c>
       <c r="V40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>68622.364514287401</v>
       </c>
       <c r="W40" s="60">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>69717.412351116276</v>
       </c>
       <c r="X40" s="60">
         <f>SUM(X37:X39)</f>
-        <v>0</v>
+        <v>69823.948178988881</v>
       </c>
       <c r="Y40" s="60">
         <f t="shared" ref="Y40:AA40" si="18">SUM(Y37:Y39)</f>
-        <v>0</v>
+        <v>69222.883840167531</v>
       </c>
       <c r="Z40" s="60">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>68262.859186146932</v>
       </c>
       <c r="AA40" s="60">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>67162.964585717826</v>
       </c>
     </row>
     <row r="41" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -8643,83 +8649,83 @@
       </c>
       <c r="H41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>5821.6195174863951</v>
       </c>
       <c r="I41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>14442.604260590984</v>
       </c>
       <c r="J41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>24432.97754716246</v>
       </c>
       <c r="K41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>35116.692142877444</v>
       </c>
       <c r="L41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>40352.034130944514</v>
       </c>
       <c r="M41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>43012.208238703424</v>
       </c>
       <c r="N41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>44454.560983149575</v>
       </c>
       <c r="O41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>45322.259143160532</v>
       </c>
       <c r="P41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>47077.740009026609</v>
       </c>
       <c r="Q41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>49814.604040326973</v>
       </c>
       <c r="R41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>53293.593129465065</v>
       </c>
       <c r="S41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>57267.064437354275</v>
       </c>
       <c r="T41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>60395.398761219862</v>
       </c>
       <c r="U41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>62613.832874960892</v>
       </c>
       <c r="V41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>64161.14954947267</v>
       </c>
       <c r="W41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>65278.130847330402</v>
       </c>
       <c r="X41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>66369.779143671258</v>
       </c>
       <c r="Y41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>67646.756660677289</v>
       </c>
       <c r="Z41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>69161.442468482404</v>
       </c>
       <c r="AA41" s="60">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>70889.523189552085</v>
       </c>
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.25">
@@ -8748,83 +8754,83 @@
       </c>
       <c r="H42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>0.47429519071310117</v>
       </c>
       <c r="I42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>0.35003323738152048</v>
       </c>
       <c r="J42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>0.26948800630395359</v>
       </c>
       <c r="K42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>0.21536811266607667</v>
       </c>
       <c r="L42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>0.1047881595639816</v>
       </c>
       <c r="M42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>5.2849869200074694E-2</v>
       </c>
       <c r="N42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>2.8440124995605387E-2</v>
       </c>
       <c r="O42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>1.6979560539362455E-2</v>
       </c>
       <c r="P42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>3.4091365983799256E-2</v>
       </c>
       <c r="Q42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>5.2742435991075816E-2</v>
       </c>
       <c r="R42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>6.6522969479927238E-2</v>
       </c>
       <c r="S42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>7.5378587198557626E-2</v>
       </c>
       <c r="T42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>5.8870597190432514E-2</v>
       </c>
       <c r="U42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>4.1410327901507116E-2</v>
       </c>
       <c r="V42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>2.8648318335114116E-2</v>
       </c>
       <c r="W42" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>2.051223928301122E-2</v>
       </c>
       <c r="X42" s="58">
         <f t="shared" ref="X42:AA42" si="21">IF(X$22=0,0,X33/X$22)</f>
-        <v>0</v>
+        <v>1.9883414387397234E-2</v>
       </c>
       <c r="Y42" s="58">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>2.3068939590875699E-2</v>
       </c>
       <c r="Z42" s="58">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>2.7139216421424531E-2</v>
       </c>
       <c r="AA42" s="58">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>3.0708717852835025E-2</v>
       </c>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.25">
@@ -8940,83 +8946,83 @@
       </c>
       <c r="H46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.19900497512437809</v>
       </c>
       <c r="I46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.24604420036030769</v>
       </c>
       <c r="J46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.27653450865465473</v>
       </c>
       <c r="K46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.29702153463744729</v>
       </c>
       <c r="L46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.33888145379281454</v>
       </c>
       <c r="M46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.35854263626495597</v>
       </c>
       <c r="N46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.36778291798273616</v>
       </c>
       <c r="O46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.37212130200402688</v>
       </c>
       <c r="P46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.33616454169816651</v>
       </c>
       <c r="Q46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.2860103760821528</v>
       </c>
       <c r="R46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.23154710931992786</v>
       </c>
       <c r="S46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.17630886715240521</v>
       </c>
       <c r="T46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.15825998557245985</v>
       </c>
       <c r="U46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.15352157447458631</v>
       </c>
       <c r="V46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.15308991804257241</v>
       </c>
       <c r="W46" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.15376344075816104</v>
       </c>
       <c r="X46" s="58">
         <f t="shared" ref="X46:AA46" si="23">IF(X$22=0,0,X37/X$22)</f>
-        <v>0</v>
+        <v>0.14743533112092866</v>
       </c>
       <c r="Y46" s="58">
         <f t="shared" si="23"/>
-        <v>0</v>
+        <v>0.13516472533554924</v>
       </c>
       <c r="Z46" s="58">
         <f t="shared" si="23"/>
-        <v>0</v>
+        <v>0.11929109616483086</v>
       </c>
       <c r="AA46" s="58">
         <f t="shared" si="23"/>
-        <v>0</v>
+        <v>0.10157068317436287</v>
       </c>
     </row>
     <row r="47" spans="1:27" x14ac:dyDescent="0.25">
@@ -9150,83 +9156,83 @@
       </c>
       <c r="H48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.13930348258706465</v>
       </c>
       <c r="I48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.17223094025221539</v>
       </c>
       <c r="J48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.19357415605825834</v>
       </c>
       <c r="K48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.20791507424621311</v>
       </c>
       <c r="L48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.23721701765497016</v>
       </c>
       <c r="M48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.25097984538546914</v>
       </c>
       <c r="N48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.25744804258791526</v>
       </c>
       <c r="O48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.26048491140281876</v>
       </c>
       <c r="P48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.26852032362799427</v>
       </c>
       <c r="Q48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.28195311566420705</v>
       </c>
       <c r="R48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.29930006792290437</v>
       </c>
       <c r="S48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.31907743063207666</v>
       </c>
       <c r="T48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.33381234034475643</v>
       </c>
       <c r="U48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.34327776751476208</v>
       </c>
       <c r="V48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.34890349311814367</v>
       </c>
       <c r="W48" s="58">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.35208549683523599</v>
       </c>
       <c r="X48" s="58">
         <f t="shared" ref="X48:AA48" si="27">IF(X$22=0,0,X39/X$22)</f>
-        <v>0</v>
+        <v>0.35505190546853083</v>
       </c>
       <c r="Y48" s="58">
         <f t="shared" si="27"/>
-        <v>0</v>
+        <v>0.35892574693492518</v>
       </c>
       <c r="Z48" s="58">
         <f t="shared" si="27"/>
-        <v>0</v>
+        <v>0.36395864844037823</v>
       </c>
       <c r="AA48" s="58">
         <f t="shared" si="27"/>
-        <v>0</v>
+        <v>0.36999253966352963</v>
       </c>
     </row>
     <row r="49" spans="1:27" x14ac:dyDescent="0.25">
@@ -9255,83 +9261,83 @@
       </c>
       <c r="H49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.18739635157545603</v>
       </c>
       <c r="I49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.23169162200595642</v>
       </c>
       <c r="J49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.26040332898313323</v>
       </c>
       <c r="K49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.27969527845026287</v>
       </c>
       <c r="L49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.31911336898823367</v>
       </c>
       <c r="M49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.33762764914950016</v>
       </c>
       <c r="N49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.34632891443374314</v>
       </c>
       <c r="O49" s="58">
         <f>IF(O22=0,0,O41/O22)</f>
-        <v>0</v>
+        <v>0.35041422605379186</v>
       </c>
       <c r="P49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.36122376869003991</v>
       </c>
       <c r="Q49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.37929407226256434</v>
       </c>
       <c r="R49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.40262985327724043</v>
       </c>
       <c r="S49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.42923511501696027</v>
       </c>
       <c r="T49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.44905707689235097</v>
       </c>
       <c r="U49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.46179033010914422</v>
       </c>
       <c r="V49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.46935827050416945</v>
       </c>
       <c r="W49" s="58">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>0.47363882312359135</v>
       </c>
       <c r="X49" s="58">
         <f t="shared" ref="X49:AA49" si="29">IF(X22=0,0,X41/X22)</f>
-        <v>0</v>
+        <v>0.47762934902314275</v>
       </c>
       <c r="Y49" s="58">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>0.48284058813864944</v>
       </c>
       <c r="Z49" s="58">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>0.489611038973366</v>
       </c>
       <c r="AA49" s="58">
         <f t="shared" si="29"/>
-        <v>0</v>
+        <v>0.49772805930927205</v>
       </c>
     </row>
     <row r="50" spans="1:27" x14ac:dyDescent="0.25">
@@ -9421,79 +9427,79 @@
       </c>
       <c r="I52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>14734.364442487693</v>
       </c>
       <c r="J52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>21819.483509096575</v>
       </c>
       <c r="K52" s="9">
         <f>MAX(0,J33)</f>
-        <v>0</v>
+        <v>25285.369557163212</v>
       </c>
       <c r="L52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>27040.198003314028</v>
       </c>
       <c r="M52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>13250.511580417538</v>
       </c>
       <c r="N52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>6732.8300426464539</v>
       </c>
       <c r="O52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>3650.5565036424659</v>
       </c>
       <c r="P52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>2196.1210067534025</v>
       </c>
       <c r="Q52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>4443.0754658203323</v>
       </c>
       <c r="R52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>6926.930203114187</v>
       </c>
       <c r="S52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>8805.2290220663272</v>
       </c>
       <c r="T52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>10056.750389878895</v>
       </c>
       <c r="U52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>7917.7311205801516</v>
       </c>
       <c r="V52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>5614.7978453976593</v>
       </c>
       <c r="W52" s="9">
         <f t="shared" si="30"/>
-        <v>0</v>
+        <v>3916.2174239855613</v>
       </c>
       <c r="X52" s="9">
         <f t="shared" ref="X52" si="31">MAX(0,W33)</f>
-        <v>0</v>
+        <v>2827.0500105071801</v>
       </c>
       <c r="Y52" s="9">
         <f t="shared" ref="Y52" si="32">MAX(0,X33)</f>
-        <v>0</v>
+        <v>2762.932856225525</v>
       </c>
       <c r="Z52" s="9">
         <f t="shared" ref="Z52" si="33">MAX(0,Y33)</f>
-        <v>0</v>
+        <v>3231.9961934842941</v>
       </c>
       <c r="AA52" s="9">
         <f t="shared" ref="AA52" si="34">MAX(0,Z33)</f>
-        <v>0</v>
+        <v>3833.6295666571982</v>
       </c>
     </row>
     <row r="53" spans="1:27" x14ac:dyDescent="0.25">
@@ -9579,79 +9585,79 @@
       </c>
       <c r="I55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>14734.364442487693</v>
       </c>
       <c r="J55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>21819.483509096575</v>
       </c>
       <c r="K55" s="9">
         <f>SUM(K52:K54)</f>
-        <v>0</v>
+        <v>25285.369557163212</v>
       </c>
       <c r="L55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>27040.198003314028</v>
       </c>
       <c r="M55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>13250.511580417538</v>
       </c>
       <c r="N55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>6732.8300426464539</v>
       </c>
       <c r="O55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>3650.5565036424659</v>
       </c>
       <c r="P55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>2196.1210067534025</v>
       </c>
       <c r="Q55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>4443.0754658203323</v>
       </c>
       <c r="R55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>6926.930203114187</v>
       </c>
       <c r="S55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>8805.2290220663272</v>
       </c>
       <c r="T55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>10056.750389878895</v>
       </c>
       <c r="U55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>7917.7311205801516</v>
       </c>
       <c r="V55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>5614.7978453976593</v>
       </c>
       <c r="W55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>3916.2174239855613</v>
       </c>
       <c r="X55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>2827.0500105071801</v>
       </c>
       <c r="Y55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>2762.932856225525</v>
       </c>
       <c r="Z55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>3231.9961934842941</v>
       </c>
       <c r="AA55" s="9">
         <f t="shared" si="35"/>
-        <v>0</v>
+        <v>3833.6295666571982</v>
       </c>
     </row>
     <row r="56" spans="1:27" x14ac:dyDescent="0.25">
@@ -9688,51 +9694,51 @@
       </c>
       <c r="P56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>6182.2508150298008</v>
       </c>
       <c r="Q56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>9155.0280457747849</v>
       </c>
       <c r="R56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>10609.245968040506</v>
       </c>
       <c r="S56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>11345.537623768123</v>
       </c>
       <c r="T56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>5559.655208566799</v>
       </c>
       <c r="U56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>2824.963654257253</v>
       </c>
       <c r="V56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>1531.7020295003351</v>
       </c>
       <c r="W56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>921.44937346296604</v>
       </c>
       <c r="X56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>1864.2274681763629</v>
       </c>
       <c r="Y56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>2906.4042810269311</v>
       </c>
       <c r="Z56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>3694.5016875802767</v>
       </c>
       <c r="AA56" s="9">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>4219.6155482009344</v>
       </c>
     </row>
     <row r="57" spans="1:27" x14ac:dyDescent="0.25">
@@ -9871,51 +9877,51 @@
       </c>
       <c r="P59" s="9">
         <f t="shared" si="38"/>
-        <v>0</v>
+        <v>6182.2508150298008</v>
       </c>
       <c r="Q59" s="9">
         <f t="shared" si="38"/>
-        <v>0</v>
+        <v>9155.0280457747849</v>
       </c>
       <c r="R59" s="9">
         <f t="shared" si="38"/>
-        <v>0</v>
+        <v>10609.245968040506</v>
       </c>
       <c r="S59" s="9">
         <f t="shared" si="38"/>
-        <v>0</v>
+        <v>11345.537623768123</v>
       </c>
       <c r="T59" s="9">
         <f t="shared" si="38"/>
-        <v>0</v>
+        <v>5559.655208566799</v>
       </c>
       <c r="U59" s="9">
         <f t="shared" si="38"/>
-        <v>0</v>
+        <v>2824.963654257253</v>
       </c>
       <c r="V59" s="9">
         <f t="shared" si="38"/>
-        <v>0</v>
+        <v>1531.7020295003351</v>
       </c>
       <c r="W59" s="9">
         <f t="shared" si="38"/>
-        <v>0</v>
+        <v>921.44937346296604</v>
       </c>
       <c r="X59" s="9">
         <f t="shared" ref="X59:AA59" si="39">SUM(X56:X58)</f>
-        <v>0</v>
+        <v>1864.2274681763629</v>
       </c>
       <c r="Y59" s="9">
         <f t="shared" si="39"/>
-        <v>0</v>
+        <v>2906.4042810269311</v>
       </c>
       <c r="Z59" s="9">
         <f t="shared" si="39"/>
-        <v>0</v>
+        <v>3694.5016875802767</v>
       </c>
       <c r="AA59" s="9">
         <f t="shared" si="39"/>
-        <v>0</v>
+        <v>4219.6155482009344</v>
       </c>
     </row>
     <row r="60" spans="1:27" x14ac:dyDescent="0.25">
@@ -10142,51 +10148,51 @@
       </c>
       <c r="I64" s="32">
         <f>IF(SUM(D29:I29)&gt;0, SUMPRODUCT(D29:I29,D$13:I$13)/SUM(D29:I29), I$13)</f>
-        <v>2.4483044266243899</v>
+        <v>2.4351247517514309</v>
       </c>
       <c r="J64" s="32">
         <f>IF(SUM(D29:J29)&gt;0, SUMPRODUCT(D29:J29,D$13:J$13)/SUM(D29:J29), J$13)</f>
-        <v>2.5111633473523298</v>
+        <v>2.4662160893820282</v>
       </c>
       <c r="K64" s="32">
         <f t="shared" ref="K64:Z64" si="41">IF(SUM(D28:K28)&gt;0, SUMPRODUCT(D28:K28,D$13:K$13)/SUM(D28:K28), K$13)</f>
-        <v>2.5772256649611598</v>
+        <v>2.4999890489208565</v>
       </c>
       <c r="L64" s="32">
         <f t="shared" si="41"/>
-        <v>2.6982252129903701</v>
+        <v>2.5257085482139687</v>
       </c>
       <c r="M64" s="32">
         <f t="shared" si="41"/>
-        <v>2.7315614500000001</v>
+        <v>2.5384399233691157</v>
       </c>
       <c r="N64" s="32">
         <f t="shared" si="41"/>
-        <v>2.82</v>
+        <v>2.5475752953146165</v>
       </c>
       <c r="O64" s="32">
         <f t="shared" si="41"/>
-        <v>2.82</v>
+        <v>2.5527908873761325</v>
       </c>
       <c r="P64" s="32">
         <f t="shared" si="41"/>
-        <v>2.82</v>
+        <v>2.5835186852638432</v>
       </c>
       <c r="Q64" s="32">
         <f t="shared" si="41"/>
-        <v>2.82</v>
+        <v>2.6347710112970324</v>
       </c>
       <c r="R64" s="32">
         <f t="shared" si="41"/>
-        <v>2.82</v>
+        <v>2.6998873054806798</v>
       </c>
       <c r="S64" s="32">
         <f t="shared" si="41"/>
-        <v>2.82</v>
+        <v>2.7805968430347869</v>
       </c>
       <c r="T64" s="32">
         <f t="shared" si="41"/>
-        <v>2.82</v>
+        <v>2.8082623528944644</v>
       </c>
       <c r="U64" s="32">
         <f t="shared" si="41"/>
@@ -10194,7 +10200,7 @@
       </c>
       <c r="V64" s="32">
         <f t="shared" si="41"/>
-        <v>2.82</v>
+        <v>2.8200000000000003</v>
       </c>
       <c r="W64" s="32">
         <f t="shared" si="41"/>
@@ -10206,15 +10212,15 @@
       </c>
       <c r="Y64" s="32">
         <f t="shared" si="41"/>
-        <v>2.82</v>
+        <v>2.8200000000000003</v>
       </c>
       <c r="Z64" s="32">
         <f t="shared" si="41"/>
-        <v>2.82</v>
+        <v>2.8200000000000003</v>
       </c>
       <c r="AA64" s="32">
         <f>IF(SUM(T28:AA28)&gt;0, SUMPRODUCT(T28:AA28,T$13:AA$13)/SUM(T28:AA28), AA$13)</f>
-        <v>2.82</v>
+        <v>2.8200000000000003</v>
       </c>
     </row>
     <row r="65" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -10348,83 +10354,83 @@
       </c>
       <c r="H66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.59691345047986666</v>
       </c>
       <c r="J66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.40888889891898228</v>
       </c>
       <c r="K66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.30423465149413026</v>
       </c>
       <c r="L66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.12974171193150025</v>
       </c>
       <c r="M66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>6.1846955008583449E-2</v>
       </c>
       <c r="N66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>3.2445551424810384E-2</v>
       </c>
       <c r="O66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>1.9145077417040052E-2</v>
       </c>
       <c r="P66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>3.7288979155105616E-2</v>
       </c>
       <c r="Q66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>5.4940997404792302E-2</v>
       </c>
       <c r="R66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>6.5279687197796074E-2</v>
       </c>
       <c r="S66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>6.9384930883542709E-2</v>
       </c>
       <c r="T66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>5.1797560543209803E-2</v>
       </c>
       <c r="U66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>3.5430415482968755E-2</v>
       </c>
       <c r="V66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>2.4116099623786972E-2</v>
       </c>
       <c r="W66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>1.7111110311508127E-2</v>
       </c>
       <c r="X66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>1.6447972411927924E-2</v>
       </c>
       <c r="Y66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>1.8877143266623642E-2</v>
       </c>
       <c r="Z66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>2.1900726094534171E-2</v>
       </c>
       <c r="AA66" s="61">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>2.4377096125318194E-2</v>
       </c>
     </row>
     <row r="67" spans="1:27" x14ac:dyDescent="0.25">
@@ -10453,83 +10459,83 @@
       </c>
       <c r="H67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>0.59691345047986677</v>
       </c>
       <c r="J67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>0.40888889891898239</v>
       </c>
       <c r="K67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>0.30423465149413026</v>
       </c>
       <c r="L67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>0.12974171193150025</v>
       </c>
       <c r="M67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>6.1846955008583449E-2</v>
       </c>
       <c r="N67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>3.2445551424810384E-2</v>
       </c>
       <c r="O67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.9145077417040052E-2</v>
       </c>
       <c r="P67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>3.7288979155105616E-2</v>
       </c>
       <c r="Q67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>5.4940997404792302E-2</v>
       </c>
       <c r="R67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>6.5279687197796074E-2</v>
       </c>
       <c r="S67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>6.9384930883542709E-2</v>
       </c>
       <c r="T67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>5.1797560543209796E-2</v>
       </c>
       <c r="U67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>3.5430415482968762E-2</v>
       </c>
       <c r="V67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>2.4116099623786968E-2</v>
       </c>
       <c r="W67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.7111110311508127E-2</v>
       </c>
       <c r="X67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.6447972411927924E-2</v>
       </c>
       <c r="Y67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.8877143266623642E-2</v>
       </c>
       <c r="Z67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>2.1900726094534174E-2</v>
       </c>
       <c r="AA67" s="61">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>2.4377096125318198E-2</v>
       </c>
     </row>
     <row r="68" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -10562,79 +10568,79 @@
       </c>
       <c r="I68" s="32">
         <f t="shared" si="45"/>
-        <v>2.7232835266243902</v>
+        <v>2.7089933241223099</v>
       </c>
       <c r="J68" s="32">
         <f t="shared" si="45"/>
-        <v>2.7888981673523299</v>
+        <v>2.7416655274889266</v>
       </c>
       <c r="K68" s="32">
         <f t="shared" si="45"/>
-        <v>2.85771620496116</v>
+        <v>2.7769721649053487</v>
       </c>
       <c r="L68" s="32">
         <f t="shared" si="45"/>
-        <v>2.9264721329903698</v>
+        <v>2.7963685466984041</v>
       </c>
       <c r="M68" s="32">
         <f t="shared" si="45"/>
-        <v>2.9611849100000001</v>
+        <v>2.8065619369041968</v>
       </c>
       <c r="N68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8127083593221878</v>
       </c>
       <c r="O68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8162174919728611</v>
       </c>
       <c r="P68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8229213981671375</v>
       </c>
       <c r="Q68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.832430509181262</v>
       </c>
       <c r="R68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8431082743770122</v>
       </c>
       <c r="S68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8537166561920286</v>
       </c>
       <c r="T68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8610865863072119</v>
       </c>
       <c r="U68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8658666246085733</v>
       </c>
       <c r="V68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8690049340538923</v>
       </c>
       <c r="W68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8711779606363135</v>
       </c>
       <c r="X68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8732310300961674</v>
       </c>
       <c r="Y68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8755485575297381</v>
       </c>
       <c r="Z68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.878186531578971</v>
       </c>
       <c r="AA68" s="32">
         <f t="shared" si="45"/>
-        <v>2.996</v>
+        <v>2.8810584818235276</v>
       </c>
     </row>
     <row r="69" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -10667,79 +10673,79 @@
       </c>
       <c r="I69" s="32">
         <f t="shared" si="46"/>
-        <v>3.8136239999999999</v>
+        <v>3.8184162959872445</v>
       </c>
       <c r="J69" s="32">
         <f t="shared" si="46"/>
-        <v>3.8017349999999999</v>
+        <v>3.8115954992384782</v>
       </c>
       <c r="K69" s="32">
         <f t="shared" si="46"/>
-        <v>3.789847</v>
+        <v>3.8049788521521393</v>
       </c>
       <c r="L69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7779579999999999</v>
+        <v>3.8014731205360723</v>
       </c>
       <c r="M69" s="32">
         <f t="shared" si="46"/>
-        <v>3.763979</v>
+        <v>3.7991542233501918</v>
       </c>
       <c r="N69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7975593874687363</v>
       </c>
       <c r="O69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7966488593137404</v>
       </c>
       <c r="P69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.794909370971181</v>
       </c>
       <c r="Q69" s="32">
         <f>IF(Q41&gt;0,Q67*Q12+(1-Q67)*P69,Q12)</f>
-        <v>3.75</v>
+        <v>3.7924420053372025</v>
       </c>
       <c r="R69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7896714045047428</v>
       </c>
       <c r="S69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7869188068451285</v>
       </c>
       <c r="T69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7850065027123847</v>
       </c>
       <c r="U69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7837662077766794</v>
       </c>
       <c r="V69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7829518985460195</v>
       </c>
       <c r="W69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7823880549750246</v>
       </c>
       <c r="X69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7818553371403194</v>
       </c>
       <c r="Y69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7812539993773151</v>
       </c>
       <c r="Z69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7805695140975937</v>
       </c>
       <c r="AA69" s="32">
         <f t="shared" si="46"/>
-        <v>3.75</v>
+        <v>3.7798243181139322</v>
       </c>
     </row>
     <row r="70" spans="1:27" x14ac:dyDescent="0.25">
@@ -10801,79 +10807,79 @@
       </c>
       <c r="I71" s="46">
         <f t="shared" si="47"/>
-        <v>2.6246962842974719</v>
+        <v>2.7204889770234395</v>
       </c>
       <c r="J71" s="46">
         <f t="shared" si="47"/>
-        <v>2.6441179149915013</v>
+        <v>2.798135215798677</v>
       </c>
       <c r="K71" s="46">
         <f t="shared" si="47"/>
-        <v>2.6646234693400936</v>
+        <v>2.8579694251486707</v>
       </c>
       <c r="L71" s="46">
         <f t="shared" si="47"/>
-        <v>2.8146267640630773</v>
+        <v>2.9890938771318822</v>
       </c>
       <c r="M71" s="46">
         <f t="shared" si="47"/>
-        <v>2.823476838208955</v>
+        <v>3.0267111118402372</v>
       </c>
       <c r="N71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.0530738950175569</v>
       </c>
       <c r="O71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.0597746177327556</v>
       </c>
       <c r="P71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.0893572951882162</v>
       </c>
       <c r="Q71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.1330398039972893</v>
       </c>
       <c r="R71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.1815404598673336</v>
       </c>
       <c r="S71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.2298011728648954</v>
       </c>
       <c r="T71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.2581361372976918</v>
       </c>
       <c r="U71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.2758336683881182</v>
       </c>
       <c r="V71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.2856296321514793</v>
       </c>
       <c r="W71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.2913818947302609</v>
       </c>
       <c r="X71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.2959241074719738</v>
       </c>
       <c r="Y71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.3013019811615849</v>
       </c>
       <c r="Z71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9618805970149253</v>
+        <v>3.3082262232238078</v>
       </c>
       <c r="AA71" s="46">
         <f>IF(AA22&gt;0,SUMPRODUCT(AA42,AA61)+SUMPRODUCT(AA46:AA47,AA64:AA65)+SUMPRODUCT(AA48:AA49,AA68:AA69),AA16)</f>
-        <v>2.9618805970149253</v>
+        <v>3.3166376317482382</v>
       </c>
     </row>
     <row r="73" spans="1:27" x14ac:dyDescent="0.25">
@@ -10931,83 +10937,83 @@
       </c>
       <c r="H74" s="13">
         <f>H19+H20</f>
-        <v>0</v>
+        <v>-201.81034552475003</v>
       </c>
       <c r="I74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-405.65148753060447</v>
       </c>
       <c r="J74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-627.97748030697539</v>
       </c>
       <c r="K74" s="13">
         <f>K19+K20</f>
-        <v>0</v>
+        <v>-861.95700227161262</v>
       </c>
       <c r="L74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-897.06941973413893</v>
       </c>
       <c r="M74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-944.93078222515908</v>
       </c>
       <c r="N74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-963.97265559273126</v>
       </c>
       <c r="O74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-979.72659800893848</v>
       </c>
       <c r="P74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-989.37120580302053</v>
       </c>
       <c r="Q74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-1006.5780005652127</v>
       </c>
       <c r="R74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-1028.694808936199</v>
       </c>
       <c r="S74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-1052.8014838752481</v>
       </c>
       <c r="T74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-1077.2722536865842</v>
       </c>
       <c r="U74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-1095.497885214302</v>
       </c>
       <c r="V74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-1110.4200784701648</v>
       </c>
       <c r="W74" s="13">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>-1122.8617212082197</v>
       </c>
       <c r="X74" s="13">
         <f t="shared" ref="X74:AA74" si="49">X19+X20</f>
-        <v>0</v>
+        <v>-1134.0669699318119</v>
       </c>
       <c r="Y74" s="13">
         <f t="shared" si="49"/>
-        <v>0</v>
+        <v>-1144.9765154434508</v>
       </c>
       <c r="Z74" s="13">
         <f t="shared" si="49"/>
-        <v>0</v>
+        <v>-1156.2945269574238</v>
       </c>
       <c r="AA74" s="13">
         <f t="shared" si="49"/>
-        <v>0</v>
+        <v>-1168.2829807615133</v>
       </c>
     </row>
     <row r="75" spans="1:27" x14ac:dyDescent="0.25">
@@ -11034,83 +11040,83 @@
       </c>
       <c r="H75" s="13">
         <f>-SUM($D21:H21)</f>
-        <v>0</v>
+        <v>-31065.810345524751</v>
       </c>
       <c r="I75" s="13">
         <f>-SUM($D21:I21)</f>
-        <v>0</v>
+        <v>-62335.461833055357</v>
       </c>
       <c r="J75" s="13">
         <f>-SUM($D21:J21)</f>
-        <v>0</v>
+        <v>-93827.439313362338</v>
       </c>
       <c r="K75" s="13">
         <f>-SUM($D21:K21)</f>
-        <v>0</v>
+        <v>-125553.39631563395</v>
       </c>
       <c r="L75" s="13">
         <f>-SUM($D21:L21)</f>
-        <v>0</v>
+        <v>-126450.46573536808</v>
       </c>
       <c r="M75" s="13">
         <f>-SUM($D21:M21)</f>
-        <v>0</v>
+        <v>-127395.39651759324</v>
       </c>
       <c r="N75" s="13">
         <f>-SUM($D21:N21)</f>
-        <v>0</v>
+        <v>-128359.36917318597</v>
       </c>
       <c r="O75" s="13">
         <f>-SUM($D21:O21)</f>
-        <v>0</v>
+        <v>-129339.09577119492</v>
       </c>
       <c r="P75" s="13">
         <f>-SUM($D21:P21)</f>
-        <v>0</v>
+        <v>-130328.46697699794</v>
       </c>
       <c r="Q75" s="13">
         <f>-SUM($D21:Q21)</f>
-        <v>0</v>
+        <v>-131335.04497756314</v>
       </c>
       <c r="R75" s="13">
         <f>-SUM($D21:R21)</f>
-        <v>0</v>
+        <v>-132363.73978649935</v>
       </c>
       <c r="S75" s="13">
         <f>-SUM($D21:S21)</f>
-        <v>0</v>
+        <v>-133416.54127037461</v>
       </c>
       <c r="T75" s="13">
         <f>-SUM($D21:T21)</f>
-        <v>0</v>
+        <v>-134493.8135240612</v>
       </c>
       <c r="U75" s="13">
         <f>-SUM($D21:U21)</f>
-        <v>0</v>
+        <v>-135589.31140927551</v>
       </c>
       <c r="V75" s="13">
         <f>-SUM($D21:V21)</f>
-        <v>0</v>
+        <v>-136699.73148774568</v>
       </c>
       <c r="W75" s="13">
         <f>-SUM($D21:W21)</f>
-        <v>0</v>
+        <v>-137822.59320895391</v>
       </c>
       <c r="X75" s="13">
         <f>-SUM($D21:X21)</f>
-        <v>0</v>
+        <v>-138956.66017888574</v>
       </c>
       <c r="Y75" s="13">
         <f>-SUM($D21:Y21)</f>
-        <v>0</v>
+        <v>-140101.63669432918</v>
       </c>
       <c r="Z75" s="13">
         <f>-SUM($D21:Z21)</f>
-        <v>0</v>
+        <v>-141257.93122128659</v>
       </c>
       <c r="AA75" s="13">
         <f>-SUM($D21:AA21)</f>
-        <v>0</v>
+        <v>-142426.21420204811</v>
       </c>
     </row>
     <row r="76" spans="1:27" x14ac:dyDescent="0.25">
@@ -11137,83 +11143,83 @@
       </c>
       <c r="H76" s="13">
         <f>SUM($D74:H74)</f>
-        <v>0</v>
+        <v>-201.81034552475003</v>
       </c>
       <c r="I76" s="13">
         <f>SUM($D74:I74)</f>
-        <v>0</v>
+        <v>-607.46183305535453</v>
       </c>
       <c r="J76" s="13">
         <f>SUM($D74:J74)</f>
-        <v>0</v>
+        <v>-1235.4393133623298</v>
       </c>
       <c r="K76" s="13">
         <f>SUM($D74:K74)</f>
-        <v>0</v>
+        <v>-2097.3963156339423</v>
       </c>
       <c r="L76" s="13">
         <f>SUM($D74:L74)</f>
-        <v>0</v>
+        <v>-2994.4657353680814</v>
       </c>
       <c r="M76" s="13">
         <f>SUM($D74:M74)</f>
-        <v>0</v>
+        <v>-3939.3965175932403</v>
       </c>
       <c r="N76" s="13">
         <f>SUM($D74:N74)</f>
-        <v>0</v>
+        <v>-4903.3691731859717</v>
       </c>
       <c r="O76" s="13">
         <f>SUM($D74:O74)</f>
-        <v>0</v>
+        <v>-5883.0957711949104</v>
       </c>
       <c r="P76" s="13">
         <f>SUM($D74:P74)</f>
-        <v>0</v>
+        <v>-6872.4669769979309</v>
       </c>
       <c r="Q76" s="13">
         <f>SUM($D74:Q74)</f>
-        <v>0</v>
+        <v>-7879.0449775631441</v>
       </c>
       <c r="R76" s="13">
         <f>SUM($D74:R74)</f>
-        <v>0</v>
+        <v>-8907.7397864993436</v>
       </c>
       <c r="S76" s="13">
         <f>SUM($D74:S74)</f>
-        <v>0</v>
+        <v>-9960.5412703745915</v>
       </c>
       <c r="T76" s="13">
         <f>SUM($D74:T74)</f>
-        <v>0</v>
+        <v>-11037.813524061175</v>
       </c>
       <c r="U76" s="13">
         <f>SUM($D74:U74)</f>
-        <v>0</v>
+        <v>-12133.311409275477</v>
       </c>
       <c r="V76" s="13">
         <f>SUM($D74:V74)</f>
-        <v>0</v>
+        <v>-13243.731487745641</v>
       </c>
       <c r="W76" s="13">
         <f>SUM($D74:W74)</f>
-        <v>0</v>
+        <v>-14366.59320895386</v>
       </c>
       <c r="X76" s="13">
         <f>SUM($D74:X74)</f>
-        <v>0</v>
+        <v>-15500.660178885671</v>
       </c>
       <c r="Y76" s="13">
         <f>SUM($D74:Y74)</f>
-        <v>0</v>
+        <v>-16645.636694329121</v>
       </c>
       <c r="Z76" s="13">
         <f>SUM($D74:Z74)</f>
-        <v>0</v>
+        <v>-17801.931221286544</v>
       </c>
       <c r="AA76" s="13">
         <f>SUM($D74:AA74)</f>
-        <v>0</v>
+        <v>-18970.214202048057</v>
       </c>
     </row>
     <row r="78" spans="1:27" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: set all input values to zero.
</commit_message>
<xml_diff>
--- a/src/assets/payload.xlsx
+++ b/src/assets/payload.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RoberJe\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5306A69-D3D3-41AC-9ACF-B25481407061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{373C16C6-4C39-4F12-902D-FD916BDA9701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" firstSheet="1" activeTab="1" xr2:uid="{983CEFC8-2B83-4647-BCB1-636BCC2A5490}"/>
   </bookViews>
@@ -2412,7 +2412,7 @@
         <v>149</v>
       </c>
       <c r="M3" s="151">
-        <v>123456</v>
+        <v>0</v>
       </c>
       <c r="N3" s="151">
         <v>0</v>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="M4" s="140">
         <f>'For user (EN)'!D6</f>
-        <v>-123456</v>
+        <v>0</v>
       </c>
       <c r="N4" s="140">
         <f>'For user (EN)'!E6</f>
@@ -2496,23 +2496,23 @@
       </c>
       <c r="M5" s="140">
         <f>'For user (EN)'!D10</f>
-        <v>-2097.3963156339423</v>
+        <v>0</v>
       </c>
       <c r="N5" s="140">
         <f>'For user (EN)'!E10</f>
-        <v>-3785.6994555609681</v>
+        <v>0</v>
       </c>
       <c r="O5" s="140">
         <f>'For user (EN)'!F10</f>
-        <v>-4077.4454991796802</v>
+        <v>0</v>
       </c>
       <c r="P5" s="140">
         <f>'For user (EN)'!G10</f>
-        <v>-4406.0519385792704</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="140">
         <f>'For user (EN)'!H10</f>
-        <v>-4603.6209930941995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="105" x14ac:dyDescent="0.25">
@@ -2544,23 +2544,23 @@
       </c>
       <c r="M6" s="140">
         <f>'For user (EN)'!D12</f>
-        <v>-125553.39631563395</v>
+        <v>0</v>
       </c>
       <c r="N6" s="140">
         <f>'For user (EN)'!E12</f>
-        <v>-3785.6994555609681</v>
+        <v>0</v>
       </c>
       <c r="O6" s="140">
         <f>'For user (EN)'!F12</f>
-        <v>-4077.4454991796802</v>
+        <v>0</v>
       </c>
       <c r="P6" s="140">
         <f>'For user (EN)'!G12</f>
-        <v>-4406.0519385792704</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="140">
         <f>'For user (EN)'!H12</f>
-        <v>-4603.6209930941995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -2588,23 +2588,23 @@
       </c>
       <c r="M7" s="140">
         <f>'For user (EN)'!D11</f>
-        <v>-125553.39631563395</v>
+        <v>0</v>
       </c>
       <c r="N7" s="140">
         <f>'For user (EN)'!E11</f>
-        <v>-129339.09577119492</v>
+        <v>0</v>
       </c>
       <c r="O7" s="140">
         <f>'For user (EN)'!F11</f>
-        <v>-133416.54127037461</v>
+        <v>0</v>
       </c>
       <c r="P7" s="140">
         <f>'For user (EN)'!G11</f>
-        <v>-137822.59320895391</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="140">
         <f>'For user (EN)'!H11</f>
-        <v>-142426.21420204811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -2632,23 +2632,23 @@
       </c>
       <c r="M8" s="140">
         <f>'For user (EN)'!D13</f>
-        <v>-2097.3963156339423</v>
+        <v>0</v>
       </c>
       <c r="N8" s="140">
         <f>'For user (EN)'!E13</f>
-        <v>-5883.0957711949104</v>
+        <v>0</v>
       </c>
       <c r="O8" s="140">
         <f>'For user (EN)'!F13</f>
-        <v>-9960.5412703745897</v>
+        <v>0</v>
       </c>
       <c r="P8" s="140">
         <f>'For user (EN)'!G13</f>
-        <v>-14366.59320895386</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="140">
         <f>'For user (EN)'!H13</f>
-        <v>-18970.214202048061</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -3014,23 +3014,23 @@
       <c r="L16" s="142"/>
       <c r="M16" s="145">
         <f>SUM(Model!E20,Model!E21)</f>
-        <v>-2097.3963156339423</v>
+        <v>0</v>
       </c>
       <c r="N16" s="145">
         <f>SUM(Model!F20,Model!F21)</f>
-        <v>-3785.6994555609681</v>
+        <v>0</v>
       </c>
       <c r="O16" s="145">
         <f>SUM(Model!G20,Model!G21)</f>
-        <v>-4077.4454991796802</v>
+        <v>0</v>
       </c>
       <c r="P16" s="145">
         <f>SUM(Model!H20,Model!H21)</f>
-        <v>-4406.0519385792704</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="145">
         <f>SUM(Model!I20,Model!I21)</f>
-        <v>-4603.6209930941995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
@@ -3060,23 +3060,23 @@
       <c r="L17" s="142"/>
       <c r="M17" s="145">
         <f>Model!E22</f>
-        <v>125553.39631563393</v>
+        <v>0</v>
       </c>
       <c r="N17" s="145">
         <f>Model!F22</f>
-        <v>3785.6994555609681</v>
+        <v>0</v>
       </c>
       <c r="O17" s="145">
         <f>Model!G22</f>
-        <v>4077.4454991796802</v>
+        <v>0</v>
       </c>
       <c r="P17" s="145">
         <f>Model!H22</f>
-        <v>4406.0519385792704</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="145">
         <f>Model!I22</f>
-        <v>4603.6209930941995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
@@ -3106,23 +3106,23 @@
       <c r="L18" s="142"/>
       <c r="M18" s="145">
         <f>Model!E23</f>
-        <v>125553.39631563395</v>
+        <v>0</v>
       </c>
       <c r="N18" s="145">
         <f>Model!F23</f>
-        <v>129339.09577119492</v>
+        <v>0</v>
       </c>
       <c r="O18" s="145">
         <f>Model!G23</f>
-        <v>133416.54127037461</v>
+        <v>0</v>
       </c>
       <c r="P18" s="145">
         <f>Model!H23</f>
-        <v>137822.59320895391</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="145">
         <f>Model!I23</f>
-        <v>142426.21420204811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
@@ -3152,23 +3152,23 @@
       <c r="L19" s="142"/>
       <c r="M19" s="145">
         <f>Model!E26</f>
-        <v>88879.415512061503</v>
+        <v>0</v>
       </c>
       <c r="N19" s="145">
         <f>Model!F26</f>
-        <v>25830.01913345986</v>
+        <v>0</v>
       </c>
       <c r="O19" s="145">
         <f>Model!G26</f>
-        <v>30231.985080879742</v>
+        <v>0</v>
       </c>
       <c r="P19" s="145">
         <f>Model!H26</f>
-        <v>20275.796400470554</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="145">
         <f>Model!I26</f>
-        <v>14202.285043145159</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.25">
@@ -3198,23 +3198,23 @@
       <c r="L20" s="142"/>
       <c r="M20" s="145">
         <f>Model!E30</f>
-        <v>63396.506169442466</v>
+        <v>0</v>
       </c>
       <c r="N20" s="145">
         <f>Model!F30</f>
-        <v>18424.209451838502</v>
+        <v>0</v>
       </c>
       <c r="O20" s="145">
         <f>Model!G30</f>
-        <v>21564.073274473656</v>
+        <v>0</v>
       </c>
       <c r="P20" s="145">
         <f>Model!H30</f>
-        <v>14462.45617376221</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="145">
         <f>Model!I30</f>
-        <v>10130.301219586054</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
@@ -3244,23 +3244,23 @@
       <c r="L21" s="142"/>
       <c r="M21" s="145">
         <f>Model!E31</f>
-        <v>35116.692142877444</v>
+        <v>0</v>
       </c>
       <c r="N21" s="145">
         <f>Model!F31</f>
-        <v>10205.56700028309</v>
+        <v>0</v>
       </c>
       <c r="O21" s="145">
         <f>Model!G31</f>
-        <v>11944.805294193742</v>
+        <v>0</v>
       </c>
       <c r="P21" s="145">
         <f>Model!H31</f>
-        <v>8011.066409976127</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="145">
         <f>Model!I31</f>
-        <v>5611.3923422216876</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
@@ -3290,23 +3290,23 @@
       <c r="L22" s="142"/>
       <c r="M22" s="145">
         <f>Model!E33</f>
-        <v>61839.217508747482</v>
+        <v>0</v>
       </c>
       <c r="N22" s="145">
         <f>Model!F33</f>
-        <v>50674.096130020487</v>
+        <v>0</v>
       </c>
       <c r="O22" s="145">
         <f>Model!G33</f>
-        <v>22371.355697754247</v>
+        <v>0</v>
       </c>
       <c r="P22" s="145">
         <f>Model!H33</f>
-        <v>27505.496779842266</v>
+        <v>0</v>
       </c>
       <c r="Q22" s="145">
         <f>Model!I33</f>
-        <v>12655.608626874198</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
@@ -3344,15 +3344,15 @@
       </c>
       <c r="O23" s="145">
         <f>Model!G37</f>
-        <v>37292.062452613216</v>
+        <v>0</v>
       </c>
       <c r="P23" s="145">
         <f>Model!H37</f>
-        <v>10837.770265787354</v>
+        <v>0</v>
       </c>
       <c r="Q23" s="145">
         <f>Model!I37</f>
-        <v>12684.748984984504</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
@@ -3382,23 +3382,23 @@
       <c r="L24" s="142"/>
       <c r="M24" s="145">
         <f>Model!E39</f>
-        <v>27040.198003314028</v>
+        <v>0</v>
       </c>
       <c r="N24" s="145">
         <f>Model!F39</f>
-        <v>2196.1210067534025</v>
+        <v>0</v>
       </c>
       <c r="O24" s="145">
         <f>Model!G39</f>
-        <v>10056.750389878895</v>
+        <v>0</v>
       </c>
       <c r="P24" s="145">
         <f>Model!H39</f>
-        <v>2827.0500105071801</v>
+        <v>0</v>
       </c>
       <c r="Q24" s="145">
         <f>Model!I39</f>
-        <v>4373.7264267781402</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
@@ -3428,23 +3428,23 @@
       <c r="L25" s="142"/>
       <c r="M25" s="145">
         <f>Model!E43</f>
-        <v>63396.506169442466</v>
+        <v>0</v>
       </c>
       <c r="N25" s="145">
         <f>Model!F43</f>
-        <v>81820.715621280979</v>
+        <v>0</v>
       </c>
       <c r="O25" s="145">
         <f>Model!G43</f>
-        <v>66092.726443141408</v>
+        <v>0</v>
       </c>
       <c r="P25" s="145">
         <f>Model!H43</f>
-        <v>69717.412351116276</v>
+        <v>0</v>
       </c>
       <c r="Q25" s="145">
         <f>Model!I43</f>
-        <v>67162.964585717826</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
@@ -3474,23 +3474,23 @@
       <c r="L26" s="142"/>
       <c r="M26" s="145">
         <f>Model!E44</f>
-        <v>35116.692142877444</v>
+        <v>0</v>
       </c>
       <c r="N26" s="145">
         <f>Model!F44</f>
-        <v>45322.259143160532</v>
+        <v>0</v>
       </c>
       <c r="O26" s="145">
         <f>Model!G44</f>
-        <v>57267.064437354275</v>
+        <v>0</v>
       </c>
       <c r="P26" s="145">
         <f>Model!H44</f>
-        <v>65278.130847330402</v>
+        <v>0</v>
       </c>
       <c r="Q26" s="145">
         <f>Model!I44</f>
-        <v>70889.523189552085</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="16:16" x14ac:dyDescent="0.25">
@@ -3614,7 +3614,7 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4">
         <f>machine_readable!M3</f>
-        <v>123456</v>
+        <v>0</v>
       </c>
       <c r="E5" s="4">
         <f>machine_readable!N3</f>
@@ -3643,7 +3643,7 @@
       <c r="C6" s="59"/>
       <c r="D6" s="59">
         <f t="shared" ref="D6:G6" si="2">D4-D5</f>
-        <v>-123456</v>
+        <v>0</v>
       </c>
       <c r="E6" s="59">
         <f t="shared" si="2"/>
@@ -3684,23 +3684,23 @@
       <c r="C10" s="13"/>
       <c r="D10" s="13">
         <f>Model!E53</f>
-        <v>-2097.3963156339423</v>
+        <v>0</v>
       </c>
       <c r="E10" s="13">
         <f>Model!F53</f>
-        <v>-3785.6994555609681</v>
+        <v>0</v>
       </c>
       <c r="F10" s="13">
         <f>Model!G53</f>
-        <v>-4077.4454991796802</v>
+        <v>0</v>
       </c>
       <c r="G10" s="13">
         <f>Model!H53</f>
-        <v>-4406.0519385792704</v>
+        <v>0</v>
       </c>
       <c r="H10" s="13">
         <f>Model!I53</f>
-        <v>-4603.6209930941995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -3713,23 +3713,23 @@
       <c r="C11" s="13"/>
       <c r="D11" s="13">
         <f>Model!E54</f>
-        <v>-125553.39631563395</v>
+        <v>0</v>
       </c>
       <c r="E11" s="13">
         <f>Model!F54</f>
-        <v>-129339.09577119492</v>
+        <v>0</v>
       </c>
       <c r="F11" s="13">
         <f>Model!G54</f>
-        <v>-133416.54127037461</v>
+        <v>0</v>
       </c>
       <c r="G11" s="13">
         <f>Model!H54</f>
-        <v>-137822.59320895391</v>
+        <v>0</v>
       </c>
       <c r="H11" s="13">
         <f>Model!I54</f>
-        <v>-142426.21420204811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -3742,23 +3742,23 @@
       <c r="C12" s="13"/>
       <c r="D12" s="13">
         <f>Model!E53+Model!E6</f>
-        <v>-125553.39631563395</v>
+        <v>0</v>
       </c>
       <c r="E12" s="13">
         <f>Model!F53+Model!F6</f>
-        <v>-3785.6994555609681</v>
+        <v>0</v>
       </c>
       <c r="F12" s="13">
         <f>Model!G53+Model!G6</f>
-        <v>-4077.4454991796802</v>
+        <v>0</v>
       </c>
       <c r="G12" s="13">
         <f>Model!H53+Model!H6</f>
-        <v>-4406.0519385792704</v>
+        <v>0</v>
       </c>
       <c r="H12" s="13">
         <f>Model!I53+Model!I6</f>
-        <v>-4603.6209930941995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -3771,23 +3771,23 @@
       <c r="C13" s="50"/>
       <c r="D13" s="50">
         <f>SUM($C10:D10)</f>
-        <v>-2097.3963156339423</v>
+        <v>0</v>
       </c>
       <c r="E13" s="50">
         <f>SUM($C10:E10)</f>
-        <v>-5883.0957711949104</v>
+        <v>0</v>
       </c>
       <c r="F13" s="50">
         <f>SUM($C10:F10)</f>
-        <v>-9960.5412703745897</v>
+        <v>0</v>
       </c>
       <c r="G13" s="50">
         <f>SUM($C10:G10)</f>
-        <v>-14366.59320895386</v>
+        <v>0</v>
       </c>
       <c r="H13" s="50">
         <f>SUM($C10:H10)</f>
-        <v>-18970.214202048061</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="90" x14ac:dyDescent="0.25">
@@ -3941,7 +3941,7 @@
       </c>
       <c r="E5" s="59">
         <f>'For user (EN)'!D5</f>
-        <v>123456</v>
+        <v>0</v>
       </c>
       <c r="F5" s="59">
         <f>'For user (EN)'!E5</f>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="E6" s="59">
         <f>'For user (EN)'!D6</f>
-        <v>-123456</v>
+        <v>0</v>
       </c>
       <c r="F6" s="59">
         <f>'For user (EN)'!E6</f>
@@ -4346,7 +4346,7 @@
       </c>
       <c r="E20" s="9">
         <f>SUM('Model Quarterly'!H19:K19)</f>
-        <v>-813.95439603616876</v>
+        <v>0</v>
       </c>
       <c r="F20" s="9">
         <f>SUM('Model Quarterly'!L19:O19)</f>
@@ -4380,23 +4380,23 @@
       </c>
       <c r="E21" s="9">
         <f>E53-E20</f>
-        <v>-1283.4419195977734</v>
+        <v>0</v>
       </c>
       <c r="F21" s="9">
         <f>F53-F20</f>
-        <v>-3785.6994555609681</v>
+        <v>0</v>
       </c>
       <c r="G21" s="9">
         <f t="shared" si="1"/>
-        <v>-4077.4454991796802</v>
+        <v>0</v>
       </c>
       <c r="H21" s="9">
         <f t="shared" si="1"/>
-        <v>-4406.0519385792704</v>
+        <v>0</v>
       </c>
       <c r="I21" s="9">
         <f t="shared" si="1"/>
-        <v>-4603.6209930941995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:23" ht="26.25" x14ac:dyDescent="0.25">
@@ -4413,23 +4413,23 @@
       </c>
       <c r="E22" s="9">
         <f>-(E6+E20+E21)</f>
-        <v>125553.39631563393</v>
+        <v>0</v>
       </c>
       <c r="F22" s="9">
         <f>-(F6+F20+F21)</f>
-        <v>3785.6994555609681</v>
+        <v>0</v>
       </c>
       <c r="G22" s="9">
         <f t="shared" si="2"/>
-        <v>4077.4454991796802</v>
+        <v>0</v>
       </c>
       <c r="H22" s="9">
         <f t="shared" si="2"/>
-        <v>4406.0519385792704</v>
+        <v>0</v>
       </c>
       <c r="I22" s="9">
         <f>-(I6+I20+I21)</f>
-        <v>4603.6209930941995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:23" ht="26.25" x14ac:dyDescent="0.25">
@@ -4446,23 +4446,23 @@
       </c>
       <c r="E23" s="9">
         <f t="shared" si="3"/>
-        <v>125553.39631563395</v>
+        <v>0</v>
       </c>
       <c r="F23" s="9">
         <f t="shared" si="3"/>
-        <v>129339.09577119492</v>
+        <v>0</v>
       </c>
       <c r="G23" s="9">
         <f t="shared" si="3"/>
-        <v>133416.54127037461</v>
+        <v>0</v>
       </c>
       <c r="H23" s="9">
         <f t="shared" si="3"/>
-        <v>137822.59320895391</v>
+        <v>0</v>
       </c>
       <c r="I23" s="9">
         <f t="shared" si="3"/>
-        <v>142426.21420204811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
@@ -4503,23 +4503,23 @@
       </c>
       <c r="E26" s="60">
         <f>SUM('Model Quarterly'!H28:K28)</f>
-        <v>88879.415512061503</v>
+        <v>0</v>
       </c>
       <c r="F26" s="60">
         <f>SUM('Model Quarterly'!L28:O28)</f>
-        <v>25830.01913345986</v>
+        <v>0</v>
       </c>
       <c r="G26" s="60">
         <f>SUM('Model Quarterly'!P28:S28)</f>
-        <v>30231.985080879742</v>
+        <v>0</v>
       </c>
       <c r="H26" s="60">
         <f>SUM('Model Quarterly'!T28:W28)</f>
-        <v>20275.796400470554</v>
+        <v>0</v>
       </c>
       <c r="I26" s="60">
         <f>SUM('Model Quarterly'!X28:AA28)</f>
-        <v>14202.285043145159</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:23" ht="26.25" x14ac:dyDescent="0.25">
@@ -4536,23 +4536,23 @@
       </c>
       <c r="E27" s="60">
         <f>SUM('Model Quarterly'!H29:K29)</f>
-        <v>37292.062452613216</v>
+        <v>0</v>
       </c>
       <c r="F27" s="60">
         <f>SUM('Model Quarterly'!L29:O29)</f>
-        <v>10837.770265787354</v>
+        <v>0</v>
       </c>
       <c r="G27" s="60">
         <f>SUM('Model Quarterly'!P29:S29)</f>
-        <v>12684.748984984504</v>
+        <v>0</v>
       </c>
       <c r="H27" s="60">
         <f>SUM('Model Quarterly'!T29:W29)</f>
-        <v>8507.3271610365955</v>
+        <v>0</v>
       </c>
       <c r="I27" s="60">
         <f>SUM('Model Quarterly'!X29:AA29)</f>
-        <v>5959.0007174035618</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:23" ht="26.25" x14ac:dyDescent="0.25">
@@ -4602,23 +4602,23 @@
       </c>
       <c r="E29" s="60">
         <f>SUM('Model Quarterly'!H31:K31)</f>
-        <v>26104.44371682925</v>
+        <v>0</v>
       </c>
       <c r="F29" s="60">
         <f>SUM('Model Quarterly'!L31:O31)</f>
-        <v>7586.4391860511469</v>
+        <v>0</v>
       </c>
       <c r="G29" s="60">
         <f>SUM('Model Quarterly'!P31:S31)</f>
-        <v>8879.3242894891519</v>
+        <v>0</v>
       </c>
       <c r="H29" s="60">
         <f>SUM('Model Quarterly'!T31:W31)</f>
-        <v>5955.1290127256152</v>
+        <v>0</v>
       </c>
       <c r="I29" s="60">
         <f>SUM('Model Quarterly'!X31:AA31)</f>
-        <v>4171.3005021824929</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
@@ -4635,23 +4635,23 @@
       </c>
       <c r="E30" s="131">
         <f t="shared" ref="E30:I30" si="4">SUM(E27:E29)</f>
-        <v>63396.506169442466</v>
+        <v>0</v>
       </c>
       <c r="F30" s="131">
         <f t="shared" si="4"/>
-        <v>18424.209451838502</v>
+        <v>0</v>
       </c>
       <c r="G30" s="131">
         <f t="shared" si="4"/>
-        <v>21564.073274473656</v>
+        <v>0</v>
       </c>
       <c r="H30" s="131">
         <f t="shared" si="4"/>
-        <v>14462.45617376221</v>
+        <v>0</v>
       </c>
       <c r="I30" s="131">
         <f t="shared" si="4"/>
-        <v>10130.301219586054</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:23" ht="26.25" x14ac:dyDescent="0.25">
@@ -4668,23 +4668,23 @@
       </c>
       <c r="E31" s="60">
         <f>SUM('Model Quarterly'!H32:K32)</f>
-        <v>35116.692142877444</v>
+        <v>0</v>
       </c>
       <c r="F31" s="60">
         <f>SUM('Model Quarterly'!L32:O32)</f>
-        <v>10205.56700028309</v>
+        <v>0</v>
       </c>
       <c r="G31" s="60">
         <f>SUM('Model Quarterly'!P32:S32)</f>
-        <v>11944.805294193742</v>
+        <v>0</v>
       </c>
       <c r="H31" s="60">
         <f>SUM('Model Quarterly'!T32:W32)</f>
-        <v>8011.066409976127</v>
+        <v>0</v>
       </c>
       <c r="I31" s="60">
         <f>SUM('Model Quarterly'!X32:AA32)</f>
-        <v>5611.3923422216876</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
@@ -4712,23 +4712,23 @@
       </c>
       <c r="E33" s="60">
         <f>SUM('Model Quarterly'!H55:K55)</f>
-        <v>61839.217508747482</v>
+        <v>0</v>
       </c>
       <c r="F33" s="60">
         <f>SUM('Model Quarterly'!L55:O55)</f>
-        <v>50674.096130020487</v>
+        <v>0</v>
       </c>
       <c r="G33" s="60">
         <f>SUM('Model Quarterly'!P55:S55)</f>
-        <v>22371.355697754247</v>
+        <v>0</v>
       </c>
       <c r="H33" s="60">
         <f>SUM('Model Quarterly'!T55:W55)</f>
-        <v>27505.496779842266</v>
+        <v>0</v>
       </c>
       <c r="I33" s="60">
         <f>SUM('Model Quarterly'!X55:AA55)</f>
-        <v>12655.608626874198</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -4753,15 +4753,15 @@
       </c>
       <c r="G34" s="60">
         <f>SUM('Model Quarterly'!P56:S56)</f>
-        <v>37292.062452613216</v>
+        <v>0</v>
       </c>
       <c r="H34" s="60">
         <f>SUM('Model Quarterly'!T56:W56)</f>
-        <v>10837.770265787354</v>
+        <v>0</v>
       </c>
       <c r="I34" s="60">
         <f>SUM('Model Quarterly'!X56:AA56)</f>
-        <v>12684.748984984504</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -4852,15 +4852,15 @@
       </c>
       <c r="G37" s="60">
         <f>SUM('Model Quarterly'!P59:S59)</f>
-        <v>37292.062452613216</v>
+        <v>0</v>
       </c>
       <c r="H37" s="60">
         <f>SUM('Model Quarterly'!T59:W59)</f>
-        <v>10837.770265787354</v>
+        <v>0</v>
       </c>
       <c r="I37" s="60">
         <f>SUM('Model Quarterly'!X59:AA59)</f>
-        <v>12684.748984984504</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -4888,23 +4888,23 @@
       </c>
       <c r="E39" s="60">
         <f>'Model Quarterly'!K36</f>
-        <v>27040.198003314028</v>
+        <v>0</v>
       </c>
       <c r="F39" s="60">
         <f>'Model Quarterly'!O36</f>
-        <v>2196.1210067534025</v>
+        <v>0</v>
       </c>
       <c r="G39" s="60">
         <f>'Model Quarterly'!S36</f>
-        <v>10056.750389878895</v>
+        <v>0</v>
       </c>
       <c r="H39" s="60">
         <f>'Model Quarterly'!W36</f>
-        <v>2827.0500105071801</v>
+        <v>0</v>
       </c>
       <c r="I39" s="60">
         <f>'Model Quarterly'!AA36</f>
-        <v>4373.7264267781402</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="26.25" x14ac:dyDescent="0.25">
@@ -4921,23 +4921,23 @@
       </c>
       <c r="E40" s="60">
         <f>'Model Quarterly'!K37</f>
-        <v>37292.062452613216</v>
+        <v>0</v>
       </c>
       <c r="F40" s="60">
         <f>'Model Quarterly'!O37</f>
-        <v>48129.832718400576</v>
+        <v>0</v>
       </c>
       <c r="G40" s="60">
         <f>'Model Quarterly'!S37</f>
-        <v>23522.519250771864</v>
+        <v>0</v>
       </c>
       <c r="H40" s="60">
         <f>'Model Quarterly'!W37</f>
-        <v>21192.076146021111</v>
+        <v>0</v>
       </c>
       <c r="I40" s="60">
         <f>'Model Quarterly'!AA37</f>
-        <v>14466.32787844017</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="26.25" x14ac:dyDescent="0.25">
@@ -4987,23 +4987,23 @@
       </c>
       <c r="E42" s="60">
         <f>'Model Quarterly'!K39</f>
-        <v>26104.44371682925</v>
+        <v>0</v>
       </c>
       <c r="F42" s="60">
         <f>'Model Quarterly'!O39</f>
-        <v>33690.882902880396</v>
+        <v>0</v>
       </c>
       <c r="G42" s="60">
         <f>'Model Quarterly'!S39</f>
-        <v>42570.207192369548</v>
+        <v>0</v>
       </c>
       <c r="H42" s="60">
         <f>'Model Quarterly'!W39</f>
-        <v>48525.336205095162</v>
+        <v>0</v>
       </c>
       <c r="I42" s="60">
         <f>'Model Quarterly'!AA39</f>
-        <v>52696.636707277656</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -5020,23 +5020,23 @@
       </c>
       <c r="E43" s="60">
         <f>'Model Quarterly'!K40</f>
-        <v>63396.506169442466</v>
+        <v>0</v>
       </c>
       <c r="F43" s="60">
         <f>'Model Quarterly'!O40</f>
-        <v>81820.715621280979</v>
+        <v>0</v>
       </c>
       <c r="G43" s="60">
         <f>'Model Quarterly'!S40</f>
-        <v>66092.726443141408</v>
+        <v>0</v>
       </c>
       <c r="H43" s="60">
         <f>'Model Quarterly'!W40</f>
-        <v>69717.412351116276</v>
+        <v>0</v>
       </c>
       <c r="I43" s="60">
         <f>'Model Quarterly'!AA40</f>
-        <v>67162.964585717826</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="26.25" x14ac:dyDescent="0.25">
@@ -5053,23 +5053,23 @@
       </c>
       <c r="E44" s="60">
         <f>'Model Quarterly'!K41</f>
-        <v>35116.692142877444</v>
+        <v>0</v>
       </c>
       <c r="F44" s="60">
         <f>'Model Quarterly'!O41</f>
-        <v>45322.259143160532</v>
+        <v>0</v>
       </c>
       <c r="G44" s="60">
         <f>'Model Quarterly'!S41</f>
-        <v>57267.064437354275</v>
+        <v>0</v>
       </c>
       <c r="H44" s="60">
         <f>'Model Quarterly'!W41</f>
-        <v>65278.130847330402</v>
+        <v>0</v>
       </c>
       <c r="I44" s="60">
         <f>'Model Quarterly'!AA41</f>
-        <v>70889.523189552085</v>
+        <v>0</v>
       </c>
       <c r="J44" s="67"/>
     </row>
@@ -5087,23 +5087,23 @@
       </c>
       <c r="E45" s="58">
         <f t="shared" si="5"/>
-        <v>0.21536811266607667</v>
+        <v>0</v>
       </c>
       <c r="F45" s="58">
         <f t="shared" si="5"/>
-        <v>1.6979560539362455E-2</v>
+        <v>0</v>
       </c>
       <c r="G45" s="58">
         <f t="shared" si="5"/>
-        <v>7.5378587198557626E-2</v>
+        <v>0</v>
       </c>
       <c r="H45" s="58">
         <f t="shared" si="5"/>
-        <v>2.051223928301122E-2</v>
+        <v>0</v>
       </c>
       <c r="I45" s="58">
         <f>IF(I23=0,0,I39/I23)</f>
-        <v>3.0708717852835025E-2</v>
+        <v>0</v>
       </c>
       <c r="J45" s="66"/>
       <c r="K45" s="66"/>
@@ -5125,23 +5125,23 @@
       </c>
       <c r="E46" s="58">
         <f t="shared" si="6"/>
-        <v>0.29702153463744729</v>
+        <v>0</v>
       </c>
       <c r="F46" s="58">
         <f t="shared" si="6"/>
-        <v>0.37212130200402688</v>
+        <v>0</v>
       </c>
       <c r="G46" s="58">
         <f t="shared" si="6"/>
-        <v>0.17630886715240521</v>
+        <v>0</v>
       </c>
       <c r="H46" s="58">
         <f t="shared" si="6"/>
-        <v>0.15376344075816104</v>
+        <v>0</v>
       </c>
       <c r="I46" s="58">
         <f>IF(I$23=0,0,I40/I$23)</f>
-        <v>0.10157068317436287</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -5191,23 +5191,23 @@
       </c>
       <c r="E48" s="58">
         <f t="shared" ref="E48:H48" si="7">IF(E$23=0,0,E42/E$23)</f>
-        <v>0.20791507424621311</v>
+        <v>0</v>
       </c>
       <c r="F48" s="58">
         <f t="shared" si="7"/>
-        <v>0.26048491140281876</v>
+        <v>0</v>
       </c>
       <c r="G48" s="58">
         <f t="shared" si="7"/>
-        <v>0.31907743063207666</v>
+        <v>0</v>
       </c>
       <c r="H48" s="58">
         <f t="shared" si="7"/>
-        <v>0.35208549683523599</v>
+        <v>0</v>
       </c>
       <c r="I48" s="58">
         <f>IF(I$23=0,0,I42/I$23)</f>
-        <v>0.36999253966352963</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
@@ -5224,23 +5224,23 @@
       </c>
       <c r="E49" s="58">
         <f t="shared" si="8"/>
-        <v>0.27969527845026287</v>
+        <v>0</v>
       </c>
       <c r="F49" s="58">
         <f t="shared" si="8"/>
-        <v>0.35041422605379186</v>
+        <v>0</v>
       </c>
       <c r="G49" s="58">
         <f t="shared" si="8"/>
-        <v>0.42923511501696027</v>
+        <v>0</v>
       </c>
       <c r="H49" s="58">
         <f t="shared" si="8"/>
-        <v>0.47363882312359135</v>
+        <v>0</v>
       </c>
       <c r="I49" s="58">
         <f t="shared" si="8"/>
-        <v>0.49772805930927205</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -5286,23 +5286,23 @@
       </c>
       <c r="E53" s="13">
         <f>SUM('Model Quarterly'!H74:K74)</f>
-        <v>-2097.3963156339423</v>
+        <v>0</v>
       </c>
       <c r="F53" s="13">
         <f>SUM('Model Quarterly'!L74:O74)</f>
-        <v>-3785.6994555609681</v>
+        <v>0</v>
       </c>
       <c r="G53" s="13">
         <f>SUM('Model Quarterly'!P74:S74)</f>
-        <v>-4077.4454991796802</v>
+        <v>0</v>
       </c>
       <c r="H53" s="13">
         <f>SUM('Model Quarterly'!T74:W74)</f>
-        <v>-4406.0519385792704</v>
+        <v>0</v>
       </c>
       <c r="I53" s="13">
         <f>SUM('Model Quarterly'!X74:AA74)</f>
-        <v>-4603.6209930941995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -5317,23 +5317,23 @@
       </c>
       <c r="E54" s="13">
         <f>'Model Quarterly'!K75</f>
-        <v>-125553.39631563395</v>
+        <v>0</v>
       </c>
       <c r="F54" s="13">
         <f>'Model Quarterly'!O75</f>
-        <v>-129339.09577119492</v>
+        <v>0</v>
       </c>
       <c r="G54" s="13">
         <f>'Model Quarterly'!S75</f>
-        <v>-133416.54127037461</v>
+        <v>0</v>
       </c>
       <c r="H54" s="13">
         <f>'Model Quarterly'!W75</f>
-        <v>-137822.59320895391</v>
+        <v>0</v>
       </c>
       <c r="I54" s="13">
         <f>'Model Quarterly'!AA75</f>
-        <v>-142426.21420204811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -5348,23 +5348,23 @@
       </c>
       <c r="E55" s="13">
         <f>SUM($D53:E53)</f>
-        <v>-2097.3963156339423</v>
+        <v>0</v>
       </c>
       <c r="F55" s="13">
         <f>SUM($D53:F53)</f>
-        <v>-5883.0957711949104</v>
+        <v>0</v>
       </c>
       <c r="G55" s="13">
         <f>SUM($D53:G53)</f>
-        <v>-9960.5412703745897</v>
+        <v>0</v>
       </c>
       <c r="H55" s="13">
         <f>SUM($D53:H53)</f>
-        <v>-14366.59320895386</v>
+        <v>0</v>
       </c>
       <c r="I55" s="13">
         <f>SUM($D53:I53)</f>
-        <v>-18970.214202048061</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -5831,19 +5831,19 @@
       </c>
       <c r="H6" s="59">
         <f>'For user (EN)'!D5/4</f>
-        <v>30864</v>
+        <v>0</v>
       </c>
       <c r="I6" s="59">
         <f>'For user (EN)'!$D5/4</f>
-        <v>30864</v>
+        <v>0</v>
       </c>
       <c r="J6" s="59">
         <f>'For user (EN)'!$D5/4</f>
-        <v>30864</v>
+        <v>0</v>
       </c>
       <c r="K6" s="59">
         <f>'For user (EN)'!$D5/4</f>
-        <v>30864</v>
+        <v>0</v>
       </c>
       <c r="L6" s="4">
         <f>'For user (EN)'!$E5/4</f>
@@ -5936,19 +5936,19 @@
       </c>
       <c r="H7" s="59">
         <f>'For user (EN)'!D6/4</f>
-        <v>-30864</v>
+        <v>0</v>
       </c>
       <c r="I7" s="59">
         <f>'For user (EN)'!$D6/4</f>
-        <v>-30864</v>
+        <v>0</v>
       </c>
       <c r="J7" s="59">
         <f>'For user (EN)'!$D6/4</f>
-        <v>-30864</v>
+        <v>0</v>
       </c>
       <c r="K7" s="59">
         <f>'For user (EN)'!$D6/4</f>
-        <v>-30864</v>
+        <v>0</v>
       </c>
       <c r="L7" s="4">
         <f>'For user (EN)'!$E6/4</f>
@@ -6793,19 +6793,19 @@
       </c>
       <c r="H19" s="9">
         <f>(H16/100)*H7/4</f>
-        <v>-201.81034552475003</v>
+        <v>0</v>
       </c>
       <c r="I19" s="9">
         <f t="shared" si="0"/>
-        <v>-202.52156529639294</v>
+        <v>0</v>
       </c>
       <c r="J19" s="9">
         <f t="shared" si="0"/>
-        <v>-204.02013832074425</v>
+        <v>0</v>
       </c>
       <c r="K19" s="9">
         <f t="shared" si="0"/>
-        <v>-205.60234689428162</v>
+        <v>0</v>
       </c>
       <c r="L19" s="9">
         <f>(L16/100)*L7/4</f>
@@ -6902,79 +6902,79 @@
       </c>
       <c r="I20" s="9">
         <f>(H71/100)*H75/4</f>
-        <v>-203.12992223421153</v>
+        <v>0</v>
       </c>
       <c r="J20" s="9">
         <f>(I71/100)*I75/4</f>
-        <v>-423.95734198623109</v>
+        <v>0</v>
       </c>
       <c r="K20" s="9">
         <f t="shared" si="2"/>
-        <v>-656.35465537733103</v>
+        <v>0</v>
       </c>
       <c r="L20" s="9">
         <f>(K71/100)*K75/4</f>
-        <v>-897.06941973413893</v>
+        <v>0</v>
       </c>
       <c r="M20" s="9">
         <f t="shared" si="2"/>
-        <v>-944.93078222515908</v>
+        <v>0</v>
       </c>
       <c r="N20" s="9">
         <f t="shared" si="2"/>
-        <v>-963.97265559273126</v>
+        <v>0</v>
       </c>
       <c r="O20" s="9">
         <f t="shared" si="2"/>
-        <v>-979.72659800893848</v>
+        <v>0</v>
       </c>
       <c r="P20" s="9">
         <f t="shared" si="2"/>
-        <v>-989.37120580302053</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="9">
         <f t="shared" si="2"/>
-        <v>-1006.5780005652127</v>
+        <v>0</v>
       </c>
       <c r="R20" s="9">
         <f t="shared" si="2"/>
-        <v>-1028.694808936199</v>
+        <v>0</v>
       </c>
       <c r="S20" s="9">
         <f t="shared" si="2"/>
-        <v>-1052.8014838752481</v>
+        <v>0</v>
       </c>
       <c r="T20" s="9">
         <f>(S71/100)*S75/4</f>
-        <v>-1077.2722536865842</v>
+        <v>0</v>
       </c>
       <c r="U20" s="9">
         <f t="shared" si="2"/>
-        <v>-1095.497885214302</v>
+        <v>0</v>
       </c>
       <c r="V20" s="9">
         <f t="shared" si="2"/>
-        <v>-1110.4200784701648</v>
+        <v>0</v>
       </c>
       <c r="W20" s="9">
         <f t="shared" si="2"/>
-        <v>-1122.8617212082197</v>
+        <v>0</v>
       </c>
       <c r="X20" s="9">
         <f>(W71/100)*W75/4</f>
-        <v>-1134.0669699318119</v>
+        <v>0</v>
       </c>
       <c r="Y20" s="9">
         <f t="shared" ref="Y20" si="3">(X71/100)*X75/4</f>
-        <v>-1144.9765154434508</v>
+        <v>0</v>
       </c>
       <c r="Z20" s="9">
         <f t="shared" ref="Z20" si="4">(Y71/100)*Y75/4</f>
-        <v>-1156.2945269574238</v>
+        <v>0</v>
       </c>
       <c r="AA20" s="9">
         <f t="shared" ref="AA20" si="5">(Z71/100)*Z75/4</f>
-        <v>-1168.2829807615133</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -7003,83 +7003,83 @@
       </c>
       <c r="H21" s="9">
         <f>-(H7+H19+H20)</f>
-        <v>31065.810345524751</v>
+        <v>0</v>
       </c>
       <c r="I21" s="9">
         <f>-(I7+I19+I20)</f>
-        <v>31269.651487530606</v>
+        <v>0</v>
       </c>
       <c r="J21" s="9">
         <f>-(J7+J19+J20)</f>
-        <v>31491.977480306978</v>
+        <v>0</v>
       </c>
       <c r="K21" s="9">
         <f t="shared" si="6"/>
-        <v>31725.957002271611</v>
+        <v>0</v>
       </c>
       <c r="L21" s="9">
         <f>-(L7+L19+L20)</f>
-        <v>897.06941973413893</v>
+        <v>0</v>
       </c>
       <c r="M21" s="9">
         <f t="shared" si="6"/>
-        <v>944.93078222515908</v>
+        <v>0</v>
       </c>
       <c r="N21" s="9">
         <f t="shared" si="6"/>
-        <v>963.97265559273126</v>
+        <v>0</v>
       </c>
       <c r="O21" s="9">
         <f t="shared" si="6"/>
-        <v>979.72659800893848</v>
+        <v>0</v>
       </c>
       <c r="P21" s="9">
         <f t="shared" si="6"/>
-        <v>989.37120580302053</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="9">
         <f t="shared" si="6"/>
-        <v>1006.5780005652127</v>
+        <v>0</v>
       </c>
       <c r="R21" s="9">
         <f t="shared" si="6"/>
-        <v>1028.694808936199</v>
+        <v>0</v>
       </c>
       <c r="S21" s="9">
         <f t="shared" si="6"/>
-        <v>1052.8014838752481</v>
+        <v>0</v>
       </c>
       <c r="T21" s="9">
         <f t="shared" si="6"/>
-        <v>1077.2722536865842</v>
+        <v>0</v>
       </c>
       <c r="U21" s="9">
         <f t="shared" si="6"/>
-        <v>1095.497885214302</v>
+        <v>0</v>
       </c>
       <c r="V21" s="9">
         <f t="shared" si="6"/>
-        <v>1110.4200784701648</v>
+        <v>0</v>
       </c>
       <c r="W21" s="9">
         <f t="shared" si="6"/>
-        <v>1122.8617212082197</v>
+        <v>0</v>
       </c>
       <c r="X21" s="9">
         <f t="shared" ref="X21:AA21" si="7">-(X7+X19+X20)</f>
-        <v>1134.0669699318119</v>
+        <v>0</v>
       </c>
       <c r="Y21" s="9">
         <f t="shared" si="7"/>
-        <v>1144.9765154434508</v>
+        <v>0</v>
       </c>
       <c r="Z21" s="9">
         <f t="shared" si="7"/>
-        <v>1156.2945269574238</v>
+        <v>0</v>
       </c>
       <c r="AA21" s="9">
         <f t="shared" si="7"/>
-        <v>1168.2829807615133</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -7108,83 +7108,83 @@
       </c>
       <c r="H22" s="9">
         <f>MAX(0,SUM($D21:H21))</f>
-        <v>31065.810345524751</v>
+        <v>0</v>
       </c>
       <c r="I22" s="9">
         <f>MAX(0,SUM($D21:I21))</f>
-        <v>62335.461833055357</v>
+        <v>0</v>
       </c>
       <c r="J22" s="9">
         <f>MAX(0,SUM($D21:J21))</f>
-        <v>93827.439313362338</v>
+        <v>0</v>
       </c>
       <c r="K22" s="9">
         <f>MAX(0,SUM($D21:K21))</f>
-        <v>125553.39631563395</v>
+        <v>0</v>
       </c>
       <c r="L22" s="9">
         <f>MAX(0,SUM($D21:L21))</f>
-        <v>126450.46573536808</v>
+        <v>0</v>
       </c>
       <c r="M22" s="9">
         <f>MAX(0,SUM($D21:M21))</f>
-        <v>127395.39651759324</v>
+        <v>0</v>
       </c>
       <c r="N22" s="9">
         <f>MAX(0,SUM($D21:N21))</f>
-        <v>128359.36917318597</v>
+        <v>0</v>
       </c>
       <c r="O22" s="9">
         <f>MAX(0,SUM($D21:O21))</f>
-        <v>129339.09577119492</v>
+        <v>0</v>
       </c>
       <c r="P22" s="9">
         <f>MAX(0,SUM($D21:P21))</f>
-        <v>130328.46697699794</v>
+        <v>0</v>
       </c>
       <c r="Q22" s="9">
         <f>MAX(0,SUM($D21:Q21))</f>
-        <v>131335.04497756314</v>
+        <v>0</v>
       </c>
       <c r="R22" s="9">
         <f>MAX(0,SUM($D21:R21))</f>
-        <v>132363.73978649935</v>
+        <v>0</v>
       </c>
       <c r="S22" s="9">
         <f>MAX(0,SUM($D21:S21))</f>
-        <v>133416.54127037461</v>
+        <v>0</v>
       </c>
       <c r="T22" s="9">
         <f>MAX(0,SUM($D21:T21))</f>
-        <v>134493.8135240612</v>
+        <v>0</v>
       </c>
       <c r="U22" s="9">
         <f>MAX(0,SUM($D21:U21))</f>
-        <v>135589.31140927551</v>
+        <v>0</v>
       </c>
       <c r="V22" s="9">
         <f>MAX(0,SUM($D21:V21))</f>
-        <v>136699.73148774568</v>
+        <v>0</v>
       </c>
       <c r="W22" s="9">
         <f>MAX(0,SUM($D21:W21))</f>
-        <v>137822.59320895391</v>
+        <v>0</v>
       </c>
       <c r="X22" s="9">
         <f>MAX(0,SUM($D21:X21))</f>
-        <v>138956.66017888574</v>
+        <v>0</v>
       </c>
       <c r="Y22" s="9">
         <f>MAX(0,SUM($D21:Y21))</f>
-        <v>140101.63669432918</v>
+        <v>0</v>
       </c>
       <c r="Z22" s="9">
         <f>MAX(0,SUM($D21:Z21))</f>
-        <v>141257.93122128659</v>
+        <v>0</v>
       </c>
       <c r="AA22" s="9">
         <f>MAX(0,SUM($D21:AA21))</f>
-        <v>142426.21420204811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.25">
@@ -7273,83 +7273,83 @@
       </c>
       <c r="H25" s="9">
         <f>IF(H$22&gt;0,MIN(MAX(SUM(H$21,H$55,H$59),0),H$22)*'Fiscal Model Import'!S44,0)</f>
-        <v>14734.364442487693</v>
+        <v>0</v>
       </c>
       <c r="I25" s="9">
         <f>IF(I$22&gt;0,MIN(MAX(SUM(I$21,I$55,I$59),0),I$22)*'Fiscal Model Import'!T44,0)</f>
-        <v>21819.483509096575</v>
+        <v>0</v>
       </c>
       <c r="J25" s="9">
         <f>IF(J$22&gt;0,MIN(MAX(SUM(J$21,J$55,J$59),0),J$22)*'Fiscal Model Import'!U44,0)</f>
-        <v>25285.369557163212</v>
+        <v>0</v>
       </c>
       <c r="K25" s="9">
         <f>IF(K$22&gt;0,MIN(MAX(SUM(K$21,K$55,K$59),0),K$22)*'Fiscal Model Import'!V44,0)</f>
-        <v>27040.198003314028</v>
+        <v>0</v>
       </c>
       <c r="L25" s="9">
         <f>IF(L$22&gt;0,MIN(MAX(SUM(L$21,L$55,L$59),0),L$22)*'Fiscal Model Import'!W44,0)</f>
-        <v>13250.511580417538</v>
+        <v>0</v>
       </c>
       <c r="M25" s="9">
         <f>IF(M$22&gt;0,MIN(MAX(SUM(M$21,M$55,M$59),0),M$22)*'Fiscal Model Import'!X44,0)</f>
-        <v>6732.8300426464539</v>
+        <v>0</v>
       </c>
       <c r="N25" s="9">
         <f>IF(N$22&gt;0,MIN(MAX(SUM(N$21,N$55,N$59),0),N$22)*'Fiscal Model Import'!Y44,0)</f>
-        <v>3650.5565036424659</v>
+        <v>0</v>
       </c>
       <c r="O25" s="9">
         <f>IF(O$22&gt;0,MIN(MAX(SUM(O$21,O$55,O$59),0),O$22)*'Fiscal Model Import'!Z44,0)</f>
-        <v>2196.1210067534025</v>
+        <v>0</v>
       </c>
       <c r="P25" s="9">
         <f>IF(P$22&gt;0,MIN(MAX(SUM(P$21,P$55,P$59),0),P$22)*'Fiscal Model Import'!AA44,0)</f>
-        <v>4443.0754658203323</v>
+        <v>0</v>
       </c>
       <c r="Q25" s="9">
         <f>IF(Q$22&gt;0,MIN(MAX(SUM(Q$21,Q$55,Q$59),0),Q$22)*'Fiscal Model Import'!AB44,0)</f>
-        <v>6926.930203114187</v>
+        <v>0</v>
       </c>
       <c r="R25" s="9">
         <f>IF(R$22&gt;0,MIN(MAX(SUM(R$21,R$55,R$59),0),R$22)*'Fiscal Model Import'!AC44,0)</f>
-        <v>8805.2290220663272</v>
+        <v>0</v>
       </c>
       <c r="S25" s="9">
         <f>IF(S$22&gt;0,MIN(MAX(SUM(S$21,S$55,S$59),0),S$22)*'Fiscal Model Import'!AD44,0)</f>
-        <v>10056.750389878895</v>
+        <v>0</v>
       </c>
       <c r="T25" s="9">
         <f>IF(T$22&gt;0,MIN(MAX(SUM(T$21,T$55,T$59),0),T$22)*'Fiscal Model Import'!AE44,0)</f>
-        <v>7917.7311205801516</v>
+        <v>0</v>
       </c>
       <c r="U25" s="9">
         <f>IF(U$22&gt;0,MIN(MAX(SUM(U$21,U$55,U$59),0),U$22)*'Fiscal Model Import'!AF44,0)</f>
-        <v>5614.7978453976593</v>
+        <v>0</v>
       </c>
       <c r="V25" s="9">
         <f>IF(V$22&gt;0,MIN(MAX(SUM(V$21,V$55,V$59),0),V$22)*'Fiscal Model Import'!AG44,0)</f>
-        <v>3916.2174239855613</v>
+        <v>0</v>
       </c>
       <c r="W25" s="9">
         <f>IF(W$22&gt;0,MIN(MAX(SUM(W$21,W$55,W$59),0),W$22)*'Fiscal Model Import'!AH44,0)</f>
-        <v>2827.0500105071801</v>
+        <v>0</v>
       </c>
       <c r="X25" s="9">
         <f>IF(X$22&gt;0,MIN(MAX(SUM(X$21,X$55,X$59),0),X$22)*'Fiscal Model Import'!AI44,0)</f>
-        <v>2762.932856225525</v>
+        <v>0</v>
       </c>
       <c r="Y25" s="9">
         <f>IF(Y$22&gt;0,MIN(MAX(SUM(Y$21,Y$55,Y$59),0),Y$22)*'Fiscal Model Import'!AJ44,0)</f>
-        <v>3231.9961934842941</v>
+        <v>0</v>
       </c>
       <c r="Z25" s="9">
         <f>IF(Z$22&gt;0,MIN(MAX(SUM(Z$21,Z$55,Z$59),0),Z$22)*'Fiscal Model Import'!AK44,0)</f>
-        <v>3833.6295666571982</v>
+        <v>0</v>
       </c>
       <c r="AA25" s="9">
         <f>IF(AA$22&gt;0,MIN(MAX(SUM(AA$21,AA$55,AA$59),0),AA$22)*'Fiscal Model Import'!AL44,0)</f>
-        <v>4373.7264267781402</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.25">
@@ -7436,83 +7436,83 @@
       </c>
       <c r="H28" s="9">
         <f t="shared" si="8"/>
-        <v>14734.364442487693</v>
+        <v>0</v>
       </c>
       <c r="I28" s="9">
         <f t="shared" si="8"/>
-        <v>21819.483509096575</v>
+        <v>0</v>
       </c>
       <c r="J28" s="9">
         <f t="shared" si="8"/>
-        <v>25285.369557163212</v>
+        <v>0</v>
       </c>
       <c r="K28" s="9">
         <f>SUM(K25:K27)</f>
-        <v>27040.198003314028</v>
+        <v>0</v>
       </c>
       <c r="L28" s="9">
         <f t="shared" si="8"/>
-        <v>13250.511580417538</v>
+        <v>0</v>
       </c>
       <c r="M28" s="9">
         <f t="shared" si="8"/>
-        <v>6732.8300426464539</v>
+        <v>0</v>
       </c>
       <c r="N28" s="9">
         <f t="shared" si="8"/>
-        <v>3650.5565036424659</v>
+        <v>0</v>
       </c>
       <c r="O28" s="9">
         <f t="shared" si="8"/>
-        <v>2196.1210067534025</v>
+        <v>0</v>
       </c>
       <c r="P28" s="9">
         <f t="shared" si="8"/>
-        <v>4443.0754658203323</v>
+        <v>0</v>
       </c>
       <c r="Q28" s="9">
         <f t="shared" si="8"/>
-        <v>6926.930203114187</v>
+        <v>0</v>
       </c>
       <c r="R28" s="9">
         <f t="shared" si="8"/>
-        <v>8805.2290220663272</v>
+        <v>0</v>
       </c>
       <c r="S28" s="9">
         <f t="shared" si="8"/>
-        <v>10056.750389878895</v>
+        <v>0</v>
       </c>
       <c r="T28" s="9">
         <f t="shared" si="8"/>
-        <v>7917.7311205801516</v>
+        <v>0</v>
       </c>
       <c r="U28" s="9">
         <f t="shared" si="8"/>
-        <v>5614.7978453976593</v>
+        <v>0</v>
       </c>
       <c r="V28" s="9">
         <f t="shared" si="8"/>
-        <v>3916.2174239855613</v>
+        <v>0</v>
       </c>
       <c r="W28" s="9">
         <f t="shared" si="8"/>
-        <v>2827.0500105071801</v>
+        <v>0</v>
       </c>
       <c r="X28" s="9">
         <f t="shared" ref="X28:AA28" si="9">SUM(X25:X27)</f>
-        <v>2762.932856225525</v>
+        <v>0</v>
       </c>
       <c r="Y28" s="9">
         <f t="shared" si="9"/>
-        <v>3231.9961934842941</v>
+        <v>0</v>
       </c>
       <c r="Z28" s="9">
         <f t="shared" si="9"/>
-        <v>3833.6295666571982</v>
+        <v>0</v>
       </c>
       <c r="AA28" s="9">
         <f t="shared" si="9"/>
-        <v>4373.7264267781402</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -7541,83 +7541,83 @@
       </c>
       <c r="H29" s="60">
         <f>IF(H22&gt;0,MIN(H22,MAX(0,SUM(H$21,H$55,H$59)))*'Fiscal Model Import'!S38,0)</f>
-        <v>6182.2508150298008</v>
+        <v>0</v>
       </c>
       <c r="I29" s="60">
         <f>IF(I22&gt;0,MIN(I22,MAX(0,SUM(I$21,I$55,I$59)))*'Fiscal Model Import'!T38,0)</f>
-        <v>9155.0280457747849</v>
+        <v>0</v>
       </c>
       <c r="J29" s="60">
         <f>IF(J22&gt;0,MIN(J22,MAX(0,SUM(J$21,J$55,J$59)))*'Fiscal Model Import'!U38,0)</f>
-        <v>10609.245968040506</v>
+        <v>0</v>
       </c>
       <c r="K29" s="60">
         <f>IF(K22&gt;0,MIN(K22,MAX(0,SUM(K$21,K$55,K$59)))*'Fiscal Model Import'!V38,0)</f>
-        <v>11345.537623768123</v>
+        <v>0</v>
       </c>
       <c r="L29" s="60">
         <f>IF(L22&gt;0,MIN(L22,MAX(0,SUM(L$21,L$55,L$59)))*'Fiscal Model Import'!W38,0)</f>
-        <v>5559.655208566799</v>
+        <v>0</v>
       </c>
       <c r="M29" s="60">
         <f>IF(M22&gt;0,MIN(M22,MAX(0,SUM(M$21,M$55,M$59)))*'Fiscal Model Import'!X38,0)</f>
-        <v>2824.963654257253</v>
+        <v>0</v>
       </c>
       <c r="N29" s="60">
         <f>IF(N22&gt;0,MIN(N22,MAX(0,SUM(N$21,N$55,N$59)))*'Fiscal Model Import'!Y38,0)</f>
-        <v>1531.7020295003351</v>
+        <v>0</v>
       </c>
       <c r="O29" s="60">
         <f>IF(O22&gt;0,MIN(O22,MAX(0,SUM(O$21,O$55,O$59)))*'Fiscal Model Import'!Z38,0)</f>
-        <v>921.44937346296604</v>
+        <v>0</v>
       </c>
       <c r="P29" s="60">
         <f>IF(P22&gt;0,MIN(P22,MAX(0,SUM(P$21,P$55,P$59)))*'Fiscal Model Import'!AA38,0)</f>
-        <v>1864.2274681763629</v>
+        <v>0</v>
       </c>
       <c r="Q29" s="60">
         <f>IF(Q22&gt;0,MIN(Q22,MAX(0,SUM(Q$21,Q$55,Q$59)))*'Fiscal Model Import'!AB38,0)</f>
-        <v>2906.4042810269311</v>
+        <v>0</v>
       </c>
       <c r="R29" s="60">
         <f>IF(R22&gt;0,MIN(R22,MAX(0,SUM(R$21,R$55,R$59)))*'Fiscal Model Import'!AC38,0)</f>
-        <v>3694.5016875802767</v>
+        <v>0</v>
       </c>
       <c r="S29" s="60">
         <f>IF(S22&gt;0,MIN(S22,MAX(0,SUM(S$21,S$55,S$59)))*'Fiscal Model Import'!AD38,0)</f>
-        <v>4219.6155482009344</v>
+        <v>0</v>
       </c>
       <c r="T29" s="60">
         <f>IF(T22&gt;0,MIN(T22,MAX(0,SUM(T$21,T$55,T$59)))*'Fiscal Model Import'!AE38,0)</f>
-        <v>3322.1249456979654</v>
+        <v>0</v>
       </c>
       <c r="U29" s="60">
         <f>IF(U22&gt;0,MIN(U22,MAX(0,SUM(U$21,U$55,U$59)))*'Fiscal Model Import'!AF38,0)</f>
-        <v>2355.8592358311853</v>
+        <v>0</v>
       </c>
       <c r="V29" s="60">
         <f>IF(V22&gt;0,MIN(V22,MAX(0,SUM(V$21,V$55,V$59)))*'Fiscal Model Import'!AG38,0)</f>
-        <v>1643.1681499240115</v>
+        <v>0</v>
       </c>
       <c r="W29" s="60">
         <f>IF(W22&gt;0,MIN(W22,MAX(0,SUM(W$21,W$55,W$59)))*'Fiscal Model Import'!AH38,0)</f>
-        <v>1186.1748295834323</v>
+        <v>0</v>
       </c>
       <c r="X29" s="60">
         <f>IF(X22&gt;0,MIN(X22,MAX(0,SUM(X$21,X$55,X$59)))*'Fiscal Model Import'!AI38,0)</f>
-        <v>1159.2725270876326</v>
+        <v>0</v>
       </c>
       <c r="Y29" s="60">
         <f>IF(Y22&gt;0,MIN(Y22,MAX(0,SUM(Y$21,Y$55,Y$59)))*'Fiscal Model Import'!AJ38,0)</f>
-        <v>1356.0823189444591</v>
+        <v>0</v>
       </c>
       <c r="Z29" s="60">
         <f>IF(Z22&gt;0,MIN(Z22,MAX(0,SUM(Z$21,Z$55,Z$59)))*'Fiscal Model Import'!AK38,0)</f>
-        <v>1608.5159020939291</v>
+        <v>0</v>
       </c>
       <c r="AA29" s="60">
         <f>IF(AA22&gt;0,MIN(AA22,MAX(0,SUM(AA$21,AA$55,AA$59)))*'Fiscal Model Import'!AL38,0)</f>
-        <v>1835.1299692775412</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -7751,83 +7751,83 @@
       </c>
       <c r="H31" s="60">
         <f>IF(H22&gt;0,MIN(H22,MAX(SUM(H$21,H$55,H$59),0))*'Fiscal Model Import'!S40,0)</f>
-        <v>4327.5755705208603</v>
+        <v>0</v>
       </c>
       <c r="I31" s="60">
         <f>IF(I22&gt;0,MIN(I22,MAX(SUM(I$21,I$55,I$59),0))*'Fiscal Model Import'!T40,0)</f>
-        <v>6408.5196320423493</v>
+        <v>0</v>
       </c>
       <c r="J31" s="60">
         <f>IF(J22&gt;0,MIN(J22,MAX(SUM(J$21,J$55,J$59),0))*'Fiscal Model Import'!U40,0)</f>
-        <v>7426.4721776283541</v>
+        <v>0</v>
       </c>
       <c r="K31" s="60">
         <f>IF(K22&gt;0,MIN(K22,MAX(SUM(K$21,K$55,K$59),0))*'Fiscal Model Import'!V40,0)</f>
-        <v>7941.8763366376852</v>
+        <v>0</v>
       </c>
       <c r="L31" s="60">
         <f>IF(L22&gt;0,MIN(L22,MAX(SUM(L$21,L$55,L$59),0))*'Fiscal Model Import'!W40,0)</f>
-        <v>3891.7586459967592</v>
+        <v>0</v>
       </c>
       <c r="M31" s="60">
         <f>IF(M22&gt;0,MIN(M22,MAX(SUM(M$21,M$55,M$59),0))*'Fiscal Model Import'!X40,0)</f>
-        <v>1977.474557980077</v>
+        <v>0</v>
       </c>
       <c r="N31" s="60">
         <f>IF(N22&gt;0,MIN(N22,MAX(SUM(N$21,N$55,N$59),0))*'Fiscal Model Import'!Y40,0)</f>
-        <v>1072.1914206502345</v>
+        <v>0</v>
       </c>
       <c r="O31" s="60">
         <f>IF(O22&gt;0,MIN(O22,MAX(SUM(O$21,O$55,O$59),0))*'Fiscal Model Import'!Z40,0)</f>
-        <v>645.01456142407619</v>
+        <v>0</v>
       </c>
       <c r="P31" s="60">
         <f>IF(P22&gt;0,MIN(P22,MAX(SUM(P$21,P$55,P$59),0))*'Fiscal Model Import'!AA40,0)</f>
-        <v>1304.959227723454</v>
+        <v>0</v>
       </c>
       <c r="Q31" s="60">
         <f>IF(Q22&gt;0,MIN(Q22,MAX(SUM(Q$21,Q$55,Q$59),0))*'Fiscal Model Import'!AB40,0)</f>
-        <v>2034.4829967188516</v>
+        <v>0</v>
       </c>
       <c r="R31" s="60">
         <f>IF(R22&gt;0,MIN(R22,MAX(SUM(R$21,R$55,R$59),0))*'Fiscal Model Import'!AC40,0)</f>
-        <v>2586.1511813061934</v>
+        <v>0</v>
       </c>
       <c r="S31" s="60">
         <f>IF(S22&gt;0,MIN(S22,MAX(SUM(S$21,S$55,S$59),0))*'Fiscal Model Import'!AD40,0)</f>
-        <v>2953.7308837406536</v>
+        <v>0</v>
       </c>
       <c r="T31" s="60">
         <f>IF(T22&gt;0,MIN(T22,MAX(SUM(T$21,T$55,T$59),0))*'Fiscal Model Import'!AE40,0)</f>
-        <v>2325.4874619885754</v>
+        <v>0</v>
       </c>
       <c r="U31" s="60">
         <f>IF(U22&gt;0,MIN(U22,MAX(SUM(U$21,U$55,U$59),0))*'Fiscal Model Import'!AF40,0)</f>
-        <v>1649.1014650818295</v>
+        <v>0</v>
       </c>
       <c r="V31" s="60">
         <f>IF(V22&gt;0,MIN(V22,MAX(SUM(V$21,V$55,V$59),0))*'Fiscal Model Import'!AG40,0)</f>
-        <v>1150.217704946808</v>
+        <v>0</v>
       </c>
       <c r="W31" s="60">
         <f>IF(W22&gt;0,MIN(W22,MAX(SUM(W$21,W$55,W$59),0))*'Fiscal Model Import'!AH40,0)</f>
-        <v>830.32238070840242</v>
+        <v>0</v>
       </c>
       <c r="X31" s="60">
         <f>IF(X22&gt;0,MIN(X22,MAX(SUM(X$21,X$55,X$59),0))*'Fiscal Model Import'!AI40,0)</f>
-        <v>811.49076896134284</v>
+        <v>0</v>
       </c>
       <c r="Y31" s="60">
         <f>IF(Y22&gt;0,MIN(Y22,MAX(SUM(Y$21,Y$55,Y$59),0))*'Fiscal Model Import'!AJ40,0)</f>
-        <v>949.25762326112124</v>
+        <v>0</v>
       </c>
       <c r="Z31" s="60">
         <f>IF(Z22&gt;0,MIN(Z22,MAX(SUM(Z$21,Z$55,Z$59),0))*'Fiscal Model Import'!AK40,0)</f>
-        <v>1125.9611314657502</v>
+        <v>0</v>
       </c>
       <c r="AA31" s="60">
         <f>IF(AA22&gt;0,MIN(AA22,MAX(SUM(AA$21,AA$55,AA$59),0))*'Fiscal Model Import'!AL40,0)</f>
-        <v>1284.5909784942787</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -7856,83 +7856,83 @@
       </c>
       <c r="H32" s="60">
         <f>IF(H22&gt;0,MIN(H22,MAX(0,SUM(H21,H55,H59)))*'Fiscal Model Import'!S36,0)</f>
-        <v>5821.6195174863951</v>
+        <v>0</v>
       </c>
       <c r="I32" s="60">
         <f>IF(I22&gt;0,MIN(I22,MAX(0,SUM(I21,I55,I59)))*'Fiscal Model Import'!T36,0)</f>
-        <v>8620.9847431045891</v>
+        <v>0</v>
       </c>
       <c r="J32" s="60">
         <f>IF(J22&gt;0,MIN(J22,MAX(0,SUM(J21,J55,J59)))*'Fiscal Model Import'!U36,0)</f>
-        <v>9990.3732865714774</v>
+        <v>0</v>
       </c>
       <c r="K32" s="60">
         <f>IF(K22&gt;0,MIN(K22,MAX(0,SUM(K21,K55,K59)))*'Fiscal Model Import'!V36,0)</f>
-        <v>10683.714595714982</v>
+        <v>0</v>
       </c>
       <c r="L32" s="60">
         <f>IF(L22&gt;0,MIN(L22,MAX(0,SUM(L21,L55,L59)))*'Fiscal Model Import'!W36,0)</f>
-        <v>5235.341988067069</v>
+        <v>0</v>
       </c>
       <c r="M32" s="60">
         <f>IF(M22&gt;0,MIN(M22,MAX(0,SUM(M21,M55,M59)))*'Fiscal Model Import'!X36,0)</f>
-        <v>2660.1741077589131</v>
+        <v>0</v>
       </c>
       <c r="N32" s="60">
         <f>IF(N22&gt;0,MIN(N22,MAX(0,SUM(N21,N55,N59)))*'Fiscal Model Import'!Y36,0)</f>
-        <v>1442.3527444461488</v>
+        <v>0</v>
       </c>
       <c r="O32" s="60">
         <f>IF(O22&gt;0,MIN(O22,MAX(0,SUM(O21,O55,O59)))*'Fiscal Model Import'!Z36,0)</f>
-        <v>867.69816001095967</v>
+        <v>0</v>
       </c>
       <c r="P32" s="60">
         <f>IF(P22&gt;0,MIN(P22,MAX(0,SUM(P21,P55,P59)))*'Fiscal Model Import'!AA36,0)</f>
-        <v>1755.480865866075</v>
+        <v>0</v>
       </c>
       <c r="Q32" s="60">
         <f>IF(Q22&gt;0,MIN(Q22,MAX(0,SUM(Q21,Q55,Q59)))*'Fiscal Model Import'!AB36,0)</f>
-        <v>2736.8640313003602</v>
+        <v>0</v>
       </c>
       <c r="R32" s="60">
         <f>IF(R22&gt;0,MIN(R22,MAX(0,SUM(R21,R55,R59)))*'Fiscal Model Import'!AC36,0)</f>
-        <v>3478.9890891380937</v>
+        <v>0</v>
       </c>
       <c r="S32" s="60">
         <f>IF(S22&gt;0,MIN(S22,MAX(0,SUM(S21,S55,S59)))*'Fiscal Model Import'!AD36,0)</f>
-        <v>3973.4713078892128</v>
+        <v>0</v>
       </c>
       <c r="T32" s="60">
         <f>IF(T22&gt;0,MIN(T22,MAX(0,SUM(T21,T55,T59)))*'Fiscal Model Import'!AE36,0)</f>
-        <v>3128.3343238655839</v>
+        <v>0</v>
       </c>
       <c r="U32" s="60">
         <f>IF(U22&gt;0,MIN(U22,MAX(0,SUM(U21,U55,U59)))*'Fiscal Model Import'!AF36,0)</f>
-        <v>2218.4341137410329</v>
+        <v>0</v>
       </c>
       <c r="V32" s="60">
         <f>IF(V22&gt;0,MIN(V22,MAX(0,SUM(V21,V55,V59)))*'Fiscal Model Import'!AG36,0)</f>
-        <v>1547.3166745117774</v>
+        <v>0</v>
       </c>
       <c r="W32" s="60">
         <f>IF(W22&gt;0,MIN(W22,MAX(0,SUM(W21,W55,W59)))*'Fiscal Model Import'!AH36,0)</f>
-        <v>1116.981297857732</v>
+        <v>0</v>
       </c>
       <c r="X32" s="60">
         <f>IF(X22&gt;0,MIN(X22,MAX(0,SUM(X21,X55,X59)))*'Fiscal Model Import'!AI36,0)</f>
-        <v>1091.6482963408541</v>
+        <v>0</v>
       </c>
       <c r="Y32" s="60">
         <f>IF(Y22&gt;0,MIN(Y22,MAX(0,SUM(Y21,Y55,Y59)))*'Fiscal Model Import'!AJ36,0)</f>
-        <v>1276.9775170060323</v>
+        <v>0</v>
       </c>
       <c r="Z32" s="60">
         <f>IF(Z22&gt;0,MIN(Z22,MAX(0,SUM(Z21,Z55,Z59)))*'Fiscal Model Import'!AK36,0)</f>
-        <v>1514.6858078051166</v>
+        <v>0</v>
       </c>
       <c r="AA32" s="60">
         <f>IF(AA22&gt;0,MIN(AA22,MAX(0,SUM(AA21,AA55,AA59)))*'Fiscal Model Import'!AL36,0)</f>
-        <v>1728.0807210696846</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.25">
@@ -7961,83 +7961,83 @@
       </c>
       <c r="H33" s="60">
         <f t="shared" si="10"/>
-        <v>14734.364442487693</v>
+        <v>0</v>
       </c>
       <c r="I33" s="60">
         <f t="shared" si="10"/>
-        <v>21819.483509096575</v>
+        <v>0</v>
       </c>
       <c r="J33" s="60">
         <f t="shared" si="10"/>
-        <v>25285.369557163212</v>
+        <v>0</v>
       </c>
       <c r="K33" s="60">
         <f t="shared" si="10"/>
-        <v>27040.198003314028</v>
+        <v>0</v>
       </c>
       <c r="L33" s="60">
         <f>L25</f>
-        <v>13250.511580417538</v>
+        <v>0</v>
       </c>
       <c r="M33" s="60">
         <f t="shared" si="10"/>
-        <v>6732.8300426464539</v>
+        <v>0</v>
       </c>
       <c r="N33" s="60">
         <f t="shared" si="10"/>
-        <v>3650.5565036424659</v>
+        <v>0</v>
       </c>
       <c r="O33" s="60">
         <f t="shared" si="10"/>
-        <v>2196.1210067534025</v>
+        <v>0</v>
       </c>
       <c r="P33" s="60">
         <f t="shared" si="10"/>
-        <v>4443.0754658203323</v>
+        <v>0</v>
       </c>
       <c r="Q33" s="60">
         <f t="shared" si="10"/>
-        <v>6926.930203114187</v>
+        <v>0</v>
       </c>
       <c r="R33" s="60">
         <f t="shared" si="10"/>
-        <v>8805.2290220663272</v>
+        <v>0</v>
       </c>
       <c r="S33" s="60">
         <f t="shared" si="10"/>
-        <v>10056.750389878895</v>
+        <v>0</v>
       </c>
       <c r="T33" s="60">
         <f t="shared" si="10"/>
-        <v>7917.7311205801516</v>
+        <v>0</v>
       </c>
       <c r="U33" s="60">
         <f t="shared" si="10"/>
-        <v>5614.7978453976593</v>
+        <v>0</v>
       </c>
       <c r="V33" s="60">
         <f t="shared" si="10"/>
-        <v>3916.2174239855613</v>
+        <v>0</v>
       </c>
       <c r="W33" s="60">
         <f t="shared" si="10"/>
-        <v>2827.0500105071801</v>
+        <v>0</v>
       </c>
       <c r="X33" s="60">
         <f t="shared" ref="X33:AA33" si="11">X25</f>
-        <v>2762.932856225525</v>
+        <v>0</v>
       </c>
       <c r="Y33" s="60">
         <f t="shared" si="11"/>
-        <v>3231.9961934842941</v>
+        <v>0</v>
       </c>
       <c r="Z33" s="60">
         <f t="shared" si="11"/>
-        <v>3833.6295666571982</v>
+        <v>0</v>
       </c>
       <c r="AA33" s="60">
         <f t="shared" si="11"/>
-        <v>4373.7264267781402</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.25">
@@ -8124,83 +8124,83 @@
       </c>
       <c r="H36" s="9">
         <f t="shared" si="12"/>
-        <v>14734.364442487693</v>
+        <v>0</v>
       </c>
       <c r="I36" s="9">
         <f t="shared" si="12"/>
-        <v>21819.483509096575</v>
+        <v>0</v>
       </c>
       <c r="J36" s="9">
         <f t="shared" si="12"/>
-        <v>25285.369557163212</v>
+        <v>0</v>
       </c>
       <c r="K36" s="9">
         <f t="shared" si="12"/>
-        <v>27040.198003314028</v>
+        <v>0</v>
       </c>
       <c r="L36" s="9">
         <f>SUM(L33:L35)</f>
-        <v>13250.511580417538</v>
+        <v>0</v>
       </c>
       <c r="M36" s="9">
         <f t="shared" si="12"/>
-        <v>6732.8300426464539</v>
+        <v>0</v>
       </c>
       <c r="N36" s="9">
         <f t="shared" si="12"/>
-        <v>3650.5565036424659</v>
+        <v>0</v>
       </c>
       <c r="O36" s="9">
         <f t="shared" si="12"/>
-        <v>2196.1210067534025</v>
+        <v>0</v>
       </c>
       <c r="P36" s="9">
         <f t="shared" si="12"/>
-        <v>4443.0754658203323</v>
+        <v>0</v>
       </c>
       <c r="Q36" s="9">
         <f t="shared" si="12"/>
-        <v>6926.930203114187</v>
+        <v>0</v>
       </c>
       <c r="R36" s="9">
         <f t="shared" si="12"/>
-        <v>8805.2290220663272</v>
+        <v>0</v>
       </c>
       <c r="S36" s="9">
         <f t="shared" si="12"/>
-        <v>10056.750389878895</v>
+        <v>0</v>
       </c>
       <c r="T36" s="9">
         <f t="shared" si="12"/>
-        <v>7917.7311205801516</v>
+        <v>0</v>
       </c>
       <c r="U36" s="9">
         <f t="shared" si="12"/>
-        <v>5614.7978453976593</v>
+        <v>0</v>
       </c>
       <c r="V36" s="9">
         <f t="shared" si="12"/>
-        <v>3916.2174239855613</v>
+        <v>0</v>
       </c>
       <c r="W36" s="9">
         <f t="shared" si="12"/>
-        <v>2827.0500105071801</v>
+        <v>0</v>
       </c>
       <c r="X36" s="9">
         <f t="shared" ref="X36:AA36" si="13">SUM(X33:X35)</f>
-        <v>2762.932856225525</v>
+        <v>0</v>
       </c>
       <c r="Y36" s="9">
         <f t="shared" si="13"/>
-        <v>3231.9961934842941</v>
+        <v>0</v>
       </c>
       <c r="Z36" s="9">
         <f t="shared" si="13"/>
-        <v>3833.6295666571982</v>
+        <v>0</v>
       </c>
       <c r="AA36" s="9">
         <f t="shared" si="13"/>
-        <v>4373.7264267781402</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -8229,83 +8229,83 @@
       </c>
       <c r="H37" s="60">
         <f t="shared" si="14"/>
-        <v>6182.2508150298008</v>
+        <v>0</v>
       </c>
       <c r="I37" s="60">
         <f t="shared" si="14"/>
-        <v>15337.278860804585</v>
+        <v>0</v>
       </c>
       <c r="J37" s="60">
         <f t="shared" si="14"/>
-        <v>25946.524828845089</v>
+        <v>0</v>
       </c>
       <c r="K37" s="60">
         <f t="shared" si="14"/>
-        <v>37292.062452613216</v>
+        <v>0</v>
       </c>
       <c r="L37" s="60">
         <f>IF(AND(L$22&gt;0,L$21+L$55+L$59&gt;0),K37+L29-L56,L$22*K46)</f>
-        <v>42851.717661180017</v>
+        <v>0</v>
       </c>
       <c r="M37" s="60">
         <f t="shared" si="14"/>
-        <v>45676.681315437272</v>
+        <v>0</v>
       </c>
       <c r="N37" s="60">
         <f t="shared" si="14"/>
-        <v>47208.383344937611</v>
+        <v>0</v>
       </c>
       <c r="O37" s="60">
         <f t="shared" si="14"/>
-        <v>48129.832718400576</v>
+        <v>0</v>
       </c>
       <c r="P37" s="60">
         <f>IF(AND(P$22&gt;0,P$21+P$55+P$59&gt;0),O37+P29-P56,P$22*O46)</f>
-        <v>43811.80937154714</v>
+        <v>0</v>
       </c>
       <c r="Q37" s="60">
         <f t="shared" si="14"/>
-        <v>37563.185606799285</v>
+        <v>0</v>
       </c>
       <c r="R37" s="60">
         <f t="shared" si="14"/>
-        <v>30648.441326339052</v>
+        <v>0</v>
       </c>
       <c r="S37" s="60">
         <f t="shared" si="14"/>
-        <v>23522.519250771864</v>
+        <v>0</v>
       </c>
       <c r="T37" s="60">
         <f t="shared" si="14"/>
-        <v>21284.988987903031</v>
+        <v>0</v>
       </c>
       <c r="U37" s="60">
         <f t="shared" si="14"/>
-        <v>20815.884569476966</v>
+        <v>0</v>
       </c>
       <c r="V37" s="60">
         <f t="shared" si="14"/>
-        <v>20927.350689900642</v>
+        <v>0</v>
       </c>
       <c r="W37" s="60">
         <f t="shared" si="14"/>
-        <v>21192.076146021111</v>
+        <v>0</v>
       </c>
       <c r="X37" s="60">
         <f t="shared" si="14"/>
-        <v>20487.12120493238</v>
+        <v>0</v>
       </c>
       <c r="Y37" s="60">
         <f t="shared" si="14"/>
-        <v>18936.799242849909</v>
+        <v>0</v>
       </c>
       <c r="Z37" s="60">
         <f t="shared" si="14"/>
-        <v>16850.813457363562</v>
+        <v>0</v>
       </c>
       <c r="AA37" s="60">
         <f t="shared" si="14"/>
-        <v>14466.32787844017</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -8439,83 +8439,83 @@
       </c>
       <c r="H39" s="60">
         <f t="shared" si="16"/>
-        <v>4327.5755705208603</v>
+        <v>0</v>
       </c>
       <c r="I39" s="60">
         <f t="shared" si="16"/>
-        <v>10736.09520256321</v>
+        <v>0</v>
       </c>
       <c r="J39" s="60">
         <f t="shared" si="16"/>
-        <v>18162.567380191565</v>
+        <v>0</v>
       </c>
       <c r="K39" s="60">
         <f t="shared" si="16"/>
-        <v>26104.44371682925</v>
+        <v>0</v>
       </c>
       <c r="L39" s="60">
         <f t="shared" si="16"/>
-        <v>29996.20236282601</v>
+        <v>0</v>
       </c>
       <c r="M39" s="60">
         <f t="shared" si="16"/>
-        <v>31973.676920806087</v>
+        <v>0</v>
       </c>
       <c r="N39" s="60">
         <f t="shared" si="16"/>
-        <v>33045.86834145632</v>
+        <v>0</v>
       </c>
       <c r="O39" s="60">
         <f t="shared" si="16"/>
-        <v>33690.882902880396</v>
+        <v>0</v>
       </c>
       <c r="P39" s="60">
         <f t="shared" si="16"/>
-        <v>34995.842130603851</v>
+        <v>0</v>
       </c>
       <c r="Q39" s="60">
         <f t="shared" si="16"/>
-        <v>37030.3251273227</v>
+        <v>0</v>
       </c>
       <c r="R39" s="60">
         <f t="shared" si="16"/>
-        <v>39616.476308628895</v>
+        <v>0</v>
       </c>
       <c r="S39" s="60">
         <f t="shared" si="16"/>
-        <v>42570.207192369548</v>
+        <v>0</v>
       </c>
       <c r="T39" s="60">
         <f t="shared" si="16"/>
-        <v>44895.694654358122</v>
+        <v>0</v>
       </c>
       <c r="U39" s="60">
         <f t="shared" si="16"/>
-        <v>46544.796119439954</v>
+        <v>0</v>
       </c>
       <c r="V39" s="60">
         <f t="shared" si="16"/>
-        <v>47695.013824386762</v>
+        <v>0</v>
       </c>
       <c r="W39" s="60">
         <f t="shared" si="16"/>
-        <v>48525.336205095162</v>
+        <v>0</v>
       </c>
       <c r="X39" s="60">
         <f t="shared" si="16"/>
-        <v>49336.826974056501</v>
+        <v>0</v>
       </c>
       <c r="Y39" s="60">
         <f t="shared" si="16"/>
-        <v>50286.084597317626</v>
+        <v>0</v>
       </c>
       <c r="Z39" s="60">
         <f t="shared" si="16"/>
-        <v>51412.045728783378</v>
+        <v>0</v>
       </c>
       <c r="AA39" s="60">
         <f t="shared" si="16"/>
-        <v>52696.636707277656</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:27" x14ac:dyDescent="0.25">
@@ -8544,83 +8544,83 @@
       </c>
       <c r="H40" s="60">
         <f t="shared" si="17"/>
-        <v>10509.826385550661</v>
+        <v>0</v>
       </c>
       <c r="I40" s="60">
         <f t="shared" si="17"/>
-        <v>26073.374063367795</v>
+        <v>0</v>
       </c>
       <c r="J40" s="60">
         <f t="shared" si="17"/>
-        <v>44109.092209036651</v>
+        <v>0</v>
       </c>
       <c r="K40" s="60">
         <f t="shared" si="17"/>
-        <v>63396.506169442466</v>
+        <v>0</v>
       </c>
       <c r="L40" s="60">
         <f t="shared" si="17"/>
-        <v>72847.920024006031</v>
+        <v>0</v>
       </c>
       <c r="M40" s="60">
         <f t="shared" si="17"/>
-        <v>77650.358236243366</v>
+        <v>0</v>
       </c>
       <c r="N40" s="60">
         <f t="shared" si="17"/>
-        <v>80254.251686393924</v>
+        <v>0</v>
       </c>
       <c r="O40" s="60">
         <f t="shared" si="17"/>
-        <v>81820.715621280979</v>
+        <v>0</v>
       </c>
       <c r="P40" s="60">
         <f t="shared" si="17"/>
-        <v>78807.651502150984</v>
+        <v>0</v>
       </c>
       <c r="Q40" s="60">
         <f t="shared" si="17"/>
-        <v>74593.510734121985</v>
+        <v>0</v>
       </c>
       <c r="R40" s="60">
         <f t="shared" si="17"/>
-        <v>70264.917634967947</v>
+        <v>0</v>
       </c>
       <c r="S40" s="60">
         <f t="shared" si="17"/>
-        <v>66092.726443141408</v>
+        <v>0</v>
       </c>
       <c r="T40" s="60">
         <f t="shared" si="17"/>
-        <v>66180.683642261152</v>
+        <v>0</v>
       </c>
       <c r="U40" s="60">
         <f t="shared" si="17"/>
-        <v>67360.680688916924</v>
+        <v>0</v>
       </c>
       <c r="V40" s="60">
         <f t="shared" si="17"/>
-        <v>68622.364514287401</v>
+        <v>0</v>
       </c>
       <c r="W40" s="60">
         <f t="shared" si="17"/>
-        <v>69717.412351116276</v>
+        <v>0</v>
       </c>
       <c r="X40" s="60">
         <f>SUM(X37:X39)</f>
-        <v>69823.948178988881</v>
+        <v>0</v>
       </c>
       <c r="Y40" s="60">
         <f t="shared" ref="Y40:AA40" si="18">SUM(Y37:Y39)</f>
-        <v>69222.883840167531</v>
+        <v>0</v>
       </c>
       <c r="Z40" s="60">
         <f t="shared" si="18"/>
-        <v>68262.859186146932</v>
+        <v>0</v>
       </c>
       <c r="AA40" s="60">
         <f t="shared" si="18"/>
-        <v>67162.964585717826</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -8649,83 +8649,83 @@
       </c>
       <c r="H41" s="60">
         <f t="shared" si="19"/>
-        <v>5821.6195174863951</v>
+        <v>0</v>
       </c>
       <c r="I41" s="60">
         <f t="shared" si="19"/>
-        <v>14442.604260590984</v>
+        <v>0</v>
       </c>
       <c r="J41" s="60">
         <f t="shared" si="19"/>
-        <v>24432.97754716246</v>
+        <v>0</v>
       </c>
       <c r="K41" s="60">
         <f t="shared" si="19"/>
-        <v>35116.692142877444</v>
+        <v>0</v>
       </c>
       <c r="L41" s="60">
         <f t="shared" si="19"/>
-        <v>40352.034130944514</v>
+        <v>0</v>
       </c>
       <c r="M41" s="60">
         <f t="shared" si="19"/>
-        <v>43012.208238703424</v>
+        <v>0</v>
       </c>
       <c r="N41" s="60">
         <f t="shared" si="19"/>
-        <v>44454.560983149575</v>
+        <v>0</v>
       </c>
       <c r="O41" s="60">
         <f t="shared" si="19"/>
-        <v>45322.259143160532</v>
+        <v>0</v>
       </c>
       <c r="P41" s="60">
         <f t="shared" si="19"/>
-        <v>47077.740009026609</v>
+        <v>0</v>
       </c>
       <c r="Q41" s="60">
         <f t="shared" si="19"/>
-        <v>49814.604040326973</v>
+        <v>0</v>
       </c>
       <c r="R41" s="60">
         <f t="shared" si="19"/>
-        <v>53293.593129465065</v>
+        <v>0</v>
       </c>
       <c r="S41" s="60">
         <f t="shared" si="19"/>
-        <v>57267.064437354275</v>
+        <v>0</v>
       </c>
       <c r="T41" s="60">
         <f t="shared" si="19"/>
-        <v>60395.398761219862</v>
+        <v>0</v>
       </c>
       <c r="U41" s="60">
         <f t="shared" si="19"/>
-        <v>62613.832874960892</v>
+        <v>0</v>
       </c>
       <c r="V41" s="60">
         <f t="shared" si="19"/>
-        <v>64161.14954947267</v>
+        <v>0</v>
       </c>
       <c r="W41" s="60">
         <f t="shared" si="19"/>
-        <v>65278.130847330402</v>
+        <v>0</v>
       </c>
       <c r="X41" s="60">
         <f t="shared" si="19"/>
-        <v>66369.779143671258</v>
+        <v>0</v>
       </c>
       <c r="Y41" s="60">
         <f t="shared" si="19"/>
-        <v>67646.756660677289</v>
+        <v>0</v>
       </c>
       <c r="Z41" s="60">
         <f t="shared" si="19"/>
-        <v>69161.442468482404</v>
+        <v>0</v>
       </c>
       <c r="AA41" s="60">
         <f t="shared" si="19"/>
-        <v>70889.523189552085</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:27" x14ac:dyDescent="0.25">
@@ -8754,83 +8754,83 @@
       </c>
       <c r="H42" s="58">
         <f t="shared" si="20"/>
-        <v>0.47429519071310117</v>
+        <v>0</v>
       </c>
       <c r="I42" s="58">
         <f t="shared" si="20"/>
-        <v>0.35003323738152048</v>
+        <v>0</v>
       </c>
       <c r="J42" s="58">
         <f t="shared" si="20"/>
-        <v>0.26948800630395359</v>
+        <v>0</v>
       </c>
       <c r="K42" s="58">
         <f t="shared" si="20"/>
-        <v>0.21536811266607667</v>
+        <v>0</v>
       </c>
       <c r="L42" s="58">
         <f t="shared" si="20"/>
-        <v>0.1047881595639816</v>
+        <v>0</v>
       </c>
       <c r="M42" s="58">
         <f t="shared" si="20"/>
-        <v>5.2849869200074694E-2</v>
+        <v>0</v>
       </c>
       <c r="N42" s="58">
         <f t="shared" si="20"/>
-        <v>2.8440124995605387E-2</v>
+        <v>0</v>
       </c>
       <c r="O42" s="58">
         <f t="shared" si="20"/>
-        <v>1.6979560539362455E-2</v>
+        <v>0</v>
       </c>
       <c r="P42" s="58">
         <f t="shared" si="20"/>
-        <v>3.4091365983799256E-2</v>
+        <v>0</v>
       </c>
       <c r="Q42" s="58">
         <f t="shared" si="20"/>
-        <v>5.2742435991075816E-2</v>
+        <v>0</v>
       </c>
       <c r="R42" s="58">
         <f t="shared" si="20"/>
-        <v>6.6522969479927238E-2</v>
+        <v>0</v>
       </c>
       <c r="S42" s="58">
         <f t="shared" si="20"/>
-        <v>7.5378587198557626E-2</v>
+        <v>0</v>
       </c>
       <c r="T42" s="58">
         <f t="shared" si="20"/>
-        <v>5.8870597190432514E-2</v>
+        <v>0</v>
       </c>
       <c r="U42" s="58">
         <f t="shared" si="20"/>
-        <v>4.1410327901507116E-2</v>
+        <v>0</v>
       </c>
       <c r="V42" s="58">
         <f t="shared" si="20"/>
-        <v>2.8648318335114116E-2</v>
+        <v>0</v>
       </c>
       <c r="W42" s="58">
         <f t="shared" si="20"/>
-        <v>2.051223928301122E-2</v>
+        <v>0</v>
       </c>
       <c r="X42" s="58">
         <f t="shared" ref="X42:AA42" si="21">IF(X$22=0,0,X33/X$22)</f>
-        <v>1.9883414387397234E-2</v>
+        <v>0</v>
       </c>
       <c r="Y42" s="58">
         <f t="shared" si="21"/>
-        <v>2.3068939590875699E-2</v>
+        <v>0</v>
       </c>
       <c r="Z42" s="58">
         <f t="shared" si="21"/>
-        <v>2.7139216421424531E-2</v>
+        <v>0</v>
       </c>
       <c r="AA42" s="58">
         <f t="shared" si="21"/>
-        <v>3.0708717852835025E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:27" x14ac:dyDescent="0.25">
@@ -8946,83 +8946,83 @@
       </c>
       <c r="H46" s="58">
         <f t="shared" si="22"/>
-        <v>0.19900497512437809</v>
+        <v>0</v>
       </c>
       <c r="I46" s="58">
         <f t="shared" si="22"/>
-        <v>0.24604420036030769</v>
+        <v>0</v>
       </c>
       <c r="J46" s="58">
         <f t="shared" si="22"/>
-        <v>0.27653450865465473</v>
+        <v>0</v>
       </c>
       <c r="K46" s="58">
         <f t="shared" si="22"/>
-        <v>0.29702153463744729</v>
+        <v>0</v>
       </c>
       <c r="L46" s="58">
         <f t="shared" si="22"/>
-        <v>0.33888145379281454</v>
+        <v>0</v>
       </c>
       <c r="M46" s="58">
         <f t="shared" si="22"/>
-        <v>0.35854263626495597</v>
+        <v>0</v>
       </c>
       <c r="N46" s="58">
         <f t="shared" si="22"/>
-        <v>0.36778291798273616</v>
+        <v>0</v>
       </c>
       <c r="O46" s="58">
         <f t="shared" si="22"/>
-        <v>0.37212130200402688</v>
+        <v>0</v>
       </c>
       <c r="P46" s="58">
         <f t="shared" si="22"/>
-        <v>0.33616454169816651</v>
+        <v>0</v>
       </c>
       <c r="Q46" s="58">
         <f t="shared" si="22"/>
-        <v>0.2860103760821528</v>
+        <v>0</v>
       </c>
       <c r="R46" s="58">
         <f t="shared" si="22"/>
-        <v>0.23154710931992786</v>
+        <v>0</v>
       </c>
       <c r="S46" s="58">
         <f t="shared" si="22"/>
-        <v>0.17630886715240521</v>
+        <v>0</v>
       </c>
       <c r="T46" s="58">
         <f t="shared" si="22"/>
-        <v>0.15825998557245985</v>
+        <v>0</v>
       </c>
       <c r="U46" s="58">
         <f t="shared" si="22"/>
-        <v>0.15352157447458631</v>
+        <v>0</v>
       </c>
       <c r="V46" s="58">
         <f t="shared" si="22"/>
-        <v>0.15308991804257241</v>
+        <v>0</v>
       </c>
       <c r="W46" s="58">
         <f t="shared" si="22"/>
-        <v>0.15376344075816104</v>
+        <v>0</v>
       </c>
       <c r="X46" s="58">
         <f t="shared" ref="X46:AA46" si="23">IF(X$22=0,0,X37/X$22)</f>
-        <v>0.14743533112092866</v>
+        <v>0</v>
       </c>
       <c r="Y46" s="58">
         <f t="shared" si="23"/>
-        <v>0.13516472533554924</v>
+        <v>0</v>
       </c>
       <c r="Z46" s="58">
         <f t="shared" si="23"/>
-        <v>0.11929109616483086</v>
+        <v>0</v>
       </c>
       <c r="AA46" s="58">
         <f t="shared" si="23"/>
-        <v>0.10157068317436287</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:27" x14ac:dyDescent="0.25">
@@ -9156,83 +9156,83 @@
       </c>
       <c r="H48" s="58">
         <f t="shared" si="26"/>
-        <v>0.13930348258706465</v>
+        <v>0</v>
       </c>
       <c r="I48" s="58">
         <f t="shared" si="26"/>
-        <v>0.17223094025221539</v>
+        <v>0</v>
       </c>
       <c r="J48" s="58">
         <f t="shared" si="26"/>
-        <v>0.19357415605825834</v>
+        <v>0</v>
       </c>
       <c r="K48" s="58">
         <f t="shared" si="26"/>
-        <v>0.20791507424621311</v>
+        <v>0</v>
       </c>
       <c r="L48" s="58">
         <f t="shared" si="26"/>
-        <v>0.23721701765497016</v>
+        <v>0</v>
       </c>
       <c r="M48" s="58">
         <f t="shared" si="26"/>
-        <v>0.25097984538546914</v>
+        <v>0</v>
       </c>
       <c r="N48" s="58">
         <f t="shared" si="26"/>
-        <v>0.25744804258791526</v>
+        <v>0</v>
       </c>
       <c r="O48" s="58">
         <f t="shared" si="26"/>
-        <v>0.26048491140281876</v>
+        <v>0</v>
       </c>
       <c r="P48" s="58">
         <f t="shared" si="26"/>
-        <v>0.26852032362799427</v>
+        <v>0</v>
       </c>
       <c r="Q48" s="58">
         <f t="shared" si="26"/>
-        <v>0.28195311566420705</v>
+        <v>0</v>
       </c>
       <c r="R48" s="58">
         <f t="shared" si="26"/>
-        <v>0.29930006792290437</v>
+        <v>0</v>
       </c>
       <c r="S48" s="58">
         <f t="shared" si="26"/>
-        <v>0.31907743063207666</v>
+        <v>0</v>
       </c>
       <c r="T48" s="58">
         <f t="shared" si="26"/>
-        <v>0.33381234034475643</v>
+        <v>0</v>
       </c>
       <c r="U48" s="58">
         <f t="shared" si="26"/>
-        <v>0.34327776751476208</v>
+        <v>0</v>
       </c>
       <c r="V48" s="58">
         <f t="shared" si="26"/>
-        <v>0.34890349311814367</v>
+        <v>0</v>
       </c>
       <c r="W48" s="58">
         <f t="shared" si="26"/>
-        <v>0.35208549683523599</v>
+        <v>0</v>
       </c>
       <c r="X48" s="58">
         <f t="shared" ref="X48:AA48" si="27">IF(X$22=0,0,X39/X$22)</f>
-        <v>0.35505190546853083</v>
+        <v>0</v>
       </c>
       <c r="Y48" s="58">
         <f t="shared" si="27"/>
-        <v>0.35892574693492518</v>
+        <v>0</v>
       </c>
       <c r="Z48" s="58">
         <f t="shared" si="27"/>
-        <v>0.36395864844037823</v>
+        <v>0</v>
       </c>
       <c r="AA48" s="58">
         <f t="shared" si="27"/>
-        <v>0.36999253966352963</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:27" x14ac:dyDescent="0.25">
@@ -9261,83 +9261,83 @@
       </c>
       <c r="H49" s="58">
         <f t="shared" si="28"/>
-        <v>0.18739635157545603</v>
+        <v>0</v>
       </c>
       <c r="I49" s="58">
         <f t="shared" si="28"/>
-        <v>0.23169162200595642</v>
+        <v>0</v>
       </c>
       <c r="J49" s="58">
         <f t="shared" si="28"/>
-        <v>0.26040332898313323</v>
+        <v>0</v>
       </c>
       <c r="K49" s="58">
         <f t="shared" si="28"/>
-        <v>0.27969527845026287</v>
+        <v>0</v>
       </c>
       <c r="L49" s="58">
         <f t="shared" si="28"/>
-        <v>0.31911336898823367</v>
+        <v>0</v>
       </c>
       <c r="M49" s="58">
         <f t="shared" si="28"/>
-        <v>0.33762764914950016</v>
+        <v>0</v>
       </c>
       <c r="N49" s="58">
         <f t="shared" si="28"/>
-        <v>0.34632891443374314</v>
+        <v>0</v>
       </c>
       <c r="O49" s="58">
         <f>IF(O22=0,0,O41/O22)</f>
-        <v>0.35041422605379186</v>
+        <v>0</v>
       </c>
       <c r="P49" s="58">
         <f t="shared" si="28"/>
-        <v>0.36122376869003991</v>
+        <v>0</v>
       </c>
       <c r="Q49" s="58">
         <f t="shared" si="28"/>
-        <v>0.37929407226256434</v>
+        <v>0</v>
       </c>
       <c r="R49" s="58">
         <f t="shared" si="28"/>
-        <v>0.40262985327724043</v>
+        <v>0</v>
       </c>
       <c r="S49" s="58">
         <f t="shared" si="28"/>
-        <v>0.42923511501696027</v>
+        <v>0</v>
       </c>
       <c r="T49" s="58">
         <f t="shared" si="28"/>
-        <v>0.44905707689235097</v>
+        <v>0</v>
       </c>
       <c r="U49" s="58">
         <f t="shared" si="28"/>
-        <v>0.46179033010914422</v>
+        <v>0</v>
       </c>
       <c r="V49" s="58">
         <f t="shared" si="28"/>
-        <v>0.46935827050416945</v>
+        <v>0</v>
       </c>
       <c r="W49" s="58">
         <f t="shared" si="28"/>
-        <v>0.47363882312359135</v>
+        <v>0</v>
       </c>
       <c r="X49" s="58">
         <f t="shared" ref="X49:AA49" si="29">IF(X22=0,0,X41/X22)</f>
-        <v>0.47762934902314275</v>
+        <v>0</v>
       </c>
       <c r="Y49" s="58">
         <f t="shared" si="29"/>
-        <v>0.48284058813864944</v>
+        <v>0</v>
       </c>
       <c r="Z49" s="58">
         <f t="shared" si="29"/>
-        <v>0.489611038973366</v>
+        <v>0</v>
       </c>
       <c r="AA49" s="58">
         <f t="shared" si="29"/>
-        <v>0.49772805930927205</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:27" x14ac:dyDescent="0.25">
@@ -9427,79 +9427,79 @@
       </c>
       <c r="I52" s="9">
         <f t="shared" si="30"/>
-        <v>14734.364442487693</v>
+        <v>0</v>
       </c>
       <c r="J52" s="9">
         <f t="shared" si="30"/>
-        <v>21819.483509096575</v>
+        <v>0</v>
       </c>
       <c r="K52" s="9">
         <f>MAX(0,J33)</f>
-        <v>25285.369557163212</v>
+        <v>0</v>
       </c>
       <c r="L52" s="9">
         <f t="shared" si="30"/>
-        <v>27040.198003314028</v>
+        <v>0</v>
       </c>
       <c r="M52" s="9">
         <f t="shared" si="30"/>
-        <v>13250.511580417538</v>
+        <v>0</v>
       </c>
       <c r="N52" s="9">
         <f t="shared" si="30"/>
-        <v>6732.8300426464539</v>
+        <v>0</v>
       </c>
       <c r="O52" s="9">
         <f t="shared" si="30"/>
-        <v>3650.5565036424659</v>
+        <v>0</v>
       </c>
       <c r="P52" s="9">
         <f t="shared" si="30"/>
-        <v>2196.1210067534025</v>
+        <v>0</v>
       </c>
       <c r="Q52" s="9">
         <f t="shared" si="30"/>
-        <v>4443.0754658203323</v>
+        <v>0</v>
       </c>
       <c r="R52" s="9">
         <f t="shared" si="30"/>
-        <v>6926.930203114187</v>
+        <v>0</v>
       </c>
       <c r="S52" s="9">
         <f t="shared" si="30"/>
-        <v>8805.2290220663272</v>
+        <v>0</v>
       </c>
       <c r="T52" s="9">
         <f t="shared" si="30"/>
-        <v>10056.750389878895</v>
+        <v>0</v>
       </c>
       <c r="U52" s="9">
         <f t="shared" si="30"/>
-        <v>7917.7311205801516</v>
+        <v>0</v>
       </c>
       <c r="V52" s="9">
         <f t="shared" si="30"/>
-        <v>5614.7978453976593</v>
+        <v>0</v>
       </c>
       <c r="W52" s="9">
         <f t="shared" si="30"/>
-        <v>3916.2174239855613</v>
+        <v>0</v>
       </c>
       <c r="X52" s="9">
         <f t="shared" ref="X52" si="31">MAX(0,W33)</f>
-        <v>2827.0500105071801</v>
+        <v>0</v>
       </c>
       <c r="Y52" s="9">
         <f t="shared" ref="Y52" si="32">MAX(0,X33)</f>
-        <v>2762.932856225525</v>
+        <v>0</v>
       </c>
       <c r="Z52" s="9">
         <f t="shared" ref="Z52" si="33">MAX(0,Y33)</f>
-        <v>3231.9961934842941</v>
+        <v>0</v>
       </c>
       <c r="AA52" s="9">
         <f t="shared" ref="AA52" si="34">MAX(0,Z33)</f>
-        <v>3833.6295666571982</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:27" x14ac:dyDescent="0.25">
@@ -9585,79 +9585,79 @@
       </c>
       <c r="I55" s="9">
         <f t="shared" si="35"/>
-        <v>14734.364442487693</v>
+        <v>0</v>
       </c>
       <c r="J55" s="9">
         <f t="shared" si="35"/>
-        <v>21819.483509096575</v>
+        <v>0</v>
       </c>
       <c r="K55" s="9">
         <f>SUM(K52:K54)</f>
-        <v>25285.369557163212</v>
+        <v>0</v>
       </c>
       <c r="L55" s="9">
         <f t="shared" si="35"/>
-        <v>27040.198003314028</v>
+        <v>0</v>
       </c>
       <c r="M55" s="9">
         <f t="shared" si="35"/>
-        <v>13250.511580417538</v>
+        <v>0</v>
       </c>
       <c r="N55" s="9">
         <f t="shared" si="35"/>
-        <v>6732.8300426464539</v>
+        <v>0</v>
       </c>
       <c r="O55" s="9">
         <f t="shared" si="35"/>
-        <v>3650.5565036424659</v>
+        <v>0</v>
       </c>
       <c r="P55" s="9">
         <f t="shared" si="35"/>
-        <v>2196.1210067534025</v>
+        <v>0</v>
       </c>
       <c r="Q55" s="9">
         <f t="shared" si="35"/>
-        <v>4443.0754658203323</v>
+        <v>0</v>
       </c>
       <c r="R55" s="9">
         <f t="shared" si="35"/>
-        <v>6926.930203114187</v>
+        <v>0</v>
       </c>
       <c r="S55" s="9">
         <f t="shared" si="35"/>
-        <v>8805.2290220663272</v>
+        <v>0</v>
       </c>
       <c r="T55" s="9">
         <f t="shared" si="35"/>
-        <v>10056.750389878895</v>
+        <v>0</v>
       </c>
       <c r="U55" s="9">
         <f t="shared" si="35"/>
-        <v>7917.7311205801516</v>
+        <v>0</v>
       </c>
       <c r="V55" s="9">
         <f t="shared" si="35"/>
-        <v>5614.7978453976593</v>
+        <v>0</v>
       </c>
       <c r="W55" s="9">
         <f t="shared" si="35"/>
-        <v>3916.2174239855613</v>
+        <v>0</v>
       </c>
       <c r="X55" s="9">
         <f t="shared" si="35"/>
-        <v>2827.0500105071801</v>
+        <v>0</v>
       </c>
       <c r="Y55" s="9">
         <f t="shared" si="35"/>
-        <v>2762.932856225525</v>
+        <v>0</v>
       </c>
       <c r="Z55" s="9">
         <f t="shared" si="35"/>
-        <v>3231.9961934842941</v>
+        <v>0</v>
       </c>
       <c r="AA55" s="9">
         <f t="shared" si="35"/>
-        <v>3833.6295666571982</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:27" x14ac:dyDescent="0.25">
@@ -9694,51 +9694,51 @@
       </c>
       <c r="P56" s="9">
         <f t="shared" si="36"/>
-        <v>6182.2508150298008</v>
+        <v>0</v>
       </c>
       <c r="Q56" s="9">
         <f t="shared" si="36"/>
-        <v>9155.0280457747849</v>
+        <v>0</v>
       </c>
       <c r="R56" s="9">
         <f t="shared" si="36"/>
-        <v>10609.245968040506</v>
+        <v>0</v>
       </c>
       <c r="S56" s="9">
         <f t="shared" si="36"/>
-        <v>11345.537623768123</v>
+        <v>0</v>
       </c>
       <c r="T56" s="9">
         <f t="shared" si="36"/>
-        <v>5559.655208566799</v>
+        <v>0</v>
       </c>
       <c r="U56" s="9">
         <f t="shared" si="36"/>
-        <v>2824.963654257253</v>
+        <v>0</v>
       </c>
       <c r="V56" s="9">
         <f t="shared" si="36"/>
-        <v>1531.7020295003351</v>
+        <v>0</v>
       </c>
       <c r="W56" s="9">
         <f t="shared" si="36"/>
-        <v>921.44937346296604</v>
+        <v>0</v>
       </c>
       <c r="X56" s="9">
         <f t="shared" si="36"/>
-        <v>1864.2274681763629</v>
+        <v>0</v>
       </c>
       <c r="Y56" s="9">
         <f t="shared" si="36"/>
-        <v>2906.4042810269311</v>
+        <v>0</v>
       </c>
       <c r="Z56" s="9">
         <f t="shared" si="36"/>
-        <v>3694.5016875802767</v>
+        <v>0</v>
       </c>
       <c r="AA56" s="9">
         <f t="shared" si="36"/>
-        <v>4219.6155482009344</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:27" x14ac:dyDescent="0.25">
@@ -9877,51 +9877,51 @@
       </c>
       <c r="P59" s="9">
         <f t="shared" si="38"/>
-        <v>6182.2508150298008</v>
+        <v>0</v>
       </c>
       <c r="Q59" s="9">
         <f t="shared" si="38"/>
-        <v>9155.0280457747849</v>
+        <v>0</v>
       </c>
       <c r="R59" s="9">
         <f t="shared" si="38"/>
-        <v>10609.245968040506</v>
+        <v>0</v>
       </c>
       <c r="S59" s="9">
         <f t="shared" si="38"/>
-        <v>11345.537623768123</v>
+        <v>0</v>
       </c>
       <c r="T59" s="9">
         <f t="shared" si="38"/>
-        <v>5559.655208566799</v>
+        <v>0</v>
       </c>
       <c r="U59" s="9">
         <f t="shared" si="38"/>
-        <v>2824.963654257253</v>
+        <v>0</v>
       </c>
       <c r="V59" s="9">
         <f t="shared" si="38"/>
-        <v>1531.7020295003351</v>
+        <v>0</v>
       </c>
       <c r="W59" s="9">
         <f t="shared" si="38"/>
-        <v>921.44937346296604</v>
+        <v>0</v>
       </c>
       <c r="X59" s="9">
         <f t="shared" ref="X59:AA59" si="39">SUM(X56:X58)</f>
-        <v>1864.2274681763629</v>
+        <v>0</v>
       </c>
       <c r="Y59" s="9">
         <f t="shared" si="39"/>
-        <v>2906.4042810269311</v>
+        <v>0</v>
       </c>
       <c r="Z59" s="9">
         <f t="shared" si="39"/>
-        <v>3694.5016875802767</v>
+        <v>0</v>
       </c>
       <c r="AA59" s="9">
         <f t="shared" si="39"/>
-        <v>4219.6155482009344</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:27" x14ac:dyDescent="0.25">
@@ -10148,51 +10148,51 @@
       </c>
       <c r="I64" s="32">
         <f>IF(SUM(D29:I29)&gt;0, SUMPRODUCT(D29:I29,D$13:I$13)/SUM(D29:I29), I$13)</f>
-        <v>2.4351247517514309</v>
+        <v>2.4483044266243899</v>
       </c>
       <c r="J64" s="32">
         <f>IF(SUM(D29:J29)&gt;0, SUMPRODUCT(D29:J29,D$13:J$13)/SUM(D29:J29), J$13)</f>
-        <v>2.4662160893820282</v>
+        <v>2.5111633473523298</v>
       </c>
       <c r="K64" s="32">
         <f t="shared" ref="K64:Z64" si="41">IF(SUM(D28:K28)&gt;0, SUMPRODUCT(D28:K28,D$13:K$13)/SUM(D28:K28), K$13)</f>
-        <v>2.4999890489208565</v>
+        <v>2.5772256649611598</v>
       </c>
       <c r="L64" s="32">
         <f t="shared" si="41"/>
-        <v>2.5257085482139687</v>
+        <v>2.6982252129903701</v>
       </c>
       <c r="M64" s="32">
         <f t="shared" si="41"/>
-        <v>2.5384399233691157</v>
+        <v>2.7315614500000001</v>
       </c>
       <c r="N64" s="32">
         <f t="shared" si="41"/>
-        <v>2.5475752953146165</v>
+        <v>2.82</v>
       </c>
       <c r="O64" s="32">
         <f t="shared" si="41"/>
-        <v>2.5527908873761325</v>
+        <v>2.82</v>
       </c>
       <c r="P64" s="32">
         <f t="shared" si="41"/>
-        <v>2.5835186852638432</v>
+        <v>2.82</v>
       </c>
       <c r="Q64" s="32">
         <f t="shared" si="41"/>
-        <v>2.6347710112970324</v>
+        <v>2.82</v>
       </c>
       <c r="R64" s="32">
         <f t="shared" si="41"/>
-        <v>2.6998873054806798</v>
+        <v>2.82</v>
       </c>
       <c r="S64" s="32">
         <f t="shared" si="41"/>
-        <v>2.7805968430347869</v>
+        <v>2.82</v>
       </c>
       <c r="T64" s="32">
         <f t="shared" si="41"/>
-        <v>2.8082623528944644</v>
+        <v>2.82</v>
       </c>
       <c r="U64" s="32">
         <f t="shared" si="41"/>
@@ -10200,7 +10200,7 @@
       </c>
       <c r="V64" s="32">
         <f t="shared" si="41"/>
-        <v>2.8200000000000003</v>
+        <v>2.82</v>
       </c>
       <c r="W64" s="32">
         <f t="shared" si="41"/>
@@ -10212,15 +10212,15 @@
       </c>
       <c r="Y64" s="32">
         <f t="shared" si="41"/>
-        <v>2.8200000000000003</v>
+        <v>2.82</v>
       </c>
       <c r="Z64" s="32">
         <f t="shared" si="41"/>
-        <v>2.8200000000000003</v>
+        <v>2.82</v>
       </c>
       <c r="AA64" s="32">
         <f>IF(SUM(T28:AA28)&gt;0, SUMPRODUCT(T28:AA28,T$13:AA$13)/SUM(T28:AA28), AA$13)</f>
-        <v>2.8200000000000003</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="65" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -10354,83 +10354,83 @@
       </c>
       <c r="H66" s="61">
         <f t="shared" si="43"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I66" s="61">
         <f t="shared" si="43"/>
-        <v>0.59691345047986666</v>
+        <v>0</v>
       </c>
       <c r="J66" s="61">
         <f t="shared" si="43"/>
-        <v>0.40888889891898228</v>
+        <v>0</v>
       </c>
       <c r="K66" s="61">
         <f t="shared" si="43"/>
-        <v>0.30423465149413026</v>
+        <v>0</v>
       </c>
       <c r="L66" s="61">
         <f t="shared" si="43"/>
-        <v>0.12974171193150025</v>
+        <v>0</v>
       </c>
       <c r="M66" s="61">
         <f t="shared" si="43"/>
-        <v>6.1846955008583449E-2</v>
+        <v>0</v>
       </c>
       <c r="N66" s="61">
         <f t="shared" si="43"/>
-        <v>3.2445551424810384E-2</v>
+        <v>0</v>
       </c>
       <c r="O66" s="61">
         <f t="shared" si="43"/>
-        <v>1.9145077417040052E-2</v>
+        <v>0</v>
       </c>
       <c r="P66" s="61">
         <f t="shared" si="43"/>
-        <v>3.7288979155105616E-2</v>
+        <v>0</v>
       </c>
       <c r="Q66" s="61">
         <f t="shared" si="43"/>
-        <v>5.4940997404792302E-2</v>
+        <v>0</v>
       </c>
       <c r="R66" s="61">
         <f t="shared" si="43"/>
-        <v>6.5279687197796074E-2</v>
+        <v>0</v>
       </c>
       <c r="S66" s="61">
         <f t="shared" si="43"/>
-        <v>6.9384930883542709E-2</v>
+        <v>0</v>
       </c>
       <c r="T66" s="61">
         <f t="shared" si="43"/>
-        <v>5.1797560543209803E-2</v>
+        <v>0</v>
       </c>
       <c r="U66" s="61">
         <f t="shared" si="43"/>
-        <v>3.5430415482968755E-2</v>
+        <v>0</v>
       </c>
       <c r="V66" s="61">
         <f t="shared" si="43"/>
-        <v>2.4116099623786972E-2</v>
+        <v>0</v>
       </c>
       <c r="W66" s="61">
         <f t="shared" si="43"/>
-        <v>1.7111110311508127E-2</v>
+        <v>0</v>
       </c>
       <c r="X66" s="61">
         <f t="shared" si="43"/>
-        <v>1.6447972411927924E-2</v>
+        <v>0</v>
       </c>
       <c r="Y66" s="61">
         <f t="shared" si="43"/>
-        <v>1.8877143266623642E-2</v>
+        <v>0</v>
       </c>
       <c r="Z66" s="61">
         <f t="shared" si="43"/>
-        <v>2.1900726094534171E-2</v>
+        <v>0</v>
       </c>
       <c r="AA66" s="61">
         <f t="shared" si="43"/>
-        <v>2.4377096125318194E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:27" x14ac:dyDescent="0.25">
@@ -10459,83 +10459,83 @@
       </c>
       <c r="H67" s="61">
         <f t="shared" si="44"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I67" s="61">
         <f t="shared" si="44"/>
-        <v>0.59691345047986677</v>
+        <v>0</v>
       </c>
       <c r="J67" s="61">
         <f t="shared" si="44"/>
-        <v>0.40888889891898239</v>
+        <v>0</v>
       </c>
       <c r="K67" s="61">
         <f t="shared" si="44"/>
-        <v>0.30423465149413026</v>
+        <v>0</v>
       </c>
       <c r="L67" s="61">
         <f t="shared" si="44"/>
-        <v>0.12974171193150025</v>
+        <v>0</v>
       </c>
       <c r="M67" s="61">
         <f t="shared" si="44"/>
-        <v>6.1846955008583449E-2</v>
+        <v>0</v>
       </c>
       <c r="N67" s="61">
         <f t="shared" si="44"/>
-        <v>3.2445551424810384E-2</v>
+        <v>0</v>
       </c>
       <c r="O67" s="61">
         <f t="shared" si="44"/>
-        <v>1.9145077417040052E-2</v>
+        <v>0</v>
       </c>
       <c r="P67" s="61">
         <f t="shared" si="44"/>
-        <v>3.7288979155105616E-2</v>
+        <v>0</v>
       </c>
       <c r="Q67" s="61">
         <f t="shared" si="44"/>
-        <v>5.4940997404792302E-2</v>
+        <v>0</v>
       </c>
       <c r="R67" s="61">
         <f t="shared" si="44"/>
-        <v>6.5279687197796074E-2</v>
+        <v>0</v>
       </c>
       <c r="S67" s="61">
         <f t="shared" si="44"/>
-        <v>6.9384930883542709E-2</v>
+        <v>0</v>
       </c>
       <c r="T67" s="61">
         <f t="shared" si="44"/>
-        <v>5.1797560543209796E-2</v>
+        <v>0</v>
       </c>
       <c r="U67" s="61">
         <f t="shared" si="44"/>
-        <v>3.5430415482968762E-2</v>
+        <v>0</v>
       </c>
       <c r="V67" s="61">
         <f t="shared" si="44"/>
-        <v>2.4116099623786968E-2</v>
+        <v>0</v>
       </c>
       <c r="W67" s="61">
         <f t="shared" si="44"/>
-        <v>1.7111110311508127E-2</v>
+        <v>0</v>
       </c>
       <c r="X67" s="61">
         <f t="shared" si="44"/>
-        <v>1.6447972411927924E-2</v>
+        <v>0</v>
       </c>
       <c r="Y67" s="61">
         <f t="shared" si="44"/>
-        <v>1.8877143266623642E-2</v>
+        <v>0</v>
       </c>
       <c r="Z67" s="61">
         <f t="shared" si="44"/>
-        <v>2.1900726094534174E-2</v>
+        <v>0</v>
       </c>
       <c r="AA67" s="61">
         <f t="shared" si="44"/>
-        <v>2.4377096125318198E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -10568,79 +10568,79 @@
       </c>
       <c r="I68" s="32">
         <f t="shared" si="45"/>
-        <v>2.7089933241223099</v>
+        <v>2.7232835266243902</v>
       </c>
       <c r="J68" s="32">
         <f t="shared" si="45"/>
-        <v>2.7416655274889266</v>
+        <v>2.7888981673523299</v>
       </c>
       <c r="K68" s="32">
         <f t="shared" si="45"/>
-        <v>2.7769721649053487</v>
+        <v>2.85771620496116</v>
       </c>
       <c r="L68" s="32">
         <f t="shared" si="45"/>
-        <v>2.7963685466984041</v>
+        <v>2.9264721329903698</v>
       </c>
       <c r="M68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8065619369041968</v>
+        <v>2.9611849100000001</v>
       </c>
       <c r="N68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8127083593221878</v>
+        <v>2.996</v>
       </c>
       <c r="O68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8162174919728611</v>
+        <v>2.996</v>
       </c>
       <c r="P68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8229213981671375</v>
+        <v>2.996</v>
       </c>
       <c r="Q68" s="32">
         <f t="shared" si="45"/>
-        <v>2.832430509181262</v>
+        <v>2.996</v>
       </c>
       <c r="R68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8431082743770122</v>
+        <v>2.996</v>
       </c>
       <c r="S68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8537166561920286</v>
+        <v>2.996</v>
       </c>
       <c r="T68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8610865863072119</v>
+        <v>2.996</v>
       </c>
       <c r="U68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8658666246085733</v>
+        <v>2.996</v>
       </c>
       <c r="V68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8690049340538923</v>
+        <v>2.996</v>
       </c>
       <c r="W68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8711779606363135</v>
+        <v>2.996</v>
       </c>
       <c r="X68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8732310300961674</v>
+        <v>2.996</v>
       </c>
       <c r="Y68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8755485575297381</v>
+        <v>2.996</v>
       </c>
       <c r="Z68" s="32">
         <f t="shared" si="45"/>
-        <v>2.878186531578971</v>
+        <v>2.996</v>
       </c>
       <c r="AA68" s="32">
         <f t="shared" si="45"/>
-        <v>2.8810584818235276</v>
+        <v>2.996</v>
       </c>
     </row>
     <row r="69" spans="1:27" ht="26.25" x14ac:dyDescent="0.25">
@@ -10673,79 +10673,79 @@
       </c>
       <c r="I69" s="32">
         <f t="shared" si="46"/>
-        <v>3.8184162959872445</v>
+        <v>3.8136239999999999</v>
       </c>
       <c r="J69" s="32">
         <f t="shared" si="46"/>
-        <v>3.8115954992384782</v>
+        <v>3.8017349999999999</v>
       </c>
       <c r="K69" s="32">
         <f t="shared" si="46"/>
-        <v>3.8049788521521393</v>
+        <v>3.789847</v>
       </c>
       <c r="L69" s="32">
         <f t="shared" si="46"/>
-        <v>3.8014731205360723</v>
+        <v>3.7779579999999999</v>
       </c>
       <c r="M69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7991542233501918</v>
+        <v>3.763979</v>
       </c>
       <c r="N69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7975593874687363</v>
+        <v>3.75</v>
       </c>
       <c r="O69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7966488593137404</v>
+        <v>3.75</v>
       </c>
       <c r="P69" s="32">
         <f t="shared" si="46"/>
-        <v>3.794909370971181</v>
+        <v>3.75</v>
       </c>
       <c r="Q69" s="32">
         <f>IF(Q41&gt;0,Q67*Q12+(1-Q67)*P69,Q12)</f>
-        <v>3.7924420053372025</v>
+        <v>3.75</v>
       </c>
       <c r="R69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7896714045047428</v>
+        <v>3.75</v>
       </c>
       <c r="S69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7869188068451285</v>
+        <v>3.75</v>
       </c>
       <c r="T69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7850065027123847</v>
+        <v>3.75</v>
       </c>
       <c r="U69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7837662077766794</v>
+        <v>3.75</v>
       </c>
       <c r="V69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7829518985460195</v>
+        <v>3.75</v>
       </c>
       <c r="W69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7823880549750246</v>
+        <v>3.75</v>
       </c>
       <c r="X69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7818553371403194</v>
+        <v>3.75</v>
       </c>
       <c r="Y69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7812539993773151</v>
+        <v>3.75</v>
       </c>
       <c r="Z69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7805695140975937</v>
+        <v>3.75</v>
       </c>
       <c r="AA69" s="32">
         <f t="shared" si="46"/>
-        <v>3.7798243181139322</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="70" spans="1:27" x14ac:dyDescent="0.25">
@@ -10807,79 +10807,79 @@
       </c>
       <c r="I71" s="46">
         <f t="shared" si="47"/>
-        <v>2.7204889770234395</v>
+        <v>2.6246962842974719</v>
       </c>
       <c r="J71" s="46">
         <f t="shared" si="47"/>
-        <v>2.798135215798677</v>
+        <v>2.6441179149915013</v>
       </c>
       <c r="K71" s="46">
         <f t="shared" si="47"/>
-        <v>2.8579694251486707</v>
+        <v>2.6646234693400936</v>
       </c>
       <c r="L71" s="46">
         <f t="shared" si="47"/>
-        <v>2.9890938771318822</v>
+        <v>2.8146267640630773</v>
       </c>
       <c r="M71" s="46">
         <f t="shared" si="47"/>
-        <v>3.0267111118402372</v>
+        <v>2.823476838208955</v>
       </c>
       <c r="N71" s="46">
         <f t="shared" si="47"/>
-        <v>3.0530738950175569</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="O71" s="46">
         <f t="shared" si="47"/>
-        <v>3.0597746177327556</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="P71" s="46">
         <f t="shared" si="47"/>
-        <v>3.0893572951882162</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="Q71" s="46">
         <f t="shared" si="47"/>
-        <v>3.1330398039972893</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="R71" s="46">
         <f t="shared" si="47"/>
-        <v>3.1815404598673336</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="S71" s="46">
         <f t="shared" si="47"/>
-        <v>3.2298011728648954</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="T71" s="46">
         <f t="shared" si="47"/>
-        <v>3.2581361372976918</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="U71" s="46">
         <f t="shared" si="47"/>
-        <v>3.2758336683881182</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="V71" s="46">
         <f t="shared" si="47"/>
-        <v>3.2856296321514793</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="W71" s="46">
         <f t="shared" si="47"/>
-        <v>3.2913818947302609</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="X71" s="46">
         <f t="shared" si="47"/>
-        <v>3.2959241074719738</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="Y71" s="46">
         <f t="shared" si="47"/>
-        <v>3.3013019811615849</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="Z71" s="46">
         <f t="shared" si="47"/>
-        <v>3.3082262232238078</v>
+        <v>2.9618805970149253</v>
       </c>
       <c r="AA71" s="46">
         <f>IF(AA22&gt;0,SUMPRODUCT(AA42,AA61)+SUMPRODUCT(AA46:AA47,AA64:AA65)+SUMPRODUCT(AA48:AA49,AA68:AA69),AA16)</f>
-        <v>3.3166376317482382</v>
+        <v>2.9618805970149253</v>
       </c>
     </row>
     <row r="73" spans="1:27" x14ac:dyDescent="0.25">
@@ -10937,83 +10937,83 @@
       </c>
       <c r="H74" s="13">
         <f>H19+H20</f>
-        <v>-201.81034552475003</v>
+        <v>0</v>
       </c>
       <c r="I74" s="13">
         <f t="shared" si="48"/>
-        <v>-405.65148753060447</v>
+        <v>0</v>
       </c>
       <c r="J74" s="13">
         <f t="shared" si="48"/>
-        <v>-627.97748030697539</v>
+        <v>0</v>
       </c>
       <c r="K74" s="13">
         <f>K19+K20</f>
-        <v>-861.95700227161262</v>
+        <v>0</v>
       </c>
       <c r="L74" s="13">
         <f t="shared" si="48"/>
-        <v>-897.06941973413893</v>
+        <v>0</v>
       </c>
       <c r="M74" s="13">
         <f t="shared" si="48"/>
-        <v>-944.93078222515908</v>
+        <v>0</v>
       </c>
       <c r="N74" s="13">
         <f t="shared" si="48"/>
-        <v>-963.97265559273126</v>
+        <v>0</v>
       </c>
       <c r="O74" s="13">
         <f t="shared" si="48"/>
-        <v>-979.72659800893848</v>
+        <v>0</v>
       </c>
       <c r="P74" s="13">
         <f t="shared" si="48"/>
-        <v>-989.37120580302053</v>
+        <v>0</v>
       </c>
       <c r="Q74" s="13">
         <f t="shared" si="48"/>
-        <v>-1006.5780005652127</v>
+        <v>0</v>
       </c>
       <c r="R74" s="13">
         <f t="shared" si="48"/>
-        <v>-1028.694808936199</v>
+        <v>0</v>
       </c>
       <c r="S74" s="13">
         <f t="shared" si="48"/>
-        <v>-1052.8014838752481</v>
+        <v>0</v>
       </c>
       <c r="T74" s="13">
         <f t="shared" si="48"/>
-        <v>-1077.2722536865842</v>
+        <v>0</v>
       </c>
       <c r="U74" s="13">
         <f t="shared" si="48"/>
-        <v>-1095.497885214302</v>
+        <v>0</v>
       </c>
       <c r="V74" s="13">
         <f t="shared" si="48"/>
-        <v>-1110.4200784701648</v>
+        <v>0</v>
       </c>
       <c r="W74" s="13">
         <f t="shared" si="48"/>
-        <v>-1122.8617212082197</v>
+        <v>0</v>
       </c>
       <c r="X74" s="13">
         <f t="shared" ref="X74:AA74" si="49">X19+X20</f>
-        <v>-1134.0669699318119</v>
+        <v>0</v>
       </c>
       <c r="Y74" s="13">
         <f t="shared" si="49"/>
-        <v>-1144.9765154434508</v>
+        <v>0</v>
       </c>
       <c r="Z74" s="13">
         <f t="shared" si="49"/>
-        <v>-1156.2945269574238</v>
+        <v>0</v>
       </c>
       <c r="AA74" s="13">
         <f t="shared" si="49"/>
-        <v>-1168.2829807615133</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:27" x14ac:dyDescent="0.25">
@@ -11040,83 +11040,83 @@
       </c>
       <c r="H75" s="13">
         <f>-SUM($D21:H21)</f>
-        <v>-31065.810345524751</v>
+        <v>0</v>
       </c>
       <c r="I75" s="13">
         <f>-SUM($D21:I21)</f>
-        <v>-62335.461833055357</v>
+        <v>0</v>
       </c>
       <c r="J75" s="13">
         <f>-SUM($D21:J21)</f>
-        <v>-93827.439313362338</v>
+        <v>0</v>
       </c>
       <c r="K75" s="13">
         <f>-SUM($D21:K21)</f>
-        <v>-125553.39631563395</v>
+        <v>0</v>
       </c>
       <c r="L75" s="13">
         <f>-SUM($D21:L21)</f>
-        <v>-126450.46573536808</v>
+        <v>0</v>
       </c>
       <c r="M75" s="13">
         <f>-SUM($D21:M21)</f>
-        <v>-127395.39651759324</v>
+        <v>0</v>
       </c>
       <c r="N75" s="13">
         <f>-SUM($D21:N21)</f>
-        <v>-128359.36917318597</v>
+        <v>0</v>
       </c>
       <c r="O75" s="13">
         <f>-SUM($D21:O21)</f>
-        <v>-129339.09577119492</v>
+        <v>0</v>
       </c>
       <c r="P75" s="13">
         <f>-SUM($D21:P21)</f>
-        <v>-130328.46697699794</v>
+        <v>0</v>
       </c>
       <c r="Q75" s="13">
         <f>-SUM($D21:Q21)</f>
-        <v>-131335.04497756314</v>
+        <v>0</v>
       </c>
       <c r="R75" s="13">
         <f>-SUM($D21:R21)</f>
-        <v>-132363.73978649935</v>
+        <v>0</v>
       </c>
       <c r="S75" s="13">
         <f>-SUM($D21:S21)</f>
-        <v>-133416.54127037461</v>
+        <v>0</v>
       </c>
       <c r="T75" s="13">
         <f>-SUM($D21:T21)</f>
-        <v>-134493.8135240612</v>
+        <v>0</v>
       </c>
       <c r="U75" s="13">
         <f>-SUM($D21:U21)</f>
-        <v>-135589.31140927551</v>
+        <v>0</v>
       </c>
       <c r="V75" s="13">
         <f>-SUM($D21:V21)</f>
-        <v>-136699.73148774568</v>
+        <v>0</v>
       </c>
       <c r="W75" s="13">
         <f>-SUM($D21:W21)</f>
-        <v>-137822.59320895391</v>
+        <v>0</v>
       </c>
       <c r="X75" s="13">
         <f>-SUM($D21:X21)</f>
-        <v>-138956.66017888574</v>
+        <v>0</v>
       </c>
       <c r="Y75" s="13">
         <f>-SUM($D21:Y21)</f>
-        <v>-140101.63669432918</v>
+        <v>0</v>
       </c>
       <c r="Z75" s="13">
         <f>-SUM($D21:Z21)</f>
-        <v>-141257.93122128659</v>
+        <v>0</v>
       </c>
       <c r="AA75" s="13">
         <f>-SUM($D21:AA21)</f>
-        <v>-142426.21420204811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:27" x14ac:dyDescent="0.25">
@@ -11143,83 +11143,83 @@
       </c>
       <c r="H76" s="13">
         <f>SUM($D74:H74)</f>
-        <v>-201.81034552475003</v>
+        <v>0</v>
       </c>
       <c r="I76" s="13">
         <f>SUM($D74:I74)</f>
-        <v>-607.46183305535453</v>
+        <v>0</v>
       </c>
       <c r="J76" s="13">
         <f>SUM($D74:J74)</f>
-        <v>-1235.4393133623298</v>
+        <v>0</v>
       </c>
       <c r="K76" s="13">
         <f>SUM($D74:K74)</f>
-        <v>-2097.3963156339423</v>
+        <v>0</v>
       </c>
       <c r="L76" s="13">
         <f>SUM($D74:L74)</f>
-        <v>-2994.4657353680814</v>
+        <v>0</v>
       </c>
       <c r="M76" s="13">
         <f>SUM($D74:M74)</f>
-        <v>-3939.3965175932403</v>
+        <v>0</v>
       </c>
       <c r="N76" s="13">
         <f>SUM($D74:N74)</f>
-        <v>-4903.3691731859717</v>
+        <v>0</v>
       </c>
       <c r="O76" s="13">
         <f>SUM($D74:O74)</f>
-        <v>-5883.0957711949104</v>
+        <v>0</v>
       </c>
       <c r="P76" s="13">
         <f>SUM($D74:P74)</f>
-        <v>-6872.4669769979309</v>
+        <v>0</v>
       </c>
       <c r="Q76" s="13">
         <f>SUM($D74:Q74)</f>
-        <v>-7879.0449775631441</v>
+        <v>0</v>
       </c>
       <c r="R76" s="13">
         <f>SUM($D74:R74)</f>
-        <v>-8907.7397864993436</v>
+        <v>0</v>
       </c>
       <c r="S76" s="13">
         <f>SUM($D74:S74)</f>
-        <v>-9960.5412703745915</v>
+        <v>0</v>
       </c>
       <c r="T76" s="13">
         <f>SUM($D74:T74)</f>
-        <v>-11037.813524061175</v>
+        <v>0</v>
       </c>
       <c r="U76" s="13">
         <f>SUM($D74:U74)</f>
-        <v>-12133.311409275477</v>
+        <v>0</v>
       </c>
       <c r="V76" s="13">
         <f>SUM($D74:V74)</f>
-        <v>-13243.731487745641</v>
+        <v>0</v>
       </c>
       <c r="W76" s="13">
         <f>SUM($D74:W74)</f>
-        <v>-14366.59320895386</v>
+        <v>0</v>
       </c>
       <c r="X76" s="13">
         <f>SUM($D74:X74)</f>
-        <v>-15500.660178885671</v>
+        <v>0</v>
       </c>
       <c r="Y76" s="13">
         <f>SUM($D74:Y74)</f>
-        <v>-16645.636694329121</v>
+        <v>0</v>
       </c>
       <c r="Z76" s="13">
         <f>SUM($D74:Z74)</f>
-        <v>-17801.931221286544</v>
+        <v>0</v>
       </c>
       <c r="AA76" s="13">
         <f>SUM($D74:AA74)</f>
-        <v>-18970.214202048057</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:27" x14ac:dyDescent="0.25">

</xml_diff>